<commit_message>
detecta A+ speed y normal speed
</commit_message>
<xml_diff>
--- a/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
+++ b/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
@@ -2,24 +2,24 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="\+0.##;\-0.##;0"/>
-    <numFmt numFmtId="165" formatCode="+0.##;-0.##;0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="+0.##;-0.##;0"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,16 +28,10 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <b val="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -46,16 +40,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFD9EAF7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00D9EAF7"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -63,43 +52,21 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -172,7 +139,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -182,44 +149,44 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546A"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E7E6E6"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ED7D31"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A5A5A5"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="FFC000"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70AD47"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563C1"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954F72"/>
+        <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
@@ -246,32 +213,14 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
@@ -298,24 +247,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -327,142 +258,166 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="35000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="80000">
               <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
+                <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="40000">
               <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
@@ -473,297 +428,297 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:AI8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="3"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="8"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="12" bestFit="1" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="13"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="16" customWidth="1" min="13" max="13"/>
     <col width="10" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="17"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
     <col width="10" customWidth="1" min="16" max="16"/>
     <col width="10" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>win rate</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>profit factor</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2">
-        <f>IF((COUNTIF(N4:N8,"&gt;0")+COUNTIF(N4:N8,"&lt;0"))=0,"",COUNTIF(N4:N8,"&gt;0")/(COUNTIF(N4:N8,"&gt;0")+COUNTIF(N4:N8,"&lt;0")))</f>
+      <c r="A2" s="1">
+        <f>IF((COUNTIF(Q4:Q8,"&gt;0")+COUNTIF(Q4:Q8,"&lt;0"))=0,"",COUNTIF(Q4:Q8,"&gt;0")/(COUNTIF(Q4:Q8,"&gt;0")+COUNTIF(Q4:Q8,"&lt;0")))</f>
         <v/>
       </c>
-      <c r="B2" s="3">
-        <f>IF(ABS(SUMIF(N4:N8,"&lt;0",N4:N8))=0,IF(SUMIF(N4:N8,"&gt;0",N4:N8)&gt;0,"INF",""),SUMIF(N4:N8,"&gt;0",N4:N8)/ABS(SUMIF(N4:N8,"&lt;0",N4:N8)))</f>
+      <c r="B2" s="2">
+        <f>IF(ABS(SUMIF(Q4:Q8,"&lt;0",Q4:Q8))=0,IF(SUMIF(Q4:Q8,"&gt;0",Q4:Q8)&gt;0,"INF",""),SUMIF(Q4:Q8,"&gt;0",Q4:Q8)/ABS(SUMIF(Q4:Q8,"&lt;0",Q4:Q8)))</f>
         <v/>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>fecha</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>or_low</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>or_high</t>
         </is>
       </c>
-      <c r="D3" s="8" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>range</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>VWAP_entry</t>
         </is>
       </c>
-      <c r="F3" s="8" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>Body</t>
         </is>
       </c>
-      <c r="G3" s="8" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>Volume_entry</t>
         </is>
       </c>
-      <c r="H3" s="8" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>Delta_entry</t>
         </is>
       </c>
-      <c r="I3" s="8" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>BreakOut_SPEED</t>
         </is>
       </c>
-      <c r="J3" s="8" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>BreakOut_TICKS_PER_SEC</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>score total</t>
         </is>
       </c>
-      <c r="K3" s="8" t="inlineStr">
+      <c r="L3" s="3" t="inlineStr">
         <is>
           <t>SL_price</t>
         </is>
       </c>
-      <c r="L3" s="8" t="inlineStr">
+      <c r="M3" s="3" t="inlineStr">
         <is>
           <t>Entry_price</t>
         </is>
       </c>
-      <c r="M3" s="8" t="inlineStr">
+      <c r="N3" s="3" t="inlineStr">
         <is>
           <t>TP_price</t>
         </is>
       </c>
-      <c r="N3" s="8" t="inlineStr">
+      <c r="O3" s="3" t="inlineStr">
+        <is>
+          <t>SL_ticks</t>
+        </is>
+      </c>
+      <c r="P3" s="3" t="inlineStr">
+        <is>
+          <t>TP_ticks</t>
+        </is>
+      </c>
+      <c r="Q3" s="3" t="inlineStr">
         <is>
           <t>result TP SL BE</t>
         </is>
       </c>
-      <c r="O3" s="9" t="inlineStr">
+      <c r="R3" s="3" t="inlineStr">
         <is>
           <t>Side</t>
         </is>
       </c>
-      <c r="P3" s="9" t="inlineStr">
+      <c r="S3" s="3" t="inlineStr">
+        <is>
+          <t>Speed_Profile</t>
+        </is>
+      </c>
+      <c r="T3" s="3" t="inlineStr">
         <is>
           <t>MAE_ticks</t>
         </is>
       </c>
-      <c r="Q3" s="9" t="inlineStr">
+      <c r="U3" s="3" t="inlineStr">
         <is>
           <t>MFE_ticks</t>
         </is>
       </c>
-      <c r="R3" s="9" t="inlineStr">
-        <is>
-          <t>BreakOut_TICKS_PER_SEC</t>
-        </is>
-      </c>
-      <c r="S3" s="9" t="inlineStr">
-        <is>
-          <t>SL_ticks</t>
-        </is>
-      </c>
-      <c r="T3" s="9" t="inlineStr">
-        <is>
-          <t>TP_ticks</t>
-        </is>
-      </c>
-      <c r="U3" s="9" t="inlineStr">
-        <is>
-          <t>Speed_Profile</t>
-        </is>
-      </c>
-      <c r="V3" s="9" t="inlineStr">
+      <c r="V3" s="3" t="inlineStr">
         <is>
           <t>Exporter_VERSION</t>
         </is>
       </c>
-      <c r="W3" s="9" t="inlineStr">
+      <c r="W3" s="3" t="inlineStr">
         <is>
           <t>EntryTime_NY</t>
         </is>
       </c>
-      <c r="X3" s="9" t="inlineStr">
+      <c r="X3" s="3" t="inlineStr">
         <is>
           <t>EntryBar</t>
         </is>
       </c>
-      <c r="Y3" s="9" t="inlineStr">
+      <c r="Y3" s="3" t="inlineStr">
         <is>
           <t>Speed_Elapsed_SECONDS</t>
         </is>
       </c>
-      <c r="Z3" s="9" t="inlineStr">
+      <c r="Z3" s="3" t="inlineStr">
         <is>
           <t>Speed_Replay_Fallback</t>
         </is>
       </c>
-      <c r="AA3" s="9" t="inlineStr">
+      <c r="AA3" s="3" t="inlineStr">
         <is>
           <t>Speed_Timing_Source</t>
         </is>
       </c>
-      <c r="AB3" s="9" t="inlineStr">
+      <c r="AB3" s="3" t="inlineStr">
         <is>
           <t>Range_OK</t>
         </is>
       </c>
-      <c r="AC3" s="9" t="inlineStr">
+      <c r="AC3" s="3" t="inlineStr">
         <is>
           <t>Body_OK</t>
         </is>
       </c>
-      <c r="AD3" s="9" t="inlineStr">
+      <c r="AD3" s="3" t="inlineStr">
         <is>
           <t>Volume_OK</t>
         </is>
       </c>
-      <c r="AE3" s="9" t="inlineStr">
+      <c r="AE3" s="3" t="inlineStr">
         <is>
           <t>Delta_OK</t>
         </is>
       </c>
-      <c r="AF3" s="9" t="inlineStr">
+      <c r="AF3" s="3" t="inlineStr">
         <is>
           <t>Time_OK</t>
         </is>
       </c>
-      <c r="AG3" s="9" t="inlineStr">
+      <c r="AG3" s="3" t="inlineStr">
         <is>
           <t>VWAP_OK</t>
         </is>
       </c>
-      <c r="AH3" s="9" t="inlineStr">
+      <c r="AH3" s="3" t="inlineStr">
         <is>
           <t>Speed_OK</t>
         </is>
       </c>
-      <c r="AI3" s="9" t="inlineStr">
+      <c r="AI3" s="3" t="inlineStr">
         <is>
           <t>Result_Label</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>2026-05-11</t>
         </is>
       </c>
-      <c r="B4" s="1" t="n">
+      <c r="B4" t="n">
         <v>29282.5</v>
       </c>
-      <c r="C4" s="1" t="n">
+      <c r="C4" t="n">
         <v>29346.25</v>
       </c>
-      <c r="D4" s="1" t="n">
+      <c r="D4" t="n">
         <v>255</v>
       </c>
-      <c r="E4" s="1" t="n">
-        <v>29316.31</v>
-      </c>
-      <c r="F4" s="1" t="n">
-        <v>25</v>
-      </c>
-      <c r="G4" s="1" t="n">
-        <v>237</v>
-      </c>
-      <c r="H4" s="1" t="n">
-        <v>51</v>
-      </c>
-      <c r="I4" s="1" t="inlineStr">
+      <c r="E4" t="n">
+        <v>29316.27</v>
+      </c>
+      <c r="F4" t="n">
+        <v>10</v>
+      </c>
+      <c r="G4" t="n">
+        <v>120</v>
+      </c>
+      <c r="H4" t="n">
+        <v>26</v>
+      </c>
+      <c r="I4" t="inlineStr">
         <is>
           <t>A+ speed</t>
         </is>
       </c>
-      <c r="J4" s="1" t="n">
+      <c r="J4" t="n">
+        <v>15.21</v>
+      </c>
+      <c r="K4" t="n">
         <v>6</v>
       </c>
-      <c r="K4" s="1" t="n">
-        <v>29327.5</v>
-      </c>
-      <c r="L4" s="1" t="n">
-        <v>29352.5</v>
-      </c>
-      <c r="M4" s="1" t="n">
-        <v>29382.5</v>
-      </c>
-      <c r="N4" s="10" t="n">
+      <c r="L4" t="n">
+        <v>29323.75</v>
+      </c>
+      <c r="M4" t="n">
+        <v>29348.75</v>
+      </c>
+      <c r="N4" t="n">
+        <v>29378.75</v>
+      </c>
+      <c r="O4" t="n">
+        <v>100</v>
+      </c>
+      <c r="P4" t="n">
         <v>120</v>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="Q4" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="R4" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="P4" t="n">
-        <v>35</v>
-      </c>
-      <c r="Q4" t="n">
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="T4" t="n">
+        <v>20</v>
+      </c>
+      <c r="U4" t="n">
         <v>120</v>
-      </c>
-      <c r="R4" t="n">
-        <v>13.38</v>
-      </c>
-      <c r="S4" t="n">
-        <v>100</v>
-      </c>
-      <c r="T4" t="n">
-        <v>120</v>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
       </c>
       <c r="V4" t="inlineStr">
         <is>
@@ -779,7 +734,7 @@
         <v>2311</v>
       </c>
       <c r="Y4" t="n">
-        <v>1.8681</v>
+        <v>0.6576</v>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
@@ -848,16 +803,16 @@
         <v>325</v>
       </c>
       <c r="E5" t="n">
-        <v>29202.58</v>
+        <v>29202.57</v>
       </c>
       <c r="F5" t="n">
         <v>10</v>
       </c>
       <c r="G5" t="n">
-        <v>86</v>
+        <v>44</v>
       </c>
       <c r="H5" t="n">
-        <v>-16</v>
+        <v>-4</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -865,44 +820,44 @@
         </is>
       </c>
       <c r="J5" t="n">
+        <v>23.77</v>
+      </c>
+      <c r="K5" t="n">
         <v>5</v>
       </c>
-      <c r="K5" t="n">
+      <c r="L5" t="n">
         <v>29205</v>
       </c>
-      <c r="L5" t="n">
+      <c r="M5" t="n">
         <v>29230</v>
       </c>
-      <c r="M5" t="n">
+      <c r="N5" t="n">
         <v>29260</v>
       </c>
-      <c r="N5" s="11" t="n">
+      <c r="O5" t="n">
+        <v>100</v>
+      </c>
+      <c r="P5" t="n">
         <v>120</v>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="Q5" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="R5" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="P5" t="n">
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="T5" t="n">
         <v>65</v>
       </c>
-      <c r="Q5" t="n">
+      <c r="U5" t="n">
         <v>120</v>
-      </c>
-      <c r="R5" t="n">
-        <v>9.710000000000001</v>
-      </c>
-      <c r="S5" t="n">
-        <v>100</v>
-      </c>
-      <c r="T5" t="n">
-        <v>120</v>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
       </c>
       <c r="V5" t="inlineStr">
         <is>
@@ -918,7 +873,7 @@
         <v>2320</v>
       </c>
       <c r="Y5" t="n">
-        <v>1.0303</v>
+        <v>0.4207</v>
       </c>
       <c r="Z5" t="inlineStr">
         <is>
@@ -1004,44 +959,44 @@
         </is>
       </c>
       <c r="J6" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="K6" t="n">
         <v>7</v>
       </c>
-      <c r="K6" t="n">
+      <c r="L6" t="n">
         <v>29258.75</v>
       </c>
-      <c r="L6" t="n">
+      <c r="M6" t="n">
         <v>29243.75</v>
       </c>
-      <c r="M6" t="n">
+      <c r="N6" t="n">
         <v>29213.75</v>
       </c>
-      <c r="N6" s="11" t="n">
+      <c r="O6" t="n">
+        <v>60</v>
+      </c>
+      <c r="P6" t="n">
+        <v>120</v>
+      </c>
+      <c r="Q6" s="4" t="n">
         <v>-60</v>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="R6" t="inlineStr">
         <is>
           <t>SELL</t>
         </is>
       </c>
-      <c r="P6" t="n">
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>SELL1</t>
+        </is>
+      </c>
+      <c r="T6" t="n">
         <v>100</v>
       </c>
-      <c r="Q6" t="n">
+      <c r="U6" t="n">
         <v>10</v>
-      </c>
-      <c r="R6" t="n">
-        <v>2.08</v>
-      </c>
-      <c r="S6" t="n">
-        <v>60</v>
-      </c>
-      <c r="T6" t="n">
-        <v>120</v>
-      </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>SELL1</t>
-        </is>
       </c>
       <c r="V6" t="inlineStr">
         <is>
@@ -1126,13 +1081,13 @@
         <v>130</v>
       </c>
       <c r="E7" t="n">
-        <v>29543.51</v>
+        <v>29543.5</v>
       </c>
       <c r="F7" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="G7" t="n">
-        <v>802</v>
+        <v>804</v>
       </c>
       <c r="H7" t="n">
         <v>262</v>
@@ -1143,44 +1098,44 @@
         </is>
       </c>
       <c r="J7" t="n">
+        <v>10.04</v>
+      </c>
+      <c r="K7" t="n">
         <v>5</v>
       </c>
-      <c r="K7" t="n">
-        <v>29490</v>
-      </c>
       <c r="L7" t="n">
-        <v>29515</v>
+        <v>29488.75</v>
       </c>
       <c r="M7" t="n">
-        <v>29545</v>
-      </c>
-      <c r="N7" s="11" t="n">
+        <v>29513.75</v>
+      </c>
+      <c r="N7" t="n">
+        <v>29543.75</v>
+      </c>
+      <c r="O7" t="n">
+        <v>100</v>
+      </c>
+      <c r="P7" t="n">
         <v>120</v>
       </c>
-      <c r="O7" t="inlineStr">
+      <c r="Q7" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="R7" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="P7" t="n">
-        <v>65</v>
-      </c>
-      <c r="Q7" t="n">
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="T7" t="n">
+        <v>60</v>
+      </c>
+      <c r="U7" t="n">
         <v>120</v>
-      </c>
-      <c r="R7" t="n">
-        <v>10.97</v>
-      </c>
-      <c r="S7" t="n">
-        <v>100</v>
-      </c>
-      <c r="T7" t="n">
-        <v>120</v>
-      </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
       </c>
       <c r="V7" t="inlineStr">
         <is>
@@ -1196,7 +1151,7 @@
         <v>2312</v>
       </c>
       <c r="Y7" t="n">
-        <v>5.9247</v>
+        <v>5.9788</v>
       </c>
       <c r="Z7" t="inlineStr">
         <is>
@@ -1271,10 +1226,10 @@
         <v>10</v>
       </c>
       <c r="G8" t="n">
-        <v>404</v>
+        <v>409</v>
       </c>
       <c r="H8" t="n">
-        <v>-174</v>
+        <v>-177</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -1282,44 +1237,44 @@
         </is>
       </c>
       <c r="J8" t="n">
+        <v>4.59</v>
+      </c>
+      <c r="K8" t="n">
         <v>6</v>
       </c>
-      <c r="K8" t="n">
+      <c r="L8" t="n">
         <v>29253.75</v>
       </c>
-      <c r="L8" t="n">
+      <c r="M8" t="n">
         <v>29238.75</v>
       </c>
-      <c r="M8" t="n">
+      <c r="N8" t="n">
         <v>29208.75</v>
       </c>
-      <c r="N8" s="11" t="n">
+      <c r="O8" t="n">
+        <v>60</v>
+      </c>
+      <c r="P8" t="n">
+        <v>120</v>
+      </c>
+      <c r="Q8" s="4" t="n">
         <v>-60</v>
       </c>
-      <c r="O8" t="inlineStr">
+      <c r="R8" t="inlineStr">
         <is>
           <t>SELL</t>
         </is>
       </c>
-      <c r="P8" t="n">
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>SELL1</t>
+        </is>
+      </c>
+      <c r="T8" t="n">
         <v>80</v>
       </c>
-      <c r="Q8" t="n">
+      <c r="U8" t="n">
         <v>15</v>
-      </c>
-      <c r="R8" t="n">
-        <v>4.61</v>
-      </c>
-      <c r="S8" t="n">
-        <v>60</v>
-      </c>
-      <c r="T8" t="n">
-        <v>120</v>
-      </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>SELL1</t>
-        </is>
       </c>
       <c r="V8" t="inlineStr">
         <is>
@@ -1335,7 +1290,7 @@
         <v>2311</v>
       </c>
       <c r="Y8" t="n">
-        <v>2.1714</v>
+        <v>2.1782</v>
       </c>
       <c r="Z8" t="inlineStr">
         <is>
@@ -1389,6 +1344,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Commit A+ speed Normal Speed OK
</commit_message>
<xml_diff>
--- a/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
+++ b/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
@@ -463,11 +463,11 @@
     </row>
     <row r="2">
       <c r="A2" s="1">
-        <f>IF((COUNTIF(Q4:Q8,"&gt;0")+COUNTIF(Q4:Q8,"&lt;0"))=0,"",COUNTIF(Q4:Q8,"&gt;0")/(COUNTIF(Q4:Q8,"&gt;0")+COUNTIF(Q4:Q8,"&lt;0")))</f>
+        <f>IF((COUNTIF(Q4:Q4,"&gt;0")+COUNTIF(Q4:Q4,"&lt;0"))=0,"",COUNTIF(Q4:Q4,"&gt;0")/(COUNTIF(Q4:Q4,"&gt;0")+COUNTIF(Q4:Q4,"&lt;0")))</f>
         <v/>
       </c>
       <c r="B2" s="2">
-        <f>IF(ABS(SUMIF(Q4:Q8,"&lt;0",Q4:Q8))=0,IF(SUMIF(Q4:Q8,"&gt;0",Q4:Q8)&gt;0,"INF",""),SUMIF(Q4:Q8,"&gt;0",Q4:Q8)/ABS(SUMIF(Q4:Q8,"&lt;0",Q4:Q8)))</f>
+        <f>IF(ABS(SUMIF(Q4:Q4,"&lt;0",Q4:Q4))=0,IF(SUMIF(Q4:Q4,"&gt;0",Q4:Q4)&gt;0,"INF",""),SUMIF(Q4:Q4,"&gt;0",Q4:Q4)/ABS(SUMIF(Q4:Q4,"&lt;0",Q4:Q4)))</f>
         <v/>
       </c>
     </row>
@@ -651,78 +651,78 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>29282.5</v>
+        <v>29241.25</v>
       </c>
       <c r="C4" t="n">
-        <v>29346.25</v>
+        <v>29291.25</v>
       </c>
       <c r="D4" t="n">
-        <v>255</v>
+        <v>200</v>
       </c>
       <c r="E4" t="n">
-        <v>29316.27</v>
+        <v>29294.96</v>
       </c>
       <c r="F4" t="n">
         <v>10</v>
       </c>
       <c r="G4" t="n">
-        <v>120</v>
+        <v>367</v>
       </c>
       <c r="H4" t="n">
-        <v>26</v>
+        <v>-145</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>A+ speed</t>
+          <t>normal speed</t>
         </is>
       </c>
       <c r="J4" t="n">
-        <v>15.21</v>
+        <v>4.64</v>
       </c>
       <c r="K4" t="n">
         <v>6</v>
       </c>
       <c r="L4" t="n">
-        <v>29323.75</v>
+        <v>29253.75</v>
       </c>
       <c r="M4" t="n">
-        <v>29348.75</v>
+        <v>29238.75</v>
       </c>
       <c r="N4" t="n">
-        <v>29378.75</v>
+        <v>29208.75</v>
       </c>
       <c r="O4" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="P4" t="n">
         <v>120</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>120</v>
+        <v>-60</v>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL1</t>
         </is>
       </c>
       <c r="T4" t="n">
-        <v>20</v>
+        <v>80</v>
       </c>
       <c r="U4" t="n">
-        <v>120</v>
+        <v>15</v>
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>score-exporter-debug-2026-05-22-e-x10</t>
+          <t>score-exporter-2026-05-22-sync-visual-speed</t>
         </is>
       </c>
       <c r="W4" t="inlineStr">
@@ -734,7 +734,7 @@
         <v>2311</v>
       </c>
       <c r="Y4" t="n">
-        <v>0.6576</v>
+        <v>2.1573</v>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
@@ -783,565 +783,21 @@
       </c>
       <c r="AI4" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>SL</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>29146.25</v>
-      </c>
-      <c r="C5" t="n">
-        <v>29227.5</v>
-      </c>
-      <c r="D5" t="n">
-        <v>325</v>
-      </c>
-      <c r="E5" t="n">
-        <v>29202.57</v>
-      </c>
-      <c r="F5" t="n">
-        <v>10</v>
-      </c>
-      <c r="G5" t="n">
-        <v>44</v>
-      </c>
-      <c r="H5" t="n">
-        <v>-4</v>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>A+ speed</t>
-        </is>
-      </c>
-      <c r="J5" t="n">
-        <v>23.77</v>
-      </c>
-      <c r="K5" t="n">
-        <v>5</v>
-      </c>
-      <c r="L5" t="n">
-        <v>29205</v>
-      </c>
-      <c r="M5" t="n">
-        <v>29230</v>
-      </c>
-      <c r="N5" t="n">
-        <v>29260</v>
-      </c>
-      <c r="O5" t="n">
-        <v>100</v>
-      </c>
-      <c r="P5" t="n">
-        <v>120</v>
-      </c>
-      <c r="Q5" s="4" t="n">
-        <v>120</v>
-      </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="T5" t="n">
-        <v>65</v>
-      </c>
-      <c r="U5" t="n">
-        <v>120</v>
-      </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>score-exporter-debug-2026-05-22-e-x10</t>
-        </is>
-      </c>
-      <c r="W5" t="inlineStr">
-        <is>
-          <t>09:40:00</t>
-        </is>
-      </c>
-      <c r="X5" t="n">
-        <v>2320</v>
-      </c>
-      <c r="Y5" t="n">
-        <v>0.4207</v>
-      </c>
-      <c r="Z5" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AA5" t="inlineStr">
-        <is>
-          <t>LastTime</t>
-        </is>
-      </c>
-      <c r="AB5" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AC5" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AD5" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AE5" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AF5" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AG5" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AH5" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AI5" t="inlineStr">
-        <is>
-          <t>TP</t>
-        </is>
-      </c>
+      <c r="Q5" s="4" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2026-05-13</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>29252.5</v>
-      </c>
-      <c r="C6" t="n">
-        <v>29288.75</v>
-      </c>
-      <c r="D6" t="n">
-        <v>145</v>
-      </c>
-      <c r="E6" t="n">
-        <v>29321.36</v>
-      </c>
-      <c r="F6" t="n">
-        <v>35</v>
-      </c>
-      <c r="G6" t="n">
-        <v>1114</v>
-      </c>
-      <c r="H6" t="n">
-        <v>-176</v>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>normal speed</t>
-        </is>
-      </c>
-      <c r="J6" t="n">
-        <v>2.08</v>
-      </c>
-      <c r="K6" t="n">
-        <v>7</v>
-      </c>
-      <c r="L6" t="n">
-        <v>29258.75</v>
-      </c>
-      <c r="M6" t="n">
-        <v>29243.75</v>
-      </c>
-      <c r="N6" t="n">
-        <v>29213.75</v>
-      </c>
-      <c r="O6" t="n">
-        <v>60</v>
-      </c>
-      <c r="P6" t="n">
-        <v>120</v>
-      </c>
-      <c r="Q6" s="4" t="n">
-        <v>-60</v>
-      </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>SELL1</t>
-        </is>
-      </c>
-      <c r="T6" t="n">
-        <v>100</v>
-      </c>
-      <c r="U6" t="n">
-        <v>10</v>
-      </c>
-      <c r="V6" t="inlineStr">
-        <is>
-          <t>score-exporter-debug-2026-05-22-e-x10</t>
-        </is>
-      </c>
-      <c r="W6" t="inlineStr">
-        <is>
-          <t>09:31:00</t>
-        </is>
-      </c>
-      <c r="X6" t="n">
-        <v>2311</v>
-      </c>
-      <c r="Y6" t="n">
-        <v>16.8169</v>
-      </c>
-      <c r="Z6" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AA6" t="inlineStr">
-        <is>
-          <t>LastTime</t>
-        </is>
-      </c>
-      <c r="AB6" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AC6" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AD6" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AE6" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AF6" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AG6" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AH6" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AI6" t="inlineStr">
-        <is>
-          <t>SL</t>
-        </is>
-      </c>
+      <c r="Q6" s="4" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>29460</v>
-      </c>
-      <c r="C7" t="n">
-        <v>29492.5</v>
-      </c>
-      <c r="D7" t="n">
-        <v>130</v>
-      </c>
-      <c r="E7" t="n">
-        <v>29543.5</v>
-      </c>
-      <c r="F7" t="n">
-        <v>60</v>
-      </c>
-      <c r="G7" t="n">
-        <v>804</v>
-      </c>
-      <c r="H7" t="n">
-        <v>262</v>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>A+ speed</t>
-        </is>
-      </c>
-      <c r="J7" t="n">
-        <v>10.04</v>
-      </c>
-      <c r="K7" t="n">
-        <v>5</v>
-      </c>
-      <c r="L7" t="n">
-        <v>29488.75</v>
-      </c>
-      <c r="M7" t="n">
-        <v>29513.75</v>
-      </c>
-      <c r="N7" t="n">
-        <v>29543.75</v>
-      </c>
-      <c r="O7" t="n">
-        <v>100</v>
-      </c>
-      <c r="P7" t="n">
-        <v>120</v>
-      </c>
-      <c r="Q7" s="4" t="n">
-        <v>120</v>
-      </c>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="S7" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="T7" t="n">
-        <v>60</v>
-      </c>
-      <c r="U7" t="n">
-        <v>120</v>
-      </c>
-      <c r="V7" t="inlineStr">
-        <is>
-          <t>score-exporter-debug-2026-05-22-e-x10</t>
-        </is>
-      </c>
-      <c r="W7" t="inlineStr">
-        <is>
-          <t>09:32:00</t>
-        </is>
-      </c>
-      <c r="X7" t="n">
-        <v>2312</v>
-      </c>
-      <c r="Y7" t="n">
-        <v>5.9788</v>
-      </c>
-      <c r="Z7" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AA7" t="inlineStr">
-        <is>
-          <t>LastTime</t>
-        </is>
-      </c>
-      <c r="AB7" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AC7" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AD7" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AE7" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AF7" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AG7" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AH7" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AI7" t="inlineStr">
-        <is>
-          <t>TP</t>
-        </is>
-      </c>
+      <c r="Q7" s="4" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>29241.25</v>
-      </c>
-      <c r="C8" t="n">
-        <v>29291.25</v>
-      </c>
-      <c r="D8" t="n">
-        <v>200</v>
-      </c>
-      <c r="E8" t="n">
-        <v>29294.95</v>
-      </c>
-      <c r="F8" t="n">
-        <v>10</v>
-      </c>
-      <c r="G8" t="n">
-        <v>409</v>
-      </c>
-      <c r="H8" t="n">
-        <v>-177</v>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>normal speed</t>
-        </is>
-      </c>
-      <c r="J8" t="n">
-        <v>4.59</v>
-      </c>
-      <c r="K8" t="n">
-        <v>6</v>
-      </c>
-      <c r="L8" t="n">
-        <v>29253.75</v>
-      </c>
-      <c r="M8" t="n">
-        <v>29238.75</v>
-      </c>
-      <c r="N8" t="n">
-        <v>29208.75</v>
-      </c>
-      <c r="O8" t="n">
-        <v>60</v>
-      </c>
-      <c r="P8" t="n">
-        <v>120</v>
-      </c>
-      <c r="Q8" s="4" t="n">
-        <v>-60</v>
-      </c>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="S8" t="inlineStr">
-        <is>
-          <t>SELL1</t>
-        </is>
-      </c>
-      <c r="T8" t="n">
-        <v>80</v>
-      </c>
-      <c r="U8" t="n">
-        <v>15</v>
-      </c>
-      <c r="V8" t="inlineStr">
-        <is>
-          <t>score-exporter-debug-2026-05-22-e-x10</t>
-        </is>
-      </c>
-      <c r="W8" t="inlineStr">
-        <is>
-          <t>09:31:00</t>
-        </is>
-      </c>
-      <c r="X8" t="n">
-        <v>2311</v>
-      </c>
-      <c r="Y8" t="n">
-        <v>2.1782</v>
-      </c>
-      <c r="Z8" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AA8" t="inlineStr">
-        <is>
-          <t>LastTime</t>
-        </is>
-      </c>
-      <c r="AB8" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AC8" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AD8" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AE8" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AF8" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AG8" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AH8" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AI8" t="inlineStr">
-        <is>
-          <t>SL</t>
-        </is>
-      </c>
+      <c r="Q8" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
solo el 15 normal speed
</commit_message>
<xml_diff>
--- a/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
+++ b/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
@@ -664,16 +664,16 @@
         <v>200</v>
       </c>
       <c r="E4" t="n">
-        <v>29294.96</v>
+        <v>29294.95</v>
       </c>
       <c r="F4" t="n">
         <v>10</v>
       </c>
       <c r="G4" t="n">
-        <v>367</v>
+        <v>405</v>
       </c>
       <c r="H4" t="n">
-        <v>-145</v>
+        <v>-173</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -681,7 +681,7 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>4.64</v>
+        <v>4.6</v>
       </c>
       <c r="K4" t="n">
         <v>6</v>
@@ -734,7 +734,7 @@
         <v>2311</v>
       </c>
       <c r="Y4" t="n">
-        <v>2.1573</v>
+        <v>2.173</v>
       </c>
       <c r="Z4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
NORMAL SPEED MODULAR OK
</commit_message>
<xml_diff>
--- a/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
+++ b/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
@@ -669,45 +669,45 @@
         <v>200</v>
       </c>
       <c r="E4" t="n">
-        <v>29294.83</v>
+        <v>29294.39</v>
       </c>
       <c r="F4" t="n">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="G4" t="n">
-        <v>707</v>
+        <v>1853</v>
       </c>
       <c r="H4" t="n">
-        <v>-285</v>
+        <v>-351</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>A+ speed</t>
+          <t>normal speed</t>
         </is>
       </c>
       <c r="J4" t="n">
-        <v>15.22</v>
+        <v>4.71</v>
       </c>
       <c r="K4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L4" t="n">
-        <v>29248.75</v>
+        <v>29237.5</v>
       </c>
       <c r="M4" t="n">
-        <v>29223.75</v>
+        <v>29222.5</v>
       </c>
       <c r="N4" t="n">
-        <v>29193.75</v>
+        <v>29192.5</v>
       </c>
       <c r="O4" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="P4" t="n">
         <v>120</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>-100</v>
+        <v>37.5</v>
       </c>
       <c r="R4" t="inlineStr">
         <is>
@@ -716,14 +716,14 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>SELL1</t>
         </is>
       </c>
       <c r="T4" t="n">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="U4" t="n">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="V4" t="inlineStr">
         <is>
@@ -739,7 +739,7 @@
         <v>2311</v>
       </c>
       <c r="Y4" t="n">
-        <v>4.5981</v>
+        <v>15.9356</v>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
@@ -763,7 +763,7 @@
       </c>
       <c r="AD4" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="AE4" t="inlineStr">
@@ -788,7 +788,7 @@
       </c>
       <c r="AI4" t="inlineStr">
         <is>
-          <t>SL</t>
+          <t>EXIT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Nivele correcto de exit imprime exit price en excel pero  nos saca antes de que el precio toque la linea de exit
</commit_message>
<xml_diff>
--- a/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
+++ b/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
@@ -669,16 +669,16 @@
         <v>200</v>
       </c>
       <c r="E4" t="n">
-        <v>29294.39</v>
+        <v>29294.95</v>
       </c>
       <c r="F4" t="n">
-        <v>75</v>
+        <v>10</v>
       </c>
       <c r="G4" t="n">
-        <v>1853</v>
+        <v>404</v>
       </c>
       <c r="H4" t="n">
-        <v>-351</v>
+        <v>-174</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -686,19 +686,19 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>4.71</v>
+        <v>4.61</v>
       </c>
       <c r="K4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L4" t="n">
-        <v>29237.5</v>
+        <v>29253.75</v>
       </c>
       <c r="M4" t="n">
-        <v>29222.5</v>
+        <v>29238.75</v>
       </c>
       <c r="N4" t="n">
-        <v>29192.5</v>
+        <v>29208.75</v>
       </c>
       <c r="O4" t="n">
         <v>60</v>
@@ -707,7 +707,7 @@
         <v>120</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>37.5</v>
+        <v>10</v>
       </c>
       <c r="R4" t="inlineStr">
         <is>
@@ -720,14 +720,14 @@
         </is>
       </c>
       <c r="T4" t="n">
-        <v>145</v>
+        <v>0</v>
       </c>
       <c r="U4" t="n">
-        <v>75</v>
+        <v>20</v>
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>score-exporter-2026-05-22-first-break-sync</t>
+          <t>score-exporter-2026-05-25-fast-exit-40mfe</t>
         </is>
       </c>
       <c r="W4" t="inlineStr">
@@ -739,7 +739,7 @@
         <v>2311</v>
       </c>
       <c r="Y4" t="n">
-        <v>15.9356</v>
+        <v>2.1714</v>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
@@ -763,33 +763,36 @@
       </c>
       <c r="AD4" t="inlineStr">
         <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AE4" t="inlineStr">
+      <c r="AF4" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AF4" t="inlineStr">
+      <c r="AG4" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AG4" t="inlineStr">
+      <c r="AH4" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AH4" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
       <c r="AI4" t="inlineStr">
         <is>
           <t>EXIT</t>
         </is>
+      </c>
+      <c r="AJ4" t="n">
+        <v>29236.25</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
Trailing + normal speed 15-05-2026
</commit_message>
<xml_diff>
--- a/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
+++ b/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
@@ -672,13 +672,13 @@
         <v>29294.95</v>
       </c>
       <c r="F4" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="G4" t="n">
-        <v>404</v>
+        <v>410</v>
       </c>
       <c r="H4" t="n">
-        <v>-174</v>
+        <v>-176</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -686,19 +686,19 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>4.61</v>
+        <v>2.28</v>
       </c>
       <c r="K4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L4" t="n">
-        <v>29253.75</v>
+        <v>29255</v>
       </c>
       <c r="M4" t="n">
-        <v>29238.75</v>
+        <v>29240</v>
       </c>
       <c r="N4" t="n">
-        <v>29208.75</v>
+        <v>29210</v>
       </c>
       <c r="O4" t="n">
         <v>60</v>
@@ -707,7 +707,7 @@
         <v>120</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>10</v>
+        <v>120</v>
       </c>
       <c r="R4" t="inlineStr">
         <is>
@@ -723,11 +723,11 @@
         <v>0</v>
       </c>
       <c r="U4" t="n">
-        <v>20</v>
+        <v>135</v>
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>score-exporter-2026-05-25-fast-exit-40mfe</t>
+          <t>score-exporter-2026-05-25-fast-exit-half-mfe</t>
         </is>
       </c>
       <c r="W4" t="inlineStr">
@@ -739,7 +739,7 @@
         <v>2311</v>
       </c>
       <c r="Y4" t="n">
-        <v>2.1714</v>
+        <v>2.1962</v>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
@@ -758,41 +758,41 @@
       </c>
       <c r="AC4" t="inlineStr">
         <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AD4" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AE4" t="inlineStr">
+      <c r="AF4" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AF4" t="inlineStr">
+      <c r="AG4" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AG4" t="inlineStr">
+      <c r="AH4" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AH4" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
       <c r="AI4" t="inlineStr">
         <is>
-          <t>EXIT</t>
+          <t>TP</t>
         </is>
       </c>
       <c r="AJ4" t="n">
-        <v>29236.25</v>
+        <v>29210</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
creation of python single results
</commit_message>
<xml_diff>
--- a/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
+++ b/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
@@ -656,29 +656,29 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>29241.25</v>
+        <v>29551.25</v>
       </c>
       <c r="C4" t="n">
-        <v>29291.25</v>
+        <v>29620</v>
       </c>
       <c r="D4" t="n">
-        <v>200</v>
+        <v>275</v>
       </c>
       <c r="E4" t="n">
-        <v>29294.95</v>
+        <v>29557.51</v>
       </c>
       <c r="F4" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="G4" t="n">
-        <v>410</v>
+        <v>823</v>
       </c>
       <c r="H4" t="n">
-        <v>-176</v>
+        <v>-3</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -686,19 +686,19 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>2.28</v>
+        <v>2.52</v>
       </c>
       <c r="K4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L4" t="n">
-        <v>29255</v>
+        <v>29610</v>
       </c>
       <c r="M4" t="n">
-        <v>29240</v>
+        <v>29625</v>
       </c>
       <c r="N4" t="n">
-        <v>29210</v>
+        <v>29655</v>
       </c>
       <c r="O4" t="n">
         <v>60</v>
@@ -707,23 +707,23 @@
         <v>120</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>120</v>
+        <v>25</v>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>SELL1</t>
+          <t>BUY1</t>
         </is>
       </c>
       <c r="T4" t="n">
         <v>0</v>
       </c>
       <c r="U4" t="n">
-        <v>135</v>
+        <v>50</v>
       </c>
       <c r="V4" t="inlineStr">
         <is>
@@ -739,7 +739,7 @@
         <v>2311</v>
       </c>
       <c r="Y4" t="n">
-        <v>2.1962</v>
+        <v>7.9313</v>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
@@ -758,41 +758,41 @@
       </c>
       <c r="AC4" t="inlineStr">
         <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="AD4" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AE4" t="inlineStr">
+      <c r="AF4" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AF4" t="inlineStr">
+      <c r="AG4" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AG4" t="inlineStr">
+      <c r="AH4" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AH4" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
       <c r="AI4" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>EXIT</t>
         </is>
       </c>
       <c r="AJ4" t="n">
-        <v>29210</v>
+        <v>29631.25</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
regresamos el python a volumen 800 obligatorio
</commit_message>
<xml_diff>
--- a/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
+++ b/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
@@ -2,24 +2,24 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="1560" yWindow="1560" windowWidth="18900" windowHeight="10965" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="+0.##;-0.##;0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="\+0.##;\-0.##;0"/>
+    <numFmt numFmtId="165" formatCode="+0.##;-0.##;0"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,15 +28,33 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9EAF7"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -56,15 +74,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -427,23 +448,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:AJ11"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="1" max="3"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="7" max="8"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="9" max="12"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="16" customWidth="1" min="13" max="13"/>
-    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="14" max="17"/>
     <col width="10" customWidth="1" min="15" max="15"/>
     <col width="10" customWidth="1" min="16" max="16"/>
     <col width="10" customWidth="1" min="17" max="17"/>
@@ -472,182 +493,182 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>fecha</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>or_low</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>or_high</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>range</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>VWAP_entry</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>Body</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="G3" s="6" t="inlineStr">
         <is>
           <t>Volume_entry</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="H3" s="6" t="inlineStr">
         <is>
           <t>Delta_entry</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="I3" s="6" t="inlineStr">
         <is>
           <t>BreakOut_SPEED</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="J3" s="6" t="inlineStr">
         <is>
           <t>BreakOut_TICKS_PER_SEC</t>
         </is>
       </c>
-      <c r="K3" s="3" t="inlineStr">
+      <c r="K3" s="6" t="inlineStr">
         <is>
           <t>score total</t>
         </is>
       </c>
-      <c r="L3" s="3" t="inlineStr">
+      <c r="L3" s="6" t="inlineStr">
         <is>
           <t>SL_price</t>
         </is>
       </c>
-      <c r="M3" s="3" t="inlineStr">
+      <c r="M3" s="6" t="inlineStr">
         <is>
           <t>Entry_price</t>
         </is>
       </c>
-      <c r="N3" s="3" t="inlineStr">
+      <c r="N3" s="6" t="inlineStr">
         <is>
           <t>TP_price</t>
         </is>
       </c>
-      <c r="O3" s="3" t="inlineStr">
+      <c r="O3" s="6" t="inlineStr">
         <is>
           <t>SL_ticks</t>
         </is>
       </c>
-      <c r="P3" s="3" t="inlineStr">
+      <c r="P3" s="6" t="inlineStr">
         <is>
           <t>TP_ticks</t>
         </is>
       </c>
-      <c r="Q3" s="3" t="inlineStr">
+      <c r="Q3" s="6" t="inlineStr">
         <is>
           <t>result TP SL BE</t>
         </is>
       </c>
-      <c r="R3" s="3" t="inlineStr">
+      <c r="R3" s="6" t="inlineStr">
         <is>
           <t>Side</t>
         </is>
       </c>
-      <c r="S3" s="3" t="inlineStr">
+      <c r="S3" s="6" t="inlineStr">
         <is>
           <t>Speed_Profile</t>
         </is>
       </c>
-      <c r="T3" s="3" t="inlineStr">
+      <c r="T3" s="6" t="inlineStr">
         <is>
           <t>MAE_ticks</t>
         </is>
       </c>
-      <c r="U3" s="3" t="inlineStr">
+      <c r="U3" s="6" t="inlineStr">
         <is>
           <t>MFE_ticks</t>
         </is>
       </c>
-      <c r="V3" s="3" t="inlineStr">
+      <c r="V3" s="6" t="inlineStr">
         <is>
           <t>Exporter_VERSION</t>
         </is>
       </c>
-      <c r="W3" s="3" t="inlineStr">
+      <c r="W3" s="6" t="inlineStr">
         <is>
           <t>EntryTime_NY</t>
         </is>
       </c>
-      <c r="X3" s="3" t="inlineStr">
+      <c r="X3" s="6" t="inlineStr">
         <is>
           <t>EntryBar</t>
         </is>
       </c>
-      <c r="Y3" s="3" t="inlineStr">
+      <c r="Y3" s="6" t="inlineStr">
         <is>
           <t>Speed_Elapsed_SECONDS</t>
         </is>
       </c>
-      <c r="Z3" s="3" t="inlineStr">
+      <c r="Z3" s="6" t="inlineStr">
         <is>
           <t>Speed_Replay_Fallback</t>
         </is>
       </c>
-      <c r="AA3" s="3" t="inlineStr">
+      <c r="AA3" s="6" t="inlineStr">
         <is>
           <t>Speed_Timing_Source</t>
         </is>
       </c>
-      <c r="AB3" s="3" t="inlineStr">
+      <c r="AB3" s="6" t="inlineStr">
         <is>
           <t>Range_OK</t>
         </is>
       </c>
-      <c r="AC3" s="3" t="inlineStr">
+      <c r="AC3" s="6" t="inlineStr">
         <is>
           <t>Body_OK</t>
         </is>
       </c>
-      <c r="AD3" s="3" t="inlineStr">
+      <c r="AD3" s="6" t="inlineStr">
         <is>
           <t>Volume_OK</t>
         </is>
       </c>
-      <c r="AE3" s="3" t="inlineStr">
+      <c r="AE3" s="6" t="inlineStr">
         <is>
           <t>Delta_OK</t>
         </is>
       </c>
-      <c r="AF3" s="3" t="inlineStr">
+      <c r="AF3" s="6" t="inlineStr">
         <is>
           <t>Time_OK</t>
         </is>
       </c>
-      <c r="AG3" s="3" t="inlineStr">
+      <c r="AG3" s="6" t="inlineStr">
         <is>
           <t>VWAP_OK</t>
         </is>
       </c>
-      <c r="AH3" s="3" t="inlineStr">
+      <c r="AH3" s="6" t="inlineStr">
         <is>
           <t>Speed_OK</t>
         </is>
       </c>
-      <c r="AI3" s="3" t="inlineStr">
+      <c r="AI3" s="6" t="inlineStr">
         <is>
           <t>Result_Label</t>
         </is>
       </c>
-      <c r="AJ3" s="3" t="inlineStr">
+      <c r="AJ3" s="6" t="inlineStr">
         <is>
           <t>Exit_price</t>
         </is>
@@ -656,29 +677,29 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>29551.25</v>
+        <v>29252.5</v>
       </c>
       <c r="C4" t="n">
-        <v>29620</v>
+        <v>29288.75</v>
       </c>
       <c r="D4" t="n">
-        <v>275</v>
+        <v>145</v>
       </c>
       <c r="E4" t="n">
-        <v>29557.51</v>
+        <v>29321.36</v>
       </c>
       <c r="F4" t="n">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="G4" t="n">
-        <v>823</v>
+        <v>1113</v>
       </c>
       <c r="H4" t="n">
-        <v>-3</v>
+        <v>-175</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -686,19 +707,19 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>2.52</v>
+        <v>2.08</v>
       </c>
       <c r="K4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L4" t="n">
-        <v>29610</v>
+        <v>29258.75</v>
       </c>
       <c r="M4" t="n">
-        <v>29625</v>
+        <v>29243.75</v>
       </c>
       <c r="N4" t="n">
-        <v>29655</v>
+        <v>29213.75</v>
       </c>
       <c r="O4" t="n">
         <v>60</v>
@@ -706,24 +727,24 @@
       <c r="P4" t="n">
         <v>120</v>
       </c>
-      <c r="Q4" s="4" t="n">
-        <v>25</v>
+      <c r="Q4" s="7" t="n">
+        <v>30</v>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>BUY1</t>
+          <t>SELL1</t>
         </is>
       </c>
       <c r="T4" t="n">
         <v>0</v>
       </c>
       <c r="U4" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="V4" t="inlineStr">
         <is>
@@ -739,7 +760,7 @@
         <v>2311</v>
       </c>
       <c r="Y4" t="n">
-        <v>7.9313</v>
+        <v>16.8109</v>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
@@ -768,7 +789,7 @@
       </c>
       <c r="AE4" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="AF4" t="inlineStr">
@@ -792,7 +813,7 @@
         </is>
       </c>
       <c r="AJ4" t="n">
-        <v>29631.25</v>
+        <v>29236.25</v>
       </c>
     </row>
     <row r="5">
@@ -807,7 +828,13 @@
     <row r="8">
       <c r="Q8" s="4" t="n"/>
     </row>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11">
+      <c r="F11" s="5" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
ya imprime el 21
</commit_message>
<xml_diff>
--- a/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
+++ b/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
@@ -677,29 +677,29 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>29252.5</v>
+        <v>29193.75</v>
       </c>
       <c r="C4" t="n">
-        <v>29288.75</v>
+        <v>29250</v>
       </c>
       <c r="D4" t="n">
-        <v>145</v>
+        <v>225</v>
       </c>
       <c r="E4" t="n">
-        <v>29321.36</v>
+        <v>29270.18</v>
       </c>
       <c r="F4" t="n">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="G4" t="n">
-        <v>1113</v>
+        <v>833</v>
       </c>
       <c r="H4" t="n">
-        <v>-175</v>
+        <v>215</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -707,19 +707,19 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>2.08</v>
+        <v>3.5</v>
       </c>
       <c r="K4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L4" t="n">
-        <v>29258.75</v>
+        <v>29238.75</v>
       </c>
       <c r="M4" t="n">
-        <v>29243.75</v>
+        <v>29253.75</v>
       </c>
       <c r="N4" t="n">
-        <v>29213.75</v>
+        <v>29283.75</v>
       </c>
       <c r="O4" t="n">
         <v>60</v>
@@ -728,23 +728,23 @@
         <v>120</v>
       </c>
       <c r="Q4" s="7" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>SELL1</t>
+          <t>BUY1</t>
         </is>
       </c>
       <c r="T4" t="n">
         <v>0</v>
       </c>
       <c r="U4" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="V4" t="inlineStr">
         <is>
@@ -753,14 +753,14 @@
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>09:31:00</t>
+          <t>09:52:00</t>
         </is>
       </c>
       <c r="X4" t="n">
-        <v>2311</v>
+        <v>2332</v>
       </c>
       <c r="Y4" t="n">
-        <v>16.8109</v>
+        <v>4.287</v>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
@@ -799,21 +799,21 @@
       </c>
       <c r="AG4" t="inlineStr">
         <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AH4" t="inlineStr">
+        <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AH4" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
       <c r="AI4" t="inlineStr">
         <is>
           <t>EXIT</t>
         </is>
       </c>
       <c r="AJ4" t="n">
-        <v>29236.25</v>
+        <v>29258.75</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
ES POSIBLE CORRER A X20 sin afectar los resultados
</commit_message>
<xml_diff>
--- a/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
+++ b/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
@@ -690,16 +690,16 @@
         <v>220</v>
       </c>
       <c r="E4" t="n">
-        <v>26835.32</v>
+        <v>26835.98</v>
       </c>
       <c r="F4" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="G4" t="n">
-        <v>1649</v>
+        <v>1071</v>
       </c>
       <c r="H4" t="n">
-        <v>-401</v>
+        <v>-273</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -707,19 +707,19 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>2.46</v>
+        <v>2.01</v>
       </c>
       <c r="K4" t="n">
         <v>7</v>
       </c>
       <c r="L4" t="n">
-        <v>26772.5</v>
+        <v>26780</v>
       </c>
       <c r="M4" t="n">
-        <v>26757.5</v>
+        <v>26765</v>
       </c>
       <c r="N4" t="n">
-        <v>26742.5</v>
+        <v>26750</v>
       </c>
       <c r="O4" t="n">
         <v>60</v>
@@ -741,7 +741,7 @@
         </is>
       </c>
       <c r="T4" t="n">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="U4" t="n">
         <v>55</v>
@@ -760,7 +760,7 @@
         <v>2310</v>
       </c>
       <c r="Y4" t="n">
-        <v>24.4085</v>
+        <v>14.9157</v>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
@@ -813,7 +813,7 @@
         </is>
       </c>
       <c r="AJ4" t="n">
-        <v>26750.63</v>
+        <v>26758.13</v>
       </c>
     </row>
     <row r="5">
@@ -832,16 +832,16 @@
         <v>165</v>
       </c>
       <c r="E5" t="n">
-        <v>26841.85</v>
+        <v>26841.86</v>
       </c>
       <c r="F5" t="n">
         <v>70</v>
       </c>
       <c r="G5" t="n">
-        <v>1313</v>
+        <v>1256</v>
       </c>
       <c r="H5" t="n">
-        <v>-117</v>
+        <v>-96</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -902,7 +902,7 @@
         <v>2312</v>
       </c>
       <c r="Y5" t="n">
-        <v>33.3476</v>
+        <v>33.2876</v>
       </c>
       <c r="Z5" t="inlineStr">
         <is>
@@ -977,13 +977,13 @@
         <v>26995.97</v>
       </c>
       <c r="F6" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="G6" t="n">
-        <v>803</v>
+        <v>800</v>
       </c>
       <c r="H6" t="n">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -991,19 +991,19 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>2.01</v>
+        <v>2.33</v>
       </c>
       <c r="K6" t="n">
         <v>7</v>
       </c>
       <c r="L6" t="n">
-        <v>27050</v>
+        <v>27051.25</v>
       </c>
       <c r="M6" t="n">
-        <v>27065</v>
+        <v>27066.25</v>
       </c>
       <c r="N6" t="n">
-        <v>27080</v>
+        <v>27081.25</v>
       </c>
       <c r="O6" t="n">
         <v>60</v>
@@ -1012,7 +1012,7 @@
         <v>60</v>
       </c>
       <c r="Q6" s="7" t="n">
-        <v>60</v>
+        <v>25</v>
       </c>
       <c r="R6" t="inlineStr">
         <is>
@@ -1025,10 +1025,10 @@
         </is>
       </c>
       <c r="T6" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="U6" t="n">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="V6" t="inlineStr">
         <is>
@@ -1044,7 +1044,7 @@
         <v>2326</v>
       </c>
       <c r="Y6" t="n">
-        <v>17.435</v>
+        <v>17.1461</v>
       </c>
       <c r="Z6" t="inlineStr">
         <is>
@@ -1093,11 +1093,11 @@
       </c>
       <c r="AI6" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>EXIT</t>
         </is>
       </c>
       <c r="AJ6" t="n">
-        <v>27080</v>
+        <v>27072.5</v>
       </c>
     </row>
     <row r="7">
@@ -1406,10 +1406,10 @@
         <v>50</v>
       </c>
       <c r="G9" t="n">
-        <v>1004</v>
+        <v>935</v>
       </c>
       <c r="H9" t="n">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -1417,7 +1417,7 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>2.05</v>
+        <v>2.15</v>
       </c>
       <c r="K9" t="n">
         <v>5</v>
@@ -1470,7 +1470,7 @@
         <v>2318</v>
       </c>
       <c r="Y9" t="n">
-        <v>24.3548</v>
+        <v>23.2757</v>
       </c>
       <c r="Z9" t="inlineStr">
         <is>
@@ -1542,13 +1542,13 @@
         <v>270</v>
       </c>
       <c r="E10" t="n">
-        <v>27241.74</v>
+        <v>27241.75</v>
       </c>
       <c r="F10" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G10" t="n">
-        <v>809</v>
+        <v>805</v>
       </c>
       <c r="H10" t="n">
         <v>-89</v>
@@ -1559,19 +1559,19 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>3.05</v>
+        <v>2.33</v>
       </c>
       <c r="K10" t="n">
         <v>7</v>
       </c>
       <c r="L10" t="n">
-        <v>27161.25</v>
+        <v>27162.5</v>
       </c>
       <c r="M10" t="n">
-        <v>27146.25</v>
+        <v>27147.5</v>
       </c>
       <c r="N10" t="n">
-        <v>27131.25</v>
+        <v>27132.5</v>
       </c>
       <c r="O10" t="n">
         <v>60</v>
@@ -1580,7 +1580,7 @@
         <v>60</v>
       </c>
       <c r="Q10" s="7" t="n">
-        <v>-60</v>
+        <v>20</v>
       </c>
       <c r="R10" t="inlineStr">
         <is>
@@ -1593,10 +1593,10 @@
         </is>
       </c>
       <c r="T10" t="n">
-        <v>65</v>
+        <v>0</v>
       </c>
       <c r="U10" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="V10" t="inlineStr">
         <is>
@@ -1612,7 +1612,7 @@
         <v>2311</v>
       </c>
       <c r="Y10" t="n">
-        <v>6.5608</v>
+        <v>6.4496</v>
       </c>
       <c r="Z10" t="inlineStr">
         <is>
@@ -1661,11 +1661,11 @@
       </c>
       <c r="AI10" t="inlineStr">
         <is>
-          <t>SL</t>
+          <t>EXIT</t>
         </is>
       </c>
       <c r="AJ10" t="n">
-        <v>27161.25</v>
+        <v>27142.5</v>
       </c>
     </row>
     <row r="11">
@@ -1684,16 +1684,16 @@
         <v>280</v>
       </c>
       <c r="E11" t="n">
-        <v>27385.43</v>
+        <v>27385.42</v>
       </c>
       <c r="F11" s="5" t="n">
         <v>25</v>
       </c>
       <c r="G11" t="n">
-        <v>993</v>
+        <v>970</v>
       </c>
       <c r="H11" t="n">
-        <v>-107</v>
+        <v>-110</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -1701,7 +1701,7 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>2.11</v>
+        <v>2.13</v>
       </c>
       <c r="K11" t="n">
         <v>5</v>
@@ -1735,7 +1735,7 @@
         </is>
       </c>
       <c r="T11" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="U11" t="n">
         <v>50</v>
@@ -1754,7 +1754,7 @@
         <v>2311</v>
       </c>
       <c r="Y11" t="n">
-        <v>11.8404</v>
+        <v>11.723</v>
       </c>
       <c r="Z11" t="inlineStr">
         <is>
@@ -1826,16 +1826,16 @@
         <v>190</v>
       </c>
       <c r="E12" t="n">
-        <v>27598.28</v>
+        <v>27598.29</v>
       </c>
       <c r="F12" t="n">
         <v>25</v>
       </c>
       <c r="G12" t="n">
-        <v>821</v>
+        <v>826</v>
       </c>
       <c r="H12" t="n">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -1843,7 +1843,7 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>3.3</v>
+        <v>3.29</v>
       </c>
       <c r="K12" t="n">
         <v>7</v>
@@ -1877,10 +1877,10 @@
         </is>
       </c>
       <c r="T12" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="U12" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="V12" t="inlineStr">
         <is>
@@ -1896,7 +1896,7 @@
         <v>2311</v>
       </c>
       <c r="Y12" t="n">
-        <v>7.5819</v>
+        <v>7.6086</v>
       </c>
       <c r="Z12" t="inlineStr">
         <is>
@@ -1968,16 +1968,16 @@
         <v>150</v>
       </c>
       <c r="E13" t="n">
-        <v>27837</v>
+        <v>27837.01</v>
       </c>
       <c r="F13" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="G13" t="n">
-        <v>1336</v>
+        <v>1331</v>
       </c>
       <c r="H13" t="n">
-        <v>-28</v>
+        <v>-25</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -1985,19 +1985,19 @@
         </is>
       </c>
       <c r="J13" t="n">
-        <v>2.52</v>
+        <v>2.25</v>
       </c>
       <c r="K13" t="n">
         <v>7</v>
       </c>
       <c r="L13" t="n">
-        <v>27841.25</v>
+        <v>27842.5</v>
       </c>
       <c r="M13" t="n">
-        <v>27826.25</v>
+        <v>27827.5</v>
       </c>
       <c r="N13" t="n">
-        <v>27811.25</v>
+        <v>27812.5</v>
       </c>
       <c r="O13" t="n">
         <v>60</v>
@@ -2019,7 +2019,7 @@
         </is>
       </c>
       <c r="T13" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="U13" t="n">
         <v>60</v>
@@ -2038,7 +2038,7 @@
         <v>2311</v>
       </c>
       <c r="Y13" t="n">
-        <v>17.8261</v>
+        <v>17.7766</v>
       </c>
       <c r="Z13" t="inlineStr">
         <is>
@@ -2091,7 +2091,7 @@
         </is>
       </c>
       <c r="AJ13" t="n">
-        <v>27811.25</v>
+        <v>27812.5</v>
       </c>
     </row>
     <row r="14">
@@ -2113,13 +2113,13 @@
         <v>27935.71</v>
       </c>
       <c r="F14" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="G14" t="n">
-        <v>846</v>
+        <v>851</v>
       </c>
       <c r="H14" t="n">
-        <v>-138</v>
+        <v>-139</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -2127,19 +2127,19 @@
         </is>
       </c>
       <c r="J14" t="n">
-        <v>2.75</v>
+        <v>3.65</v>
       </c>
       <c r="K14" t="n">
         <v>5</v>
       </c>
       <c r="L14" t="n">
-        <v>27997.5</v>
+        <v>27996.25</v>
       </c>
       <c r="M14" t="n">
-        <v>27982.5</v>
+        <v>27981.25</v>
       </c>
       <c r="N14" t="n">
-        <v>27967.5</v>
+        <v>27966.25</v>
       </c>
       <c r="O14" t="n">
         <v>60</v>
@@ -2148,7 +2148,7 @@
         <v>60</v>
       </c>
       <c r="Q14" s="7" t="n">
-        <v>22.5</v>
+        <v>20</v>
       </c>
       <c r="R14" t="inlineStr">
         <is>
@@ -2161,10 +2161,10 @@
         </is>
       </c>
       <c r="T14" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="U14" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="V14" t="inlineStr">
         <is>
@@ -2180,7 +2180,7 @@
         <v>2310</v>
       </c>
       <c r="Y14" t="n">
-        <v>5.4566</v>
+        <v>5.4765</v>
       </c>
       <c r="Z14" t="inlineStr">
         <is>
@@ -2233,7 +2233,7 @@
         </is>
       </c>
       <c r="AJ14" t="n">
-        <v>27976.88</v>
+        <v>27976.25</v>
       </c>
     </row>
     <row r="15">
@@ -2252,16 +2252,16 @@
         <v>225</v>
       </c>
       <c r="E15" t="n">
-        <v>28455.82</v>
+        <v>28455.83</v>
       </c>
       <c r="F15" t="n">
         <v>25</v>
       </c>
       <c r="G15" t="n">
-        <v>845</v>
+        <v>835</v>
       </c>
       <c r="H15" t="n">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -2269,7 +2269,7 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>2.11</v>
+        <v>2.13</v>
       </c>
       <c r="K15" t="n">
         <v>5</v>
@@ -2322,7 +2322,7 @@
         <v>2313</v>
       </c>
       <c r="Y15" t="n">
-        <v>11.8532</v>
+        <v>11.7309</v>
       </c>
       <c r="Z15" t="inlineStr">
         <is>
@@ -2397,13 +2397,13 @@
         <v>28745.29</v>
       </c>
       <c r="F16" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="G16" t="n">
-        <v>810</v>
+        <v>801</v>
       </c>
       <c r="H16" t="n">
-        <v>218</v>
+        <v>209</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -2411,19 +2411,19 @@
         </is>
       </c>
       <c r="J16" t="n">
-        <v>4.85</v>
+        <v>4.21</v>
       </c>
       <c r="K16" t="n">
         <v>7</v>
       </c>
       <c r="L16" t="n">
-        <v>28781.25</v>
+        <v>28780</v>
       </c>
       <c r="M16" t="n">
-        <v>28796.25</v>
+        <v>28795</v>
       </c>
       <c r="N16" t="n">
-        <v>28811.25</v>
+        <v>28810</v>
       </c>
       <c r="O16" t="n">
         <v>60</v>
@@ -2448,7 +2448,7 @@
         <v>60</v>
       </c>
       <c r="U16" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="V16" t="inlineStr">
         <is>
@@ -2464,7 +2464,7 @@
         <v>2335</v>
       </c>
       <c r="Y16" t="n">
-        <v>7.223</v>
+        <v>7.1334</v>
       </c>
       <c r="Z16" t="inlineStr">
         <is>
@@ -2517,7 +2517,7 @@
         </is>
       </c>
       <c r="AJ16" t="n">
-        <v>28781.25</v>
+        <v>28780</v>
       </c>
     </row>
     <row r="17">
@@ -2542,10 +2542,10 @@
         <v>50</v>
       </c>
       <c r="G17" t="n">
-        <v>1576</v>
+        <v>1573</v>
       </c>
       <c r="H17" t="n">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -2553,7 +2553,7 @@
         </is>
       </c>
       <c r="J17" t="n">
-        <v>2.18</v>
+        <v>2.19</v>
       </c>
       <c r="K17" t="n">
         <v>7</v>
@@ -2587,7 +2587,7 @@
         </is>
       </c>
       <c r="T17" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="U17" t="n">
         <v>65</v>
@@ -2606,7 +2606,7 @@
         <v>2311</v>
       </c>
       <c r="Y17" t="n">
-        <v>22.9021</v>
+        <v>22.8326</v>
       </c>
       <c r="Z17" t="inlineStr">
         <is>
@@ -2732,7 +2732,7 @@
         <v>15</v>
       </c>
       <c r="U18" t="n">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="V18" t="inlineStr">
         <is>
@@ -2874,7 +2874,7 @@
         <v>60</v>
       </c>
       <c r="U19" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="V19" t="inlineStr">
         <is>
@@ -2968,10 +2968,10 @@
         <v>35</v>
       </c>
       <c r="G20" t="n">
-        <v>1113</v>
+        <v>1116</v>
       </c>
       <c r="H20" t="n">
-        <v>-175</v>
+        <v>-176</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -3032,7 +3032,7 @@
         <v>2311</v>
       </c>
       <c r="Y20" t="n">
-        <v>16.8109</v>
+        <v>16.8195</v>
       </c>
       <c r="Z20" t="inlineStr">
         <is>
@@ -3104,16 +3104,16 @@
         <v>130</v>
       </c>
       <c r="E21" t="n">
-        <v>29543.5</v>
+        <v>29543.51</v>
       </c>
       <c r="F21" t="n">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="G21" t="n">
-        <v>806</v>
+        <v>802</v>
       </c>
       <c r="H21" t="n">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -3121,19 +3121,19 @@
         </is>
       </c>
       <c r="J21" t="n">
-        <v>9.960000000000001</v>
+        <v>10.97</v>
       </c>
       <c r="K21" t="n">
         <v>5</v>
       </c>
       <c r="L21" t="n">
-        <v>29488.75</v>
+        <v>29490</v>
       </c>
       <c r="M21" t="n">
-        <v>29513.75</v>
+        <v>29515</v>
       </c>
       <c r="N21" t="n">
-        <v>29543.75</v>
+        <v>29545</v>
       </c>
       <c r="O21" t="n">
         <v>100</v>
@@ -3155,7 +3155,7 @@
         </is>
       </c>
       <c r="T21" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="U21" t="n">
         <v>120</v>
@@ -3174,7 +3174,7 @@
         <v>2312</v>
       </c>
       <c r="Y21" t="n">
-        <v>6.026</v>
+        <v>5.9247</v>
       </c>
       <c r="Z21" t="inlineStr">
         <is>
@@ -3227,7 +3227,7 @@
         </is>
       </c>
       <c r="AJ21" t="n">
-        <v>29543.75</v>
+        <v>29545</v>
       </c>
     </row>
     <row r="22">
@@ -3246,16 +3246,16 @@
         <v>200</v>
       </c>
       <c r="E22" t="n">
-        <v>29294.79</v>
+        <v>29294.78</v>
       </c>
       <c r="F22" t="n">
         <v>90</v>
       </c>
       <c r="G22" t="n">
-        <v>808</v>
+        <v>814</v>
       </c>
       <c r="H22" t="n">
-        <v>-354</v>
+        <v>-358</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -3263,7 +3263,7 @@
         </is>
       </c>
       <c r="J22" t="n">
-        <v>18.2</v>
+        <v>18.05</v>
       </c>
       <c r="K22" t="n">
         <v>7</v>
@@ -3316,7 +3316,7 @@
         <v>2311</v>
       </c>
       <c r="Y22" t="n">
-        <v>4.9439</v>
+        <v>4.9856</v>
       </c>
       <c r="Z22" t="inlineStr">
         <is>
@@ -3391,13 +3391,13 @@
         <v>29211.89</v>
       </c>
       <c r="F23" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="G23" t="n">
-        <v>802</v>
+        <v>800</v>
       </c>
       <c r="H23" t="n">
-        <v>-158</v>
+        <v>-160</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -3405,19 +3405,19 @@
         </is>
       </c>
       <c r="J23" t="n">
-        <v>3.88</v>
+        <v>4.69</v>
       </c>
       <c r="K23" t="n">
         <v>5</v>
       </c>
       <c r="L23" t="n">
-        <v>29298.75</v>
+        <v>29296.25</v>
       </c>
       <c r="M23" t="n">
-        <v>29283.75</v>
+        <v>29281.25</v>
       </c>
       <c r="N23" t="n">
-        <v>29268.75</v>
+        <v>29266.25</v>
       </c>
       <c r="O23" t="n">
         <v>60</v>
@@ -3458,7 +3458,7 @@
         <v>2313</v>
       </c>
       <c r="Y23" t="n">
-        <v>12.8979</v>
+        <v>12.781</v>
       </c>
       <c r="Z23" t="inlineStr">
         <is>
@@ -3511,7 +3511,7 @@
         </is>
       </c>
       <c r="AJ23" t="n">
-        <v>29298.75</v>
+        <v>29296.25</v>
       </c>
     </row>
     <row r="24">
@@ -3536,10 +3536,10 @@
         <v>40</v>
       </c>
       <c r="G24" t="n">
-        <v>820</v>
+        <v>805</v>
       </c>
       <c r="H24" t="n">
-        <v>124</v>
+        <v>111</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -3547,7 +3547,7 @@
         </is>
       </c>
       <c r="J24" t="n">
-        <v>2.77</v>
+        <v>2.78</v>
       </c>
       <c r="K24" t="n">
         <v>6</v>
@@ -3600,7 +3600,7 @@
         <v>2312</v>
       </c>
       <c r="Y24" t="n">
-        <v>14.4236</v>
+        <v>14.4064</v>
       </c>
       <c r="Z24" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
TIME_OVER +  NO_TRADE y GENERA EL EXCEL EN 90 SEGUNDOS
</commit_message>
<xml_diff>
--- a/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
+++ b/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
@@ -656,191 +656,61 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>29460</v>
-      </c>
-      <c r="C4" t="n">
-        <v>29492.5</v>
-      </c>
-      <c r="D4" t="n">
-        <v>130</v>
-      </c>
-      <c r="E4" t="n">
-        <v>29543.47</v>
-      </c>
-      <c r="F4" t="n">
-        <v>55</v>
-      </c>
-      <c r="G4" t="n">
-        <v>881</v>
-      </c>
-      <c r="H4" t="n">
-        <v>241</v>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>A+ speed</t>
-        </is>
-      </c>
-      <c r="J4" t="n">
-        <v>8</v>
-      </c>
-      <c r="K4" t="n">
-        <v>7</v>
-      </c>
-      <c r="L4" t="n">
-        <v>29497.5</v>
-      </c>
-      <c r="M4" t="n">
-        <v>29512.5</v>
-      </c>
-      <c r="N4" t="n">
-        <v>29527.5</v>
-      </c>
-      <c r="O4" t="n">
-        <v>60</v>
-      </c>
-      <c r="P4" t="n">
-        <v>60</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>29527.5</v>
-      </c>
-      <c r="R4" s="4" t="n">
-        <v>60</v>
-      </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>POTENTIAL_RUNNER</t>
-        </is>
-      </c>
-      <c r="U4" t="n">
-        <v>0</v>
-      </c>
-      <c r="V4" t="n">
-        <v>70</v>
-      </c>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t>score-exporter-2026-05-27-strict-speed-window</t>
-        </is>
-      </c>
-      <c r="X4" t="inlineStr">
-        <is>
-          <t>09:32:00</t>
-        </is>
-      </c>
-      <c r="Y4" t="n">
-        <v>2312</v>
-      </c>
-      <c r="Z4" t="n">
-        <v>6.871</v>
-      </c>
-      <c r="AA4" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AB4" t="inlineStr">
-        <is>
-          <t>LastTime</t>
-        </is>
-      </c>
-      <c r="AC4" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AD4" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AE4" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AF4" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AG4" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AH4" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AI4" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AJ4" t="inlineStr">
-        <is>
-          <t>TP</t>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="R4" s="4" t="inlineStr">
+        <is>
+          <t>NO_TRADE</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>29241.25</v>
+        <v>27176.25</v>
       </c>
       <c r="C5" t="n">
-        <v>29291.25</v>
+        <v>27223.75</v>
       </c>
       <c r="D5" t="n">
-        <v>200</v>
+        <v>190</v>
       </c>
       <c r="E5" t="n">
-        <v>29294.78</v>
+        <v>27208.66</v>
       </c>
       <c r="F5" t="n">
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="G5" t="n">
-        <v>825</v>
+        <v>1287</v>
       </c>
       <c r="H5" t="n">
-        <v>-353</v>
+        <v>173</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>A+ speed</t>
+          <t>normal speed</t>
         </is>
       </c>
       <c r="J5" t="n">
-        <v>17.51</v>
+        <v>2.06</v>
       </c>
       <c r="K5" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="L5" t="n">
-        <v>29233.75</v>
+        <v>27228.75</v>
       </c>
       <c r="M5" t="n">
-        <v>29218.75</v>
+        <v>27243.75</v>
       </c>
       <c r="N5" t="n">
-        <v>29203.75</v>
+        <v>27258.75</v>
       </c>
       <c r="O5" t="n">
         <v>60</v>
@@ -849,26 +719,26 @@
         <v>60</v>
       </c>
       <c r="Q5" t="n">
-        <v>29203.75</v>
+        <v>27228.75</v>
       </c>
       <c r="R5" s="4" t="n">
+        <v>-60</v>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>SCALP_NORMAL</t>
+        </is>
+      </c>
+      <c r="U5" t="n">
         <v>60</v>
       </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>POTENTIAL_RUNNER</t>
-        </is>
-      </c>
-      <c r="U5" t="n">
-        <v>25</v>
-      </c>
       <c r="V5" t="n">
-        <v>60</v>
+        <v>10</v>
       </c>
       <c r="W5" t="inlineStr">
         <is>
@@ -877,14 +747,14 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>09:31:00</t>
+          <t>09:34:00</t>
         </is>
       </c>
       <c r="Y5" t="n">
-        <v>2311</v>
+        <v>2314</v>
       </c>
       <c r="Z5" t="n">
-        <v>5.1395</v>
+        <v>36.4114</v>
       </c>
       <c r="AA5" t="inlineStr">
         <is>
@@ -933,36 +803,36 @@
       </c>
       <c r="AJ5" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>SL</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>29305</v>
+        <v>27363.75</v>
       </c>
       <c r="C6" t="n">
-        <v>29356.25</v>
+        <v>27435</v>
       </c>
       <c r="D6" t="n">
-        <v>205</v>
+        <v>285</v>
       </c>
       <c r="E6" t="n">
-        <v>29211.89</v>
+        <v>27430.76</v>
       </c>
       <c r="F6" t="n">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="G6" t="n">
-        <v>802</v>
+        <v>843</v>
       </c>
       <c r="H6" t="n">
-        <v>-158</v>
+        <v>-169</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -970,19 +840,19 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>3.88</v>
+        <v>2.01</v>
       </c>
       <c r="K6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L6" t="n">
-        <v>29298.75</v>
+        <v>27370</v>
       </c>
       <c r="M6" t="n">
-        <v>29283.75</v>
+        <v>27355</v>
       </c>
       <c r="N6" t="n">
-        <v>29268.75</v>
+        <v>27340</v>
       </c>
       <c r="O6" t="n">
         <v>60</v>
@@ -991,7 +861,7 @@
         <v>60</v>
       </c>
       <c r="Q6" t="n">
-        <v>29298.75</v>
+        <v>27370</v>
       </c>
       <c r="R6" s="4" t="n">
         <v>-60</v>
@@ -1010,7 +880,7 @@
         <v>60</v>
       </c>
       <c r="V6" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="W6" t="inlineStr">
         <is>
@@ -1019,14 +889,14 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>09:33:00</t>
+          <t>09:36:00</t>
         </is>
       </c>
       <c r="Y6" t="n">
-        <v>2313</v>
+        <v>2316</v>
       </c>
       <c r="Z6" t="n">
-        <v>12.8979</v>
+        <v>17.4372</v>
       </c>
       <c r="AA6" t="inlineStr">
         <is>
@@ -1065,7 +935,7 @@
       </c>
       <c r="AH6" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="AI6" t="inlineStr">

</xml_diff>

<commit_message>
Velocidad X10 BreakOUT speed OK TIMEOVER OK
</commit_message>
<xml_diff>
--- a/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
+++ b/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ6"/>
+  <dimension ref="A1:AJ25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -463,11 +463,11 @@
     </row>
     <row r="2">
       <c r="A2" s="1">
-        <f>IF((COUNTIF(R4:R6,"&gt;0")+COUNTIF(R4:R6,"&lt;0"))=0,"",COUNTIF(R4:R6,"&gt;0")/(COUNTIF(R4:R6,"&gt;0")+COUNTIF(R4:R6,"&lt;0")))</f>
+        <f>IF((COUNTIF(R4:R25,"&gt;0")+COUNTIF(R4:R25,"&lt;0"))=0,"",COUNTIF(R4:R25,"&gt;0")/(COUNTIF(R4:R25,"&gt;0")+COUNTIF(R4:R25,"&lt;0")))</f>
         <v/>
       </c>
       <c r="B2" s="2">
-        <f>IF(ABS(SUMIF(R4:R6,"&lt;0",R4:R6))=0,IF(SUMIF(R4:R6,"&gt;0",R4:R6)&gt;0,"INF",""),SUMIF(R4:R6,"&gt;0",R4:R6)/ABS(SUMIF(R4:R6,"&lt;0",R4:R6)))</f>
+        <f>IF(ABS(SUMIF(R4:R25,"&lt;0",R4:R25))=0,IF(SUMIF(R4:R25,"&gt;0",R4:R25)&gt;0,"INF",""),SUMIF(R4:R25,"&gt;0",R4:R25)/ABS(SUMIF(R4:R25,"&lt;0",R4:R25)))</f>
         <v/>
       </c>
     </row>
@@ -656,41 +656,171 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
-        </is>
-      </c>
-      <c r="R4" s="4" t="inlineStr">
-        <is>
-          <t>NO_TRADE</t>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>26772.5</v>
+      </c>
+      <c r="C4" t="n">
+        <v>26827.5</v>
+      </c>
+      <c r="D4" t="n">
+        <v>220</v>
+      </c>
+      <c r="E4" t="n">
+        <v>26835.26</v>
+      </c>
+      <c r="F4" t="n">
+        <v>60</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1693</v>
+      </c>
+      <c r="H4" t="n">
+        <v>-445</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>normal speed</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>2.46</v>
+      </c>
+      <c r="K4" t="n">
+        <v>8</v>
+      </c>
+      <c r="L4" t="n">
+        <v>26772.5</v>
+      </c>
+      <c r="M4" t="n">
+        <v>26757.5</v>
+      </c>
+      <c r="N4" t="n">
+        <v>26742.5</v>
+      </c>
+      <c r="O4" t="n">
+        <v>60</v>
+      </c>
+      <c r="P4" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>26742.5</v>
+      </c>
+      <c r="R4" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>SCALP_NORMAL</t>
+        </is>
+      </c>
+      <c r="U4" t="n">
+        <v>45</v>
+      </c>
+      <c r="V4" t="n">
+        <v>65</v>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-time-over-0940-ny</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>09:31:00</t>
+        </is>
+      </c>
+      <c r="Y4" t="n">
+        <v>2310</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>24.4173</v>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ4" t="inlineStr">
+        <is>
+          <t>TP</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>27176.25</v>
+        <v>26852.5</v>
       </c>
       <c r="C5" t="n">
-        <v>27223.75</v>
+        <v>26893.75</v>
       </c>
       <c r="D5" t="n">
-        <v>190</v>
+        <v>165</v>
       </c>
       <c r="E5" t="n">
-        <v>27208.66</v>
+        <v>26841.85</v>
       </c>
       <c r="F5" t="n">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="G5" t="n">
-        <v>1287</v>
+        <v>1306</v>
       </c>
       <c r="H5" t="n">
-        <v>173</v>
+        <v>-116</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -698,19 +828,19 @@
         </is>
       </c>
       <c r="J5" t="n">
-        <v>2.06</v>
+        <v>2.1</v>
       </c>
       <c r="K5" t="n">
         <v>8</v>
       </c>
       <c r="L5" t="n">
-        <v>27228.75</v>
+        <v>26836.25</v>
       </c>
       <c r="M5" t="n">
-        <v>27243.75</v>
+        <v>26821.25</v>
       </c>
       <c r="N5" t="n">
-        <v>27258.75</v>
+        <v>26806.25</v>
       </c>
       <c r="O5" t="n">
         <v>60</v>
@@ -719,14 +849,14 @@
         <v>60</v>
       </c>
       <c r="Q5" t="n">
-        <v>27228.75</v>
+        <v>26836.25</v>
       </c>
       <c r="R5" s="4" t="n">
         <v>-60</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -735,26 +865,26 @@
         </is>
       </c>
       <c r="U5" t="n">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="V5" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>score-exporter-2026-05-27-strict-speed-window</t>
+          <t>score-exporter-2026-05-30-time-over-0940-ny</t>
         </is>
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>09:34:00</t>
+          <t>09:33:00</t>
         </is>
       </c>
       <c r="Y5" t="n">
-        <v>2314</v>
+        <v>2312</v>
       </c>
       <c r="Z5" t="n">
-        <v>36.4114</v>
+        <v>33.3088</v>
       </c>
       <c r="AA5" t="inlineStr">
         <is>
@@ -810,140 +940,2535 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>26965</v>
+      </c>
+      <c r="C6" t="n">
+        <v>27016.25</v>
+      </c>
+      <c r="D6" t="n">
+        <v>205</v>
+      </c>
+      <c r="R6" s="4" t="inlineStr">
+        <is>
+          <t>TIME_OVER</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-time-over-0940-ny</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>09:40:00</t>
+        </is>
+      </c>
+      <c r="AG6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ6" t="inlineStr">
+        <is>
+          <t>TIME_OVER</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>27176.25</v>
+      </c>
+      <c r="C7" t="n">
+        <v>27223.75</v>
+      </c>
+      <c r="D7" t="n">
+        <v>190</v>
+      </c>
+      <c r="E7" t="n">
+        <v>27208.66</v>
+      </c>
+      <c r="F7" t="n">
+        <v>75</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1287</v>
+      </c>
+      <c r="H7" t="n">
+        <v>173</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>normal speed</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="K7" t="n">
+        <v>8</v>
+      </c>
+      <c r="L7" t="n">
+        <v>27228.75</v>
+      </c>
+      <c r="M7" t="n">
+        <v>27243.75</v>
+      </c>
+      <c r="N7" t="n">
+        <v>27258.75</v>
+      </c>
+      <c r="O7" t="n">
+        <v>60</v>
+      </c>
+      <c r="P7" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>27228.75</v>
+      </c>
+      <c r="R7" s="4" t="n">
+        <v>-60</v>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>SCALP_NORMAL</t>
+        </is>
+      </c>
+      <c r="U7" t="n">
+        <v>60</v>
+      </c>
+      <c r="V7" t="n">
+        <v>10</v>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-time-over-0940-ny</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>09:34:00</t>
+        </is>
+      </c>
+      <c r="Y7" t="n">
+        <v>2314</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>36.4114</v>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE7" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF7" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG7" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH7" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI7" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ7" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>2026-04-27</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B8" t="n">
         <v>27363.75</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C8" t="n">
         <v>27435</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D8" t="n">
         <v>285</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E8" t="n">
         <v>27430.76</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F8" t="n">
         <v>35</v>
       </c>
-      <c r="G6" t="n">
+      <c r="G8" t="n">
         <v>843</v>
       </c>
-      <c r="H6" t="n">
+      <c r="H8" t="n">
         <v>-169</v>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>normal speed</t>
         </is>
       </c>
-      <c r="J6" t="n">
+      <c r="J8" t="n">
         <v>2.01</v>
       </c>
-      <c r="K6" t="n">
+      <c r="K8" t="n">
         <v>8</v>
       </c>
-      <c r="L6" t="n">
+      <c r="L8" t="n">
         <v>27370</v>
       </c>
-      <c r="M6" t="n">
+      <c r="M8" t="n">
         <v>27355</v>
       </c>
-      <c r="N6" t="n">
+      <c r="N8" t="n">
         <v>27340</v>
       </c>
-      <c r="O6" t="n">
-        <v>60</v>
-      </c>
-      <c r="P6" t="n">
-        <v>60</v>
-      </c>
-      <c r="Q6" t="n">
+      <c r="O8" t="n">
+        <v>60</v>
+      </c>
+      <c r="P8" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q8" t="n">
         <v>27370</v>
       </c>
-      <c r="R6" s="4" t="n">
+      <c r="R8" s="4" t="n">
         <v>-60</v>
       </c>
-      <c r="S6" t="inlineStr">
+      <c r="S8" t="inlineStr">
         <is>
           <t>SELL</t>
         </is>
       </c>
-      <c r="T6" t="inlineStr">
+      <c r="T8" t="inlineStr">
         <is>
           <t>SCALP_NORMAL</t>
         </is>
       </c>
-      <c r="U6" t="n">
-        <v>60</v>
-      </c>
-      <c r="V6" t="n">
+      <c r="U8" t="n">
+        <v>60</v>
+      </c>
+      <c r="V8" t="n">
         <v>5</v>
       </c>
-      <c r="W6" t="inlineStr">
-        <is>
-          <t>score-exporter-2026-05-27-strict-speed-window</t>
-        </is>
-      </c>
-      <c r="X6" t="inlineStr">
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-time-over-0940-ny</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
         <is>
           <t>09:36:00</t>
         </is>
       </c>
-      <c r="Y6" t="n">
+      <c r="Y8" t="n">
         <v>2316</v>
       </c>
-      <c r="Z6" t="n">
+      <c r="Z8" t="n">
         <v>17.4372</v>
       </c>
-      <c r="AA6" t="inlineStr">
+      <c r="AA8" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="AB6" t="inlineStr">
+      <c r="AB8" t="inlineStr">
         <is>
           <t>LastTime</t>
         </is>
       </c>
-      <c r="AC6" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AD6" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AE6" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AF6" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AG6" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AH6" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AI6" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AJ6" t="inlineStr">
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ8" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>27082.5</v>
+      </c>
+      <c r="C9" t="n">
+        <v>27162.5</v>
+      </c>
+      <c r="D9" t="n">
+        <v>320</v>
+      </c>
+      <c r="E9" t="n">
+        <v>27189.12</v>
+      </c>
+      <c r="F9" t="n">
+        <v>50</v>
+      </c>
+      <c r="G9" t="n">
+        <v>935</v>
+      </c>
+      <c r="H9" t="n">
+        <v>131</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>normal speed</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="K9" t="n">
+        <v>6</v>
+      </c>
+      <c r="L9" t="n">
+        <v>27168.75</v>
+      </c>
+      <c r="M9" t="n">
+        <v>27183.75</v>
+      </c>
+      <c r="N9" t="n">
+        <v>27198.75</v>
+      </c>
+      <c r="O9" t="n">
+        <v>60</v>
+      </c>
+      <c r="P9" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>27168.75</v>
+      </c>
+      <c r="R9" s="4" t="n">
+        <v>-60</v>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>SCALP_NORMAL</t>
+        </is>
+      </c>
+      <c r="U9" t="n">
+        <v>60</v>
+      </c>
+      <c r="V9" t="n">
+        <v>15</v>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-time-over-0940-ny</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>09:38:00</t>
+        </is>
+      </c>
+      <c r="Y9" t="n">
+        <v>2318</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>23.2757</v>
+      </c>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF9" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG9" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH9" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AI9" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ9" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>27151.25</v>
+      </c>
+      <c r="C10" t="n">
+        <v>27218.75</v>
+      </c>
+      <c r="D10" t="n">
+        <v>270</v>
+      </c>
+      <c r="E10" t="n">
+        <v>27241.75</v>
+      </c>
+      <c r="F10" t="n">
+        <v>15</v>
+      </c>
+      <c r="G10" t="n">
+        <v>805</v>
+      </c>
+      <c r="H10" t="n">
+        <v>-89</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>normal speed</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="K10" t="n">
+        <v>8</v>
+      </c>
+      <c r="L10" t="n">
+        <v>27162.5</v>
+      </c>
+      <c r="M10" t="n">
+        <v>27147.5</v>
+      </c>
+      <c r="N10" t="n">
+        <v>27132.5</v>
+      </c>
+      <c r="O10" t="n">
+        <v>60</v>
+      </c>
+      <c r="P10" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>27162.5</v>
+      </c>
+      <c r="R10" s="4" t="n">
+        <v>-60</v>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>SCALP_NORMAL</t>
+        </is>
+      </c>
+      <c r="U10" t="n">
+        <v>60</v>
+      </c>
+      <c r="V10" t="n">
+        <v>40</v>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-time-over-0940-ny</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>09:31:00</t>
+        </is>
+      </c>
+      <c r="Y10" t="n">
+        <v>2311</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>6.4496</v>
+      </c>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE10" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF10" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG10" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH10" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI10" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ10" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>27422.5</v>
+      </c>
+      <c r="C11" t="n">
+        <v>27492.5</v>
+      </c>
+      <c r="D11" t="n">
+        <v>280</v>
+      </c>
+      <c r="E11" t="n">
+        <v>27385.43</v>
+      </c>
+      <c r="F11" t="n">
+        <v>25</v>
+      </c>
+      <c r="G11" t="n">
+        <v>987</v>
+      </c>
+      <c r="H11" t="n">
+        <v>-107</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>normal speed</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="K11" t="n">
+        <v>6</v>
+      </c>
+      <c r="L11" t="n">
+        <v>27431.25</v>
+      </c>
+      <c r="M11" t="n">
+        <v>27416.25</v>
+      </c>
+      <c r="N11" t="n">
+        <v>27401.25</v>
+      </c>
+      <c r="O11" t="n">
+        <v>60</v>
+      </c>
+      <c r="P11" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>27401.25</v>
+      </c>
+      <c r="R11" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>SCALP_NORMAL</t>
+        </is>
+      </c>
+      <c r="U11" t="n">
+        <v>45</v>
+      </c>
+      <c r="V11" t="n">
+        <v>60</v>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-time-over-0940-ny</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>09:31:00</t>
+        </is>
+      </c>
+      <c r="Y11" t="n">
+        <v>2311</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>11.8019</v>
+      </c>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE11" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF11" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG11" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH11" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AI11" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ11" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>27618.75</v>
+      </c>
+      <c r="C12" t="n">
+        <v>27666.25</v>
+      </c>
+      <c r="D12" t="n">
+        <v>190</v>
+      </c>
+      <c r="E12" t="n">
+        <v>27598.3</v>
+      </c>
+      <c r="F12" t="n">
+        <v>20</v>
+      </c>
+      <c r="G12" t="n">
+        <v>846</v>
+      </c>
+      <c r="H12" t="n">
+        <v>254</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>normal speed</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>2.61</v>
+      </c>
+      <c r="K12" t="n">
+        <v>8</v>
+      </c>
+      <c r="L12" t="n">
+        <v>27656.25</v>
+      </c>
+      <c r="M12" t="n">
+        <v>27671.25</v>
+      </c>
+      <c r="N12" t="n">
+        <v>27686.25</v>
+      </c>
+      <c r="O12" t="n">
+        <v>60</v>
+      </c>
+      <c r="P12" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>27686.25</v>
+      </c>
+      <c r="R12" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>SCALP_NORMAL</t>
+        </is>
+      </c>
+      <c r="U12" t="n">
+        <v>5</v>
+      </c>
+      <c r="V12" t="n">
+        <v>60</v>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-time-over-0940-ny</t>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>09:31:00</t>
+        </is>
+      </c>
+      <c r="Y12" t="n">
+        <v>2311</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>7.666</v>
+      </c>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AB12" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE12" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF12" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG12" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH12" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI12" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ12" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>27837.5</v>
+      </c>
+      <c r="C13" t="n">
+        <v>27875</v>
+      </c>
+      <c r="D13" t="n">
+        <v>150</v>
+      </c>
+      <c r="E13" t="n">
+        <v>27837.01</v>
+      </c>
+      <c r="F13" t="n">
+        <v>40</v>
+      </c>
+      <c r="G13" t="n">
+        <v>1342</v>
+      </c>
+      <c r="H13" t="n">
+        <v>-24</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>normal speed</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>2.23</v>
+      </c>
+      <c r="K13" t="n">
+        <v>7</v>
+      </c>
+      <c r="L13" t="n">
+        <v>27842.5</v>
+      </c>
+      <c r="M13" t="n">
+        <v>27827.5</v>
+      </c>
+      <c r="N13" t="n">
+        <v>27812.5</v>
+      </c>
+      <c r="O13" t="n">
+        <v>60</v>
+      </c>
+      <c r="P13" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>27812.5</v>
+      </c>
+      <c r="R13" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>SCALP_NORMAL</t>
+        </is>
+      </c>
+      <c r="U13" t="n">
+        <v>10</v>
+      </c>
+      <c r="V13" t="n">
+        <v>60</v>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-time-over-0940-ny</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>09:31:00</t>
+        </is>
+      </c>
+      <c r="Y13" t="n">
+        <v>2311</v>
+      </c>
+      <c r="Z13" t="n">
+        <v>17.9196</v>
+      </c>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AB13" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE13" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF13" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AG13" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH13" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI13" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ13" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>27986.25</v>
+      </c>
+      <c r="C14" t="n">
+        <v>28023.75</v>
+      </c>
+      <c r="D14" t="n">
+        <v>150</v>
+      </c>
+      <c r="E14" t="n">
+        <v>27935.72</v>
+      </c>
+      <c r="F14" t="n">
+        <v>20</v>
+      </c>
+      <c r="G14" t="n">
+        <v>868</v>
+      </c>
+      <c r="H14" t="n">
+        <v>-146</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>normal speed</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="K14" t="n">
+        <v>6</v>
+      </c>
+      <c r="L14" t="n">
+        <v>27996.25</v>
+      </c>
+      <c r="M14" t="n">
+        <v>27981.25</v>
+      </c>
+      <c r="N14" t="n">
+        <v>27966.25</v>
+      </c>
+      <c r="O14" t="n">
+        <v>60</v>
+      </c>
+      <c r="P14" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>27996.25</v>
+      </c>
+      <c r="R14" s="4" t="n">
+        <v>-60</v>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>SCALP_NORMAL</t>
+        </is>
+      </c>
+      <c r="U14" t="n">
+        <v>60</v>
+      </c>
+      <c r="V14" t="n">
+        <v>40</v>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-time-over-0940-ny</t>
+        </is>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>09:31:00</t>
+        </is>
+      </c>
+      <c r="Y14" t="n">
+        <v>2310</v>
+      </c>
+      <c r="Z14" t="n">
+        <v>5.528</v>
+      </c>
+      <c r="AA14" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AB14" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE14" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF14" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG14" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH14" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AI14" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ14" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>28336.25</v>
+      </c>
+      <c r="C15" t="n">
+        <v>28392.5</v>
+      </c>
+      <c r="D15" t="n">
+        <v>225</v>
+      </c>
+      <c r="E15" t="n">
+        <v>28455.83</v>
+      </c>
+      <c r="F15" t="n">
+        <v>25</v>
+      </c>
+      <c r="G15" t="n">
+        <v>837</v>
+      </c>
+      <c r="H15" t="n">
+        <v>27</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>normal speed</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="K15" t="n">
+        <v>6</v>
+      </c>
+      <c r="L15" t="n">
+        <v>28411.25</v>
+      </c>
+      <c r="M15" t="n">
+        <v>28426.25</v>
+      </c>
+      <c r="N15" t="n">
+        <v>28441.25</v>
+      </c>
+      <c r="O15" t="n">
+        <v>60</v>
+      </c>
+      <c r="P15" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>28411.25</v>
+      </c>
+      <c r="R15" s="4" t="n">
+        <v>-60</v>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>SCALP_NORMAL</t>
+        </is>
+      </c>
+      <c r="U15" t="n">
+        <v>60</v>
+      </c>
+      <c r="V15" t="n">
+        <v>0</v>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-time-over-0940-ny</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>09:33:00</t>
+        </is>
+      </c>
+      <c r="Y15" t="n">
+        <v>2313</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>11.7515</v>
+      </c>
+      <c r="AA15" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AB15" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AC15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH15" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AI15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ15" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>28730</v>
+      </c>
+      <c r="C16" t="n">
+        <v>28766.25</v>
+      </c>
+      <c r="D16" t="n">
+        <v>145</v>
+      </c>
+      <c r="R16" s="4" t="inlineStr">
+        <is>
+          <t>TIME_OVER</t>
+        </is>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-time-over-0940-ny</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>09:40:00</t>
+        </is>
+      </c>
+      <c r="AG16" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ16" t="inlineStr">
+        <is>
+          <t>TIME_OVER</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>28860</v>
+      </c>
+      <c r="C17" t="n">
+        <v>28903.75</v>
+      </c>
+      <c r="D17" t="n">
+        <v>175</v>
+      </c>
+      <c r="E17" t="n">
+        <v>28876.6</v>
+      </c>
+      <c r="F17" t="n">
+        <v>50</v>
+      </c>
+      <c r="G17" t="n">
+        <v>1574</v>
+      </c>
+      <c r="H17" t="n">
+        <v>208</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>normal speed</t>
+        </is>
+      </c>
+      <c r="J17" t="n">
+        <v>2.19</v>
+      </c>
+      <c r="K17" t="n">
+        <v>8</v>
+      </c>
+      <c r="L17" t="n">
+        <v>28901.25</v>
+      </c>
+      <c r="M17" t="n">
+        <v>28916.25</v>
+      </c>
+      <c r="N17" t="n">
+        <v>28931.25</v>
+      </c>
+      <c r="O17" t="n">
+        <v>60</v>
+      </c>
+      <c r="P17" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>28931.25</v>
+      </c>
+      <c r="R17" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>SCALP_NORMAL</t>
+        </is>
+      </c>
+      <c r="U17" t="n">
+        <v>45</v>
+      </c>
+      <c r="V17" t="n">
+        <v>65</v>
+      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-time-over-0940-ny</t>
+        </is>
+      </c>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>09:31:00</t>
+        </is>
+      </c>
+      <c r="Y17" t="n">
+        <v>2311</v>
+      </c>
+      <c r="Z17" t="n">
+        <v>22.8326</v>
+      </c>
+      <c r="AA17" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AB17" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE17" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF17" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG17" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH17" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI17" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ17" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>29282.5</v>
+      </c>
+      <c r="C18" t="n">
+        <v>29346.25</v>
+      </c>
+      <c r="D18" t="n">
+        <v>255</v>
+      </c>
+      <c r="E18" t="n">
+        <v>29316.62</v>
+      </c>
+      <c r="F18" t="n">
+        <v>75</v>
+      </c>
+      <c r="G18" t="n">
+        <v>815</v>
+      </c>
+      <c r="H18" t="n">
+        <v>137</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>A+ speed</t>
+        </is>
+      </c>
+      <c r="J18" t="n">
+        <v>10.71</v>
+      </c>
+      <c r="K18" t="n">
+        <v>9</v>
+      </c>
+      <c r="L18" t="n">
+        <v>29350</v>
+      </c>
+      <c r="M18" t="n">
+        <v>29365</v>
+      </c>
+      <c r="N18" t="n">
+        <v>29380</v>
+      </c>
+      <c r="O18" t="n">
+        <v>60</v>
+      </c>
+      <c r="P18" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>29380</v>
+      </c>
+      <c r="R18" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>POTENTIAL_RUNNER</t>
+        </is>
+      </c>
+      <c r="U18" t="n">
+        <v>15</v>
+      </c>
+      <c r="V18" t="n">
+        <v>60</v>
+      </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-time-over-0940-ny</t>
+        </is>
+      </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>09:31:00</t>
+        </is>
+      </c>
+      <c r="Y18" t="n">
+        <v>2311</v>
+      </c>
+      <c r="Z18" t="n">
+        <v>6.9997</v>
+      </c>
+      <c r="AA18" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AB18" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AC18" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD18" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE18" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF18" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG18" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH18" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI18" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ18" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>29146.25</v>
+      </c>
+      <c r="C19" t="n">
+        <v>29227.5</v>
+      </c>
+      <c r="D19" t="n">
+        <v>325</v>
+      </c>
+      <c r="R19" s="4" t="inlineStr">
+        <is>
+          <t>TIME_OVER</t>
+        </is>
+      </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-time-over-0940-ny</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>09:40:00</t>
+        </is>
+      </c>
+      <c r="AG19" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ19" t="inlineStr">
+        <is>
+          <t>TIME_OVER</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>29252.5</v>
+      </c>
+      <c r="C20" t="n">
+        <v>29288.75</v>
+      </c>
+      <c r="D20" t="n">
+        <v>145</v>
+      </c>
+      <c r="E20" t="n">
+        <v>29321.36</v>
+      </c>
+      <c r="F20" t="n">
+        <v>35</v>
+      </c>
+      <c r="G20" t="n">
+        <v>1114</v>
+      </c>
+      <c r="H20" t="n">
+        <v>-176</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>normal speed</t>
+        </is>
+      </c>
+      <c r="J20" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="K20" t="n">
+        <v>8</v>
+      </c>
+      <c r="L20" t="n">
+        <v>29258.75</v>
+      </c>
+      <c r="M20" t="n">
+        <v>29243.75</v>
+      </c>
+      <c r="N20" t="n">
+        <v>29228.75</v>
+      </c>
+      <c r="O20" t="n">
+        <v>60</v>
+      </c>
+      <c r="P20" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>29228.75</v>
+      </c>
+      <c r="R20" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>SCALP_NORMAL</t>
+        </is>
+      </c>
+      <c r="U20" t="n">
+        <v>0</v>
+      </c>
+      <c r="V20" t="n">
+        <v>60</v>
+      </c>
+      <c r="W20" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-time-over-0940-ny</t>
+        </is>
+      </c>
+      <c r="X20" t="inlineStr">
+        <is>
+          <t>09:31:00</t>
+        </is>
+      </c>
+      <c r="Y20" t="n">
+        <v>2311</v>
+      </c>
+      <c r="Z20" t="n">
+        <v>16.8169</v>
+      </c>
+      <c r="AA20" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AB20" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AC20" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD20" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE20" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF20" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG20" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH20" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI20" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ20" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>29460</v>
+      </c>
+      <c r="C21" t="n">
+        <v>29492.5</v>
+      </c>
+      <c r="D21" t="n">
+        <v>130</v>
+      </c>
+      <c r="E21" t="n">
+        <v>29543.51</v>
+      </c>
+      <c r="F21" t="n">
+        <v>65</v>
+      </c>
+      <c r="G21" t="n">
+        <v>802</v>
+      </c>
+      <c r="H21" t="n">
+        <v>262</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>A+ speed</t>
+        </is>
+      </c>
+      <c r="J21" t="n">
+        <v>10.97</v>
+      </c>
+      <c r="K21" t="n">
+        <v>7</v>
+      </c>
+      <c r="L21" t="n">
+        <v>29500</v>
+      </c>
+      <c r="M21" t="n">
+        <v>29515</v>
+      </c>
+      <c r="N21" t="n">
+        <v>29530</v>
+      </c>
+      <c r="O21" t="n">
+        <v>60</v>
+      </c>
+      <c r="P21" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>29530</v>
+      </c>
+      <c r="R21" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>POTENTIAL_RUNNER</t>
+        </is>
+      </c>
+      <c r="U21" t="n">
+        <v>20</v>
+      </c>
+      <c r="V21" t="n">
+        <v>60</v>
+      </c>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-time-over-0940-ny</t>
+        </is>
+      </c>
+      <c r="X21" t="inlineStr">
+        <is>
+          <t>09:32:00</t>
+        </is>
+      </c>
+      <c r="Y21" t="n">
+        <v>2312</v>
+      </c>
+      <c r="Z21" t="n">
+        <v>5.9247</v>
+      </c>
+      <c r="AA21" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AB21" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AC21" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD21" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE21" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF21" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG21" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH21" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AI21" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ21" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>29241.25</v>
+      </c>
+      <c r="C22" t="n">
+        <v>29291.25</v>
+      </c>
+      <c r="D22" t="n">
+        <v>200</v>
+      </c>
+      <c r="E22" t="n">
+        <v>29294.78</v>
+      </c>
+      <c r="F22" t="n">
+        <v>90</v>
+      </c>
+      <c r="G22" t="n">
+        <v>814</v>
+      </c>
+      <c r="H22" t="n">
+        <v>-358</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>A+ speed</t>
+        </is>
+      </c>
+      <c r="J22" t="n">
+        <v>18.05</v>
+      </c>
+      <c r="K22" t="n">
+        <v>9</v>
+      </c>
+      <c r="L22" t="n">
+        <v>29233.75</v>
+      </c>
+      <c r="M22" t="n">
+        <v>29218.75</v>
+      </c>
+      <c r="N22" t="n">
+        <v>29203.75</v>
+      </c>
+      <c r="O22" t="n">
+        <v>60</v>
+      </c>
+      <c r="P22" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>29203.75</v>
+      </c>
+      <c r="R22" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>POTENTIAL_RUNNER</t>
+        </is>
+      </c>
+      <c r="U22" t="n">
+        <v>25</v>
+      </c>
+      <c r="V22" t="n">
+        <v>60</v>
+      </c>
+      <c r="W22" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-time-over-0940-ny</t>
+        </is>
+      </c>
+      <c r="X22" t="inlineStr">
+        <is>
+          <t>09:31:00</t>
+        </is>
+      </c>
+      <c r="Y22" t="n">
+        <v>2311</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>4.9856</v>
+      </c>
+      <c r="AA22" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AB22" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AC22" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD22" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE22" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF22" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG22" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH22" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI22" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ22" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>29305</v>
+      </c>
+      <c r="C23" t="n">
+        <v>29356.25</v>
+      </c>
+      <c r="D23" t="n">
+        <v>205</v>
+      </c>
+      <c r="E23" t="n">
+        <v>29211.89</v>
+      </c>
+      <c r="F23" t="n">
+        <v>50</v>
+      </c>
+      <c r="G23" t="n">
+        <v>802</v>
+      </c>
+      <c r="H23" t="n">
+        <v>-158</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>normal speed</t>
+        </is>
+      </c>
+      <c r="J23" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="K23" t="n">
+        <v>6</v>
+      </c>
+      <c r="L23" t="n">
+        <v>29298.75</v>
+      </c>
+      <c r="M23" t="n">
+        <v>29283.75</v>
+      </c>
+      <c r="N23" t="n">
+        <v>29268.75</v>
+      </c>
+      <c r="O23" t="n">
+        <v>60</v>
+      </c>
+      <c r="P23" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>29298.75</v>
+      </c>
+      <c r="R23" s="4" t="n">
+        <v>-60</v>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>SCALP_NORMAL</t>
+        </is>
+      </c>
+      <c r="U23" t="n">
+        <v>60</v>
+      </c>
+      <c r="V23" t="n">
+        <v>5</v>
+      </c>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-time-over-0940-ny</t>
+        </is>
+      </c>
+      <c r="X23" t="inlineStr">
+        <is>
+          <t>09:33:00</t>
+        </is>
+      </c>
+      <c r="Y23" t="n">
+        <v>2313</v>
+      </c>
+      <c r="Z23" t="n">
+        <v>12.8979</v>
+      </c>
+      <c r="AA23" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AB23" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AC23" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD23" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE23" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF23" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG23" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH23" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AI23" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ23" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>28851.25</v>
+      </c>
+      <c r="C24" t="n">
+        <v>28943.75</v>
+      </c>
+      <c r="D24" t="n">
+        <v>370</v>
+      </c>
+      <c r="E24" t="n">
+        <v>28925.15</v>
+      </c>
+      <c r="F24" t="n">
+        <v>40</v>
+      </c>
+      <c r="G24" t="n">
+        <v>820</v>
+      </c>
+      <c r="H24" t="n">
+        <v>124</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>normal speed</t>
+        </is>
+      </c>
+      <c r="J24" t="n">
+        <v>2.77</v>
+      </c>
+      <c r="K24" t="n">
+        <v>7</v>
+      </c>
+      <c r="L24" t="n">
+        <v>28938.75</v>
+      </c>
+      <c r="M24" t="n">
+        <v>28953.75</v>
+      </c>
+      <c r="N24" t="n">
+        <v>28968.75</v>
+      </c>
+      <c r="O24" t="n">
+        <v>60</v>
+      </c>
+      <c r="P24" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>28968.75</v>
+      </c>
+      <c r="R24" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>SCALP_NORMAL</t>
+        </is>
+      </c>
+      <c r="U24" t="n">
+        <v>10</v>
+      </c>
+      <c r="V24" t="n">
+        <v>65</v>
+      </c>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-time-over-0940-ny</t>
+        </is>
+      </c>
+      <c r="X24" t="inlineStr">
+        <is>
+          <t>09:32:00</t>
+        </is>
+      </c>
+      <c r="Y24" t="n">
+        <v>2312</v>
+      </c>
+      <c r="Z24" t="n">
+        <v>14.4236</v>
+      </c>
+      <c r="AA24" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AB24" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AC24" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AD24" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE24" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF24" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG24" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH24" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI24" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ24" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>29070</v>
+      </c>
+      <c r="C25" t="n">
+        <v>29122.5</v>
+      </c>
+      <c r="D25" t="n">
+        <v>210</v>
+      </c>
+      <c r="E25" t="n">
+        <v>29074.59</v>
+      </c>
+      <c r="F25" t="n">
+        <v>25</v>
+      </c>
+      <c r="G25" t="n">
+        <v>1130</v>
+      </c>
+      <c r="H25" t="n">
+        <v>184</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>normal speed</t>
+        </is>
+      </c>
+      <c r="J25" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="K25" t="n">
+        <v>8</v>
+      </c>
+      <c r="L25" t="n">
+        <v>29113.75</v>
+      </c>
+      <c r="M25" t="n">
+        <v>29128.75</v>
+      </c>
+      <c r="N25" t="n">
+        <v>29143.75</v>
+      </c>
+      <c r="O25" t="n">
+        <v>60</v>
+      </c>
+      <c r="P25" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>29113.75</v>
+      </c>
+      <c r="R25" s="4" t="n">
+        <v>-60</v>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>SCALP_NORMAL</t>
+        </is>
+      </c>
+      <c r="U25" t="n">
+        <v>60</v>
+      </c>
+      <c r="V25" t="n">
+        <v>30</v>
+      </c>
+      <c r="W25" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-time-over-0940-ny</t>
+        </is>
+      </c>
+      <c r="X25" t="inlineStr">
+        <is>
+          <t>09:31:00</t>
+        </is>
+      </c>
+      <c r="Y25" t="n">
+        <v>2311</v>
+      </c>
+      <c r="Z25" t="n">
+        <v>8.0563</v>
+      </c>
+      <c r="AA25" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AB25" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AC25" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD25" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE25" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF25" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG25" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH25" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI25" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ25" t="inlineStr">
         <is>
           <t>SL</t>
         </is>

</xml_diff>

<commit_message>
A+ Structure labels by setup side
</commit_message>
<xml_diff>
--- a/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
+++ b/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
@@ -694,16 +694,16 @@
         <v>165</v>
       </c>
       <c r="E4" t="n">
-        <v>26841.85</v>
+        <v>26841.84</v>
       </c>
       <c r="F4" t="n">
         <v>70</v>
       </c>
       <c r="G4" t="n">
-        <v>1316</v>
+        <v>1319</v>
       </c>
       <c r="H4" t="n">
-        <v>-116</v>
+        <v>-117</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -711,7 +711,7 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>2.1</v>
+        <v>2.09</v>
       </c>
       <c r="K4" t="n">
         <v>8</v>
@@ -755,7 +755,7 @@
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>score-exporter-2026-05-30-time-over-0940-ny</t>
+          <t>score-exporter-2026-05-30-aplus-structure-export</t>
         </is>
       </c>
       <c r="X4" t="inlineStr">
@@ -767,7 +767,7 @@
         <v>2312</v>
       </c>
       <c r="Z4" t="n">
-        <v>33.3865</v>
+        <v>33.4256</v>
       </c>
       <c r="AA4" t="inlineStr">
         <is>
@@ -821,11 +821,19 @@
       </c>
       <c r="AK4" t="inlineStr">
         <is>
-          <t>FALSE</t>
-        </is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AL4" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="AM4" t="n">
+        <v>26876.25</v>
       </c>
       <c r="AN4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AO4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Export A+ Structure only when imbalance side matches trade side
</commit_message>
<xml_diff>
--- a/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
+++ b/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
@@ -694,16 +694,16 @@
         <v>165</v>
       </c>
       <c r="E4" t="n">
-        <v>26841.84</v>
+        <v>26841.85</v>
       </c>
       <c r="F4" t="n">
         <v>70</v>
       </c>
       <c r="G4" t="n">
-        <v>1319</v>
+        <v>1300</v>
       </c>
       <c r="H4" t="n">
-        <v>-117</v>
+        <v>-120</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -711,7 +711,7 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>2.09</v>
+        <v>2.1</v>
       </c>
       <c r="K4" t="n">
         <v>8</v>
@@ -767,7 +767,7 @@
         <v>2312</v>
       </c>
       <c r="Z4" t="n">
-        <v>33.4256</v>
+        <v>33.2933</v>
       </c>
       <c r="AA4" t="inlineStr">
         <is>
@@ -826,11 +826,11 @@
       </c>
       <c r="AL4" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="AM4" t="n">
-        <v>26876.25</v>
+        <v>26852.5</v>
       </c>
       <c r="AN4" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
STRUCTURE CON ETIQUETA DETECTORA DE IMBALANCES SEPARADOS
</commit_message>
<xml_diff>
--- a/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
+++ b/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
@@ -700,10 +700,10 @@
         <v>70</v>
       </c>
       <c r="G4" t="n">
-        <v>1300</v>
+        <v>1305</v>
       </c>
       <c r="H4" t="n">
-        <v>-120</v>
+        <v>-115</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -767,7 +767,7 @@
         <v>2312</v>
       </c>
       <c r="Z4" t="n">
-        <v>33.2933</v>
+        <v>33.3002</v>
       </c>
       <c r="AA4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
A+ Structure trade + EXCEL generado
</commit_message>
<xml_diff>
--- a/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
+++ b/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
@@ -694,36 +694,36 @@
         <v>165</v>
       </c>
       <c r="E4" t="n">
-        <v>26841.85</v>
+        <v>26842.09</v>
       </c>
       <c r="F4" t="n">
-        <v>70</v>
+        <v>5</v>
       </c>
       <c r="G4" t="n">
-        <v>1305</v>
+        <v>1173</v>
       </c>
       <c r="H4" t="n">
-        <v>-115</v>
+        <v>-229</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>normal speed</t>
+          <t>A+ structure</t>
         </is>
       </c>
       <c r="J4" t="n">
-        <v>2.1</v>
+        <v>0.14</v>
       </c>
       <c r="K4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L4" t="n">
+        <v>26866.25</v>
+      </c>
+      <c r="M4" t="n">
+        <v>26851.25</v>
+      </c>
+      <c r="N4" t="n">
         <v>26836.25</v>
-      </c>
-      <c r="M4" t="n">
-        <v>26821.25</v>
-      </c>
-      <c r="N4" t="n">
-        <v>26806.25</v>
       </c>
       <c r="O4" t="n">
         <v>60</v>
@@ -735,7 +735,7 @@
         <v>26836.25</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>-60</v>
+        <v>60</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
@@ -744,30 +744,30 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>SCALP_NORMAL</t>
+          <t>POTENTIAL_RUNNER</t>
         </is>
       </c>
       <c r="U4" t="n">
-        <v>65</v>
+        <v>0</v>
       </c>
       <c r="V4" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>score-exporter-2026-05-30-aplus-structure-export</t>
+          <t>score-exporter-2026-05-30-aplus-bypass-speed</t>
         </is>
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>09:33:00</t>
+          <t>09:32:00</t>
         </is>
       </c>
       <c r="Y4" t="n">
-        <v>2312</v>
+        <v>2311</v>
       </c>
       <c r="Z4" t="n">
-        <v>33.3002</v>
+        <v>35.9291</v>
       </c>
       <c r="AA4" t="inlineStr">
         <is>
@@ -786,58 +786,55 @@
       </c>
       <c r="AD4" t="inlineStr">
         <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AE4" t="inlineStr">
+      <c r="AF4" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AF4" t="inlineStr">
+      <c r="AG4" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AG4" t="inlineStr">
+      <c r="AH4" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AI4" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AJ4" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="AK4" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AH4" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AI4" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AJ4" t="inlineStr">
-        <is>
-          <t>SL</t>
-        </is>
-      </c>
-      <c r="AK4" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
       <c r="AL4" t="inlineStr">
         <is>
           <t>SELL</t>
         </is>
-      </c>
-      <c r="AM4" t="n">
-        <v>26852.5</v>
       </c>
       <c r="AN4" t="n">
         <v>3</v>
       </c>
       <c r="AO4" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
REGRESAMOS A STRUCTURE CON ETIQUETA DETECTORA DE IMBALANCES SEPARADOS + PYTHON ACTUALIZADO PARA VALIDAR QUE NADA SE ROMPA
</commit_message>
<xml_diff>
--- a/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
+++ b/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
@@ -463,11 +463,11 @@
     </row>
     <row r="2">
       <c r="A2" s="1">
-        <f>IF((COUNTIF(R4:R4,"&gt;0")+COUNTIF(R4:R4,"&lt;0"))=0,"",COUNTIF(R4:R4,"&gt;0")/(COUNTIF(R4:R4,"&gt;0")+COUNTIF(R4:R4,"&lt;0")))</f>
+        <f>IF((COUNTIF(R4:R7,"&gt;0")+COUNTIF(R4:R7,"&lt;0"))=0,"",COUNTIF(R4:R7,"&gt;0")/(COUNTIF(R4:R7,"&gt;0")+COUNTIF(R4:R7,"&lt;0")))</f>
         <v/>
       </c>
       <c r="B2" s="2">
-        <f>IF(ABS(SUMIF(R4:R4,"&lt;0",R4:R4))=0,IF(SUMIF(R4:R4,"&gt;0",R4:R4)&gt;0,"INF",""),SUMIF(R4:R4,"&gt;0",R4:R4)/ABS(SUMIF(R4:R4,"&lt;0",R4:R4)))</f>
+        <f>IF(ABS(SUMIF(R4:R7,"&lt;0",R4:R7))=0,IF(SUMIF(R4:R7,"&gt;0",R4:R7)&gt;0,"INF",""),SUMIF(R4:R7,"&gt;0",R4:R7)/ABS(SUMIF(R4:R7,"&lt;0",R4:R7)))</f>
         <v/>
       </c>
     </row>
@@ -694,36 +694,36 @@
         <v>165</v>
       </c>
       <c r="E4" t="n">
-        <v>26842.09</v>
+        <v>26841.85</v>
       </c>
       <c r="F4" t="n">
-        <v>5</v>
+        <v>70</v>
       </c>
       <c r="G4" t="n">
-        <v>1173</v>
+        <v>1306</v>
       </c>
       <c r="H4" t="n">
-        <v>-229</v>
+        <v>-116</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>A+ structure</t>
+          <t>normal speed</t>
         </is>
       </c>
       <c r="J4" t="n">
-        <v>0.14</v>
+        <v>2.1</v>
       </c>
       <c r="K4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L4" t="n">
-        <v>26866.25</v>
+        <v>26836.25</v>
       </c>
       <c r="M4" t="n">
-        <v>26851.25</v>
+        <v>26821.25</v>
       </c>
       <c r="N4" t="n">
-        <v>26836.25</v>
+        <v>26806.25</v>
       </c>
       <c r="O4" t="n">
         <v>60</v>
@@ -735,7 +735,7 @@
         <v>26836.25</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>60</v>
+        <v>-60</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
@@ -744,30 +744,30 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>POTENTIAL_RUNNER</t>
+          <t>SCALP_NORMAL</t>
         </is>
       </c>
       <c r="U4" t="n">
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="V4" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>score-exporter-2026-05-30-aplus-bypass-speed</t>
+          <t>score-exporter-2026-05-30-aplus-structure-export</t>
         </is>
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>09:32:00</t>
+          <t>09:33:00</t>
         </is>
       </c>
       <c r="Y4" t="n">
-        <v>2311</v>
+        <v>2312</v>
       </c>
       <c r="Z4" t="n">
-        <v>35.9291</v>
+        <v>33.3088</v>
       </c>
       <c r="AA4" t="inlineStr">
         <is>
@@ -786,7 +786,7 @@
       </c>
       <c r="AD4" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="AE4" t="inlineStr">
@@ -806,17 +806,17 @@
       </c>
       <c r="AH4" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="AI4" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="AJ4" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>SL</t>
         </is>
       </c>
       <c r="AK4" t="inlineStr">
@@ -828,24 +828,491 @@
         <is>
           <t>SELL</t>
         </is>
+      </c>
+      <c r="AM4" t="n">
+        <v>26852.5</v>
       </c>
       <c r="AN4" t="n">
         <v>3</v>
       </c>
       <c r="AO4" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="R5" s="4" t="n"/>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>29252.5</v>
+      </c>
+      <c r="C5" t="n">
+        <v>29288.75</v>
+      </c>
+      <c r="D5" t="n">
+        <v>145</v>
+      </c>
+      <c r="E5" t="n">
+        <v>29321.36</v>
+      </c>
+      <c r="F5" t="n">
+        <v>35</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1117</v>
+      </c>
+      <c r="H5" t="n">
+        <v>-175</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>normal speed</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="K5" t="n">
+        <v>8</v>
+      </c>
+      <c r="L5" t="n">
+        <v>29258.75</v>
+      </c>
+      <c r="M5" t="n">
+        <v>29243.75</v>
+      </c>
+      <c r="N5" t="n">
+        <v>29228.75</v>
+      </c>
+      <c r="O5" t="n">
+        <v>60</v>
+      </c>
+      <c r="P5" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>29228.75</v>
+      </c>
+      <c r="R5" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>SCALP_NORMAL</t>
+        </is>
+      </c>
+      <c r="U5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V5" t="n">
+        <v>60</v>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-aplus-structure-export</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>09:31:00</t>
+        </is>
+      </c>
+      <c r="Y5" t="n">
+        <v>2311</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>16.8224</v>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ5" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="AK5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AN5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="R6" s="4" t="n"/>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>29460</v>
+      </c>
+      <c r="C6" t="n">
+        <v>29492.5</v>
+      </c>
+      <c r="D6" t="n">
+        <v>130</v>
+      </c>
+      <c r="E6" t="n">
+        <v>29543.51</v>
+      </c>
+      <c r="F6" t="n">
+        <v>65</v>
+      </c>
+      <c r="G6" t="n">
+        <v>801</v>
+      </c>
+      <c r="H6" t="n">
+        <v>263</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>A+ speed</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>11.01</v>
+      </c>
+      <c r="K6" t="n">
+        <v>7</v>
+      </c>
+      <c r="L6" t="n">
+        <v>29500</v>
+      </c>
+      <c r="M6" t="n">
+        <v>29515</v>
+      </c>
+      <c r="N6" t="n">
+        <v>29530</v>
+      </c>
+      <c r="O6" t="n">
+        <v>60</v>
+      </c>
+      <c r="P6" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>29530</v>
+      </c>
+      <c r="R6" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>POTENTIAL_RUNNER</t>
+        </is>
+      </c>
+      <c r="U6" t="n">
+        <v>20</v>
+      </c>
+      <c r="V6" t="n">
+        <v>60</v>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-aplus-structure-export</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>09:32:00</t>
+        </is>
+      </c>
+      <c r="Y6" t="n">
+        <v>2312</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>5.9038</v>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH6" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AI6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ6" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="AK6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AL6" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="AM6" t="n">
+        <v>29501.25</v>
+      </c>
+      <c r="AN6" t="n">
+        <v>3</v>
+      </c>
+      <c r="AO6" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="R7" s="4" t="n"/>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>29241.25</v>
+      </c>
+      <c r="C7" t="n">
+        <v>29291.25</v>
+      </c>
+      <c r="D7" t="n">
+        <v>200</v>
+      </c>
+      <c r="E7" t="n">
+        <v>29294.78</v>
+      </c>
+      <c r="F7" t="n">
+        <v>90</v>
+      </c>
+      <c r="G7" t="n">
+        <v>814</v>
+      </c>
+      <c r="H7" t="n">
+        <v>-358</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>A+ speed</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>18.05</v>
+      </c>
+      <c r="K7" t="n">
+        <v>9</v>
+      </c>
+      <c r="L7" t="n">
+        <v>29233.75</v>
+      </c>
+      <c r="M7" t="n">
+        <v>29218.75</v>
+      </c>
+      <c r="N7" t="n">
+        <v>29203.75</v>
+      </c>
+      <c r="O7" t="n">
+        <v>60</v>
+      </c>
+      <c r="P7" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>29203.75</v>
+      </c>
+      <c r="R7" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>POTENTIAL_RUNNER</t>
+        </is>
+      </c>
+      <c r="U7" t="n">
+        <v>30</v>
+      </c>
+      <c r="V7" t="n">
+        <v>60</v>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-aplus-structure-export</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>09:31:00</t>
+        </is>
+      </c>
+      <c r="Y7" t="n">
+        <v>2311</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>4.9856</v>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE7" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF7" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG7" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH7" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI7" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ7" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="AK7" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AN7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO7" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="R8" s="4" t="n"/>

</xml_diff>

<commit_message>
Refactor de logica Visual a TRADE MANAGER para que logica VISUAL SOLO PINTE
EN ESTE CAMBIO EL BREAKOUT SPEED SIGUE IGUAL Y Y LOS RESULTADOS NO CAMBIAN
</commit_message>
<xml_diff>
--- a/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
+++ b/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
@@ -700,10 +700,10 @@
         <v>70</v>
       </c>
       <c r="G4" t="n">
-        <v>1306</v>
+        <v>1313</v>
       </c>
       <c r="H4" t="n">
-        <v>-116</v>
+        <v>-117</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -767,7 +767,7 @@
         <v>2312</v>
       </c>
       <c r="Z4" t="n">
-        <v>33.3088</v>
+        <v>33.3476</v>
       </c>
       <c r="AA4" t="inlineStr">
         <is>
@@ -863,7 +863,7 @@
         <v>35</v>
       </c>
       <c r="G5" t="n">
-        <v>1117</v>
+        <v>1113</v>
       </c>
       <c r="H5" t="n">
         <v>-175</v>
@@ -930,7 +930,7 @@
         <v>2311</v>
       </c>
       <c r="Z5" t="n">
-        <v>16.8224</v>
+        <v>16.8109</v>
       </c>
       <c r="AA5" t="inlineStr">
         <is>
@@ -1012,16 +1012,16 @@
         <v>130</v>
       </c>
       <c r="E6" t="n">
-        <v>29543.51</v>
+        <v>29543.5</v>
       </c>
       <c r="F6" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="G6" t="n">
-        <v>801</v>
+        <v>804</v>
       </c>
       <c r="H6" t="n">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -1029,19 +1029,19 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>11.01</v>
+        <v>10.04</v>
       </c>
       <c r="K6" t="n">
         <v>7</v>
       </c>
       <c r="L6" t="n">
-        <v>29500</v>
+        <v>29498.75</v>
       </c>
       <c r="M6" t="n">
-        <v>29515</v>
+        <v>29513.75</v>
       </c>
       <c r="N6" t="n">
-        <v>29530</v>
+        <v>29528.75</v>
       </c>
       <c r="O6" t="n">
         <v>60</v>
@@ -1050,7 +1050,7 @@
         <v>60</v>
       </c>
       <c r="Q6" t="n">
-        <v>29530</v>
+        <v>29528.75</v>
       </c>
       <c r="R6" s="4" t="n">
         <v>60</v>
@@ -1066,10 +1066,10 @@
         </is>
       </c>
       <c r="U6" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="V6" t="n">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="W6" t="inlineStr">
         <is>
@@ -1085,7 +1085,7 @@
         <v>2312</v>
       </c>
       <c r="Z6" t="n">
-        <v>5.9038</v>
+        <v>5.9788</v>
       </c>
       <c r="AA6" t="inlineStr">
         <is>
@@ -1229,7 +1229,7 @@
         </is>
       </c>
       <c r="U7" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="V7" t="n">
         <v>60</v>

</xml_diff>

<commit_message>
A+ structure with small BUG
</commit_message>
<xml_diff>
--- a/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
+++ b/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
@@ -463,11 +463,11 @@
     </row>
     <row r="2">
       <c r="A2" s="1">
-        <f>IF((COUNTIF(R4:R7,"&gt;0")+COUNTIF(R4:R7,"&lt;0"))=0,"",COUNTIF(R4:R7,"&gt;0")/(COUNTIF(R4:R7,"&gt;0")+COUNTIF(R4:R7,"&lt;0")))</f>
+        <f>IF((COUNTIF(R4:R5,"&gt;0")+COUNTIF(R4:R5,"&lt;0"))=0,"",COUNTIF(R4:R5,"&gt;0")/(COUNTIF(R4:R5,"&gt;0")+COUNTIF(R4:R5,"&lt;0")))</f>
         <v/>
       </c>
       <c r="B2" s="2">
-        <f>IF(ABS(SUMIF(R4:R7,"&lt;0",R4:R7))=0,IF(SUMIF(R4:R7,"&gt;0",R4:R7)&gt;0,"INF",""),SUMIF(R4:R7,"&gt;0",R4:R7)/ABS(SUMIF(R4:R7,"&lt;0",R4:R7)))</f>
+        <f>IF(ABS(SUMIF(R4:R5,"&lt;0",R4:R5))=0,IF(SUMIF(R4:R5,"&gt;0",R4:R5)&gt;0,"INF",""),SUMIF(R4:R5,"&gt;0",R4:R5)/ABS(SUMIF(R4:R5,"&lt;0",R4:R5)))</f>
         <v/>
       </c>
     </row>
@@ -681,49 +681,49 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>26852.5</v>
+        <v>29460</v>
       </c>
       <c r="C4" t="n">
-        <v>26893.75</v>
+        <v>29492.5</v>
       </c>
       <c r="D4" t="n">
-        <v>165</v>
+        <v>130</v>
       </c>
       <c r="E4" t="n">
-        <v>26841.85</v>
+        <v>29543.5</v>
       </c>
       <c r="F4" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="G4" t="n">
-        <v>1313</v>
+        <v>805</v>
       </c>
       <c r="H4" t="n">
-        <v>-117</v>
+        <v>261</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>normal speed</t>
+          <t>A+ speed</t>
         </is>
       </c>
       <c r="J4" t="n">
-        <v>2.1</v>
+        <v>9.99</v>
       </c>
       <c r="K4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L4" t="n">
-        <v>26836.25</v>
+        <v>29498.75</v>
       </c>
       <c r="M4" t="n">
-        <v>26821.25</v>
+        <v>29513.75</v>
       </c>
       <c r="N4" t="n">
-        <v>26806.25</v>
+        <v>29528.75</v>
       </c>
       <c r="O4" t="n">
         <v>60</v>
@@ -732,26 +732,26 @@
         <v>60</v>
       </c>
       <c r="Q4" t="n">
-        <v>26836.25</v>
+        <v>29528.75</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>-60</v>
+        <v>60</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>SCALP_NORMAL</t>
+          <t>POTENTIAL_RUNNER</t>
         </is>
       </c>
       <c r="U4" t="n">
-        <v>65</v>
+        <v>0</v>
       </c>
       <c r="V4" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="W4" t="inlineStr">
         <is>
@@ -760,14 +760,14 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>09:33:00</t>
+          <t>09:32:00</t>
         </is>
       </c>
       <c r="Y4" t="n">
         <v>2312</v>
       </c>
       <c r="Z4" t="n">
-        <v>33.3476</v>
+        <v>6.0088</v>
       </c>
       <c r="AA4" t="inlineStr">
         <is>
@@ -806,7 +806,7 @@
       </c>
       <c r="AH4" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="AI4" t="inlineStr">
@@ -816,24 +816,16 @@
       </c>
       <c r="AJ4" t="inlineStr">
         <is>
-          <t>SL</t>
+          <t>TP</t>
         </is>
       </c>
       <c r="AK4" t="inlineStr">
         <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AL4" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="AM4" t="n">
-        <v>26852.5</v>
+          <t>FALSE</t>
+        </is>
       </c>
       <c r="AN4" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AO4" t="inlineStr">
         <is>
@@ -844,49 +836,49 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>29252.5</v>
+        <v>29241.25</v>
       </c>
       <c r="C5" t="n">
-        <v>29288.75</v>
+        <v>29291.25</v>
       </c>
       <c r="D5" t="n">
-        <v>145</v>
+        <v>200</v>
       </c>
       <c r="E5" t="n">
-        <v>29321.36</v>
+        <v>29294.78</v>
       </c>
       <c r="F5" t="n">
-        <v>35</v>
+        <v>90</v>
       </c>
       <c r="G5" t="n">
-        <v>1113</v>
+        <v>821</v>
       </c>
       <c r="H5" t="n">
-        <v>-175</v>
+        <v>-355</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>normal speed</t>
+          <t>A+ speed</t>
         </is>
       </c>
       <c r="J5" t="n">
-        <v>2.08</v>
+        <v>17.73</v>
       </c>
       <c r="K5" t="n">
         <v>8</v>
       </c>
       <c r="L5" t="n">
-        <v>29258.75</v>
+        <v>29233.75</v>
       </c>
       <c r="M5" t="n">
-        <v>29243.75</v>
+        <v>29218.75</v>
       </c>
       <c r="N5" t="n">
-        <v>29228.75</v>
+        <v>29203.75</v>
       </c>
       <c r="O5" t="n">
         <v>60</v>
@@ -895,7 +887,7 @@
         <v>60</v>
       </c>
       <c r="Q5" t="n">
-        <v>29228.75</v>
+        <v>29203.75</v>
       </c>
       <c r="R5" s="4" t="n">
         <v>60</v>
@@ -907,11 +899,11 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>SCALP_NORMAL</t>
+          <t>POTENTIAL_RUNNER</t>
         </is>
       </c>
       <c r="U5" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="V5" t="n">
         <v>60</v>
@@ -930,7 +922,7 @@
         <v>2311</v>
       </c>
       <c r="Z5" t="n">
-        <v>16.8109</v>
+        <v>5.0756</v>
       </c>
       <c r="AA5" t="inlineStr">
         <is>
@@ -997,322 +989,10 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>29460</v>
-      </c>
-      <c r="C6" t="n">
-        <v>29492.5</v>
-      </c>
-      <c r="D6" t="n">
-        <v>130</v>
-      </c>
-      <c r="E6" t="n">
-        <v>29543.5</v>
-      </c>
-      <c r="F6" t="n">
-        <v>60</v>
-      </c>
-      <c r="G6" t="n">
-        <v>804</v>
-      </c>
-      <c r="H6" t="n">
-        <v>262</v>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>A+ speed</t>
-        </is>
-      </c>
-      <c r="J6" t="n">
-        <v>10.04</v>
-      </c>
-      <c r="K6" t="n">
-        <v>7</v>
-      </c>
-      <c r="L6" t="n">
-        <v>29498.75</v>
-      </c>
-      <c r="M6" t="n">
-        <v>29513.75</v>
-      </c>
-      <c r="N6" t="n">
-        <v>29528.75</v>
-      </c>
-      <c r="O6" t="n">
-        <v>60</v>
-      </c>
-      <c r="P6" t="n">
-        <v>60</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>29528.75</v>
-      </c>
-      <c r="R6" s="4" t="n">
-        <v>60</v>
-      </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="T6" t="inlineStr">
-        <is>
-          <t>POTENTIAL_RUNNER</t>
-        </is>
-      </c>
-      <c r="U6" t="n">
-        <v>15</v>
-      </c>
-      <c r="V6" t="n">
-        <v>65</v>
-      </c>
-      <c r="W6" t="inlineStr">
-        <is>
-          <t>score-exporter-2026-05-30-aplus-structure-export</t>
-        </is>
-      </c>
-      <c r="X6" t="inlineStr">
-        <is>
-          <t>09:32:00</t>
-        </is>
-      </c>
-      <c r="Y6" t="n">
-        <v>2312</v>
-      </c>
-      <c r="Z6" t="n">
-        <v>5.9788</v>
-      </c>
-      <c r="AA6" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AB6" t="inlineStr">
-        <is>
-          <t>LastTime</t>
-        </is>
-      </c>
-      <c r="AC6" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AD6" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AE6" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AF6" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AG6" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AH6" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AI6" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AJ6" t="inlineStr">
-        <is>
-          <t>TP</t>
-        </is>
-      </c>
-      <c r="AK6" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AL6" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="AM6" t="n">
-        <v>29501.25</v>
-      </c>
-      <c r="AN6" t="n">
-        <v>3</v>
-      </c>
-      <c r="AO6" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
+      <c r="R6" s="4" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>29241.25</v>
-      </c>
-      <c r="C7" t="n">
-        <v>29291.25</v>
-      </c>
-      <c r="D7" t="n">
-        <v>200</v>
-      </c>
-      <c r="E7" t="n">
-        <v>29294.78</v>
-      </c>
-      <c r="F7" t="n">
-        <v>90</v>
-      </c>
-      <c r="G7" t="n">
-        <v>814</v>
-      </c>
-      <c r="H7" t="n">
-        <v>-358</v>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>A+ speed</t>
-        </is>
-      </c>
-      <c r="J7" t="n">
-        <v>18.05</v>
-      </c>
-      <c r="K7" t="n">
-        <v>9</v>
-      </c>
-      <c r="L7" t="n">
-        <v>29233.75</v>
-      </c>
-      <c r="M7" t="n">
-        <v>29218.75</v>
-      </c>
-      <c r="N7" t="n">
-        <v>29203.75</v>
-      </c>
-      <c r="O7" t="n">
-        <v>60</v>
-      </c>
-      <c r="P7" t="n">
-        <v>60</v>
-      </c>
-      <c r="Q7" t="n">
-        <v>29203.75</v>
-      </c>
-      <c r="R7" s="4" t="n">
-        <v>60</v>
-      </c>
-      <c r="S7" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="T7" t="inlineStr">
-        <is>
-          <t>POTENTIAL_RUNNER</t>
-        </is>
-      </c>
-      <c r="U7" t="n">
-        <v>25</v>
-      </c>
-      <c r="V7" t="n">
-        <v>60</v>
-      </c>
-      <c r="W7" t="inlineStr">
-        <is>
-          <t>score-exporter-2026-05-30-aplus-structure-export</t>
-        </is>
-      </c>
-      <c r="X7" t="inlineStr">
-        <is>
-          <t>09:31:00</t>
-        </is>
-      </c>
-      <c r="Y7" t="n">
-        <v>2311</v>
-      </c>
-      <c r="Z7" t="n">
-        <v>4.9856</v>
-      </c>
-      <c r="AA7" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AB7" t="inlineStr">
-        <is>
-          <t>LastTime</t>
-        </is>
-      </c>
-      <c r="AC7" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AD7" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AE7" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AF7" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AG7" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AH7" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AI7" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AJ7" t="inlineStr">
-        <is>
-          <t>TP</t>
-        </is>
-      </c>
-      <c r="AK7" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AN7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO7" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
+      <c r="R7" s="4" t="n"/>
     </row>
     <row r="8">
       <c r="R8" s="4" t="n"/>

</xml_diff>

<commit_message>
ETIQUETAS Y LINEAS DE DEBUG  para A+ STRUCTURE
</commit_message>
<xml_diff>
--- a/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
+++ b/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
@@ -681,49 +681,49 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>29460</v>
+        <v>26852.5</v>
       </c>
       <c r="C4" t="n">
-        <v>29492.5</v>
+        <v>26893.75</v>
       </c>
       <c r="D4" t="n">
-        <v>130</v>
+        <v>165</v>
       </c>
       <c r="E4" t="n">
-        <v>29543.5</v>
+        <v>26842.09</v>
       </c>
       <c r="F4" t="n">
-        <v>60</v>
+        <v>5</v>
       </c>
       <c r="G4" t="n">
-        <v>805</v>
+        <v>1168</v>
       </c>
       <c r="H4" t="n">
-        <v>261</v>
+        <v>-230</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>A+ speed</t>
+          <t>normal speed</t>
         </is>
       </c>
       <c r="J4" t="n">
-        <v>9.99</v>
+        <v>0.14</v>
       </c>
       <c r="K4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L4" t="n">
-        <v>29498.75</v>
+        <v>26866.25</v>
       </c>
       <c r="M4" t="n">
-        <v>29513.75</v>
+        <v>26851.25</v>
       </c>
       <c r="N4" t="n">
-        <v>29528.75</v>
+        <v>26836.25</v>
       </c>
       <c r="O4" t="n">
         <v>60</v>
@@ -732,19 +732,19 @@
         <v>60</v>
       </c>
       <c r="Q4" t="n">
-        <v>29528.75</v>
+        <v>26836.25</v>
       </c>
       <c r="R4" s="4" t="n">
         <v>60</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>POTENTIAL_RUNNER</t>
+          <t>SCALP_NORMAL</t>
         </is>
       </c>
       <c r="U4" t="n">
@@ -764,10 +764,10 @@
         </is>
       </c>
       <c r="Y4" t="n">
-        <v>2312</v>
+        <v>2311</v>
       </c>
       <c r="Z4" t="n">
-        <v>6.0088</v>
+        <v>35.6594</v>
       </c>
       <c r="AA4" t="inlineStr">
         <is>
@@ -776,7 +776,7 @@
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>LastTime</t>
+          <t>A+ structure</t>
         </is>
       </c>
       <c r="AC4" t="inlineStr">
@@ -786,7 +786,7 @@
       </c>
       <c r="AD4" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="AE4" t="inlineStr">
@@ -821,64 +821,72 @@
       </c>
       <c r="AK4" t="inlineStr">
         <is>
-          <t>FALSE</t>
-        </is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AL4" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="AM4" t="n">
+        <v>26852.5</v>
       </c>
       <c r="AN4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AO4" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>29241.25</v>
+        <v>29460</v>
       </c>
       <c r="C5" t="n">
-        <v>29291.25</v>
+        <v>29492.5</v>
       </c>
       <c r="D5" t="n">
-        <v>200</v>
+        <v>130</v>
       </c>
       <c r="E5" t="n">
-        <v>29294.78</v>
+        <v>29544.64</v>
       </c>
       <c r="F5" t="n">
-        <v>90</v>
+        <v>40</v>
       </c>
       <c r="G5" t="n">
-        <v>821</v>
+        <v>1620</v>
       </c>
       <c r="H5" t="n">
-        <v>-355</v>
+        <v>0</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>A+ speed</t>
+          <t>normal speed</t>
         </is>
       </c>
       <c r="J5" t="n">
-        <v>17.73</v>
+        <v>1.89</v>
       </c>
       <c r="K5" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L5" t="n">
-        <v>29233.75</v>
+        <v>29487.5</v>
       </c>
       <c r="M5" t="n">
-        <v>29218.75</v>
+        <v>29502.5</v>
       </c>
       <c r="N5" t="n">
-        <v>29203.75</v>
+        <v>29517.5</v>
       </c>
       <c r="O5" t="n">
         <v>60</v>
@@ -886,27 +894,24 @@
       <c r="P5" t="n">
         <v>60</v>
       </c>
-      <c r="Q5" t="n">
-        <v>29203.75</v>
-      </c>
       <c r="R5" s="4" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>POTENTIAL_RUNNER</t>
+          <t>SCALP_NORMAL</t>
         </is>
       </c>
       <c r="U5" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="V5" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="W5" t="inlineStr">
         <is>
@@ -922,7 +927,7 @@
         <v>2311</v>
       </c>
       <c r="Z5" t="n">
-        <v>5.0756</v>
+        <v>21.22</v>
       </c>
       <c r="AA5" t="inlineStr">
         <is>
@@ -931,7 +936,7 @@
       </c>
       <c r="AB5" t="inlineStr">
         <is>
-          <t>LastTime</t>
+          <t>A+ structure</t>
         </is>
       </c>
       <c r="AC5" t="inlineStr">
@@ -951,7 +956,7 @@
       </c>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="AG5" t="inlineStr">
@@ -961,7 +966,7 @@
       </c>
       <c r="AH5" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="AI5" t="inlineStr">
@@ -971,20 +976,28 @@
       </c>
       <c r="AJ5" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>OPEN</t>
         </is>
       </c>
       <c r="AK5" t="inlineStr">
         <is>
-          <t>FALSE</t>
-        </is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AL5" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="AM5" t="n">
+        <v>29501.25</v>
       </c>
       <c r="AN5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AO5" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Commit antes de meter la absorcion, conservamos las etiquetas y laas lineas azules
</commit_message>
<xml_diff>
--- a/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
+++ b/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
@@ -463,11 +463,11 @@
     </row>
     <row r="2">
       <c r="A2" s="1">
-        <f>IF((COUNTIF(R4:R5,"&gt;0")+COUNTIF(R4:R5,"&lt;0"))=0,"",COUNTIF(R4:R5,"&gt;0")/(COUNTIF(R4:R5,"&gt;0")+COUNTIF(R4:R5,"&lt;0")))</f>
+        <f>IF((COUNTIF(R4:R25,"&gt;0")+COUNTIF(R4:R25,"&lt;0"))=0,"",COUNTIF(R4:R25,"&gt;0")/(COUNTIF(R4:R25,"&gt;0")+COUNTIF(R4:R25,"&lt;0")))</f>
         <v/>
       </c>
       <c r="B2" s="2">
-        <f>IF(ABS(SUMIF(R4:R5,"&lt;0",R4:R5))=0,IF(SUMIF(R4:R5,"&gt;0",R4:R5)&gt;0,"INF",""),SUMIF(R4:R5,"&gt;0",R4:R5)/ABS(SUMIF(R4:R5,"&lt;0",R4:R5)))</f>
+        <f>IF(ABS(SUMIF(R4:R25,"&lt;0",R4:R25))=0,IF(SUMIF(R4:R25,"&gt;0",R4:R25)&gt;0,"INF",""),SUMIF(R4:R25,"&gt;0",R4:R25)/ABS(SUMIF(R4:R25,"&lt;0",R4:R25)))</f>
         <v/>
       </c>
     </row>
@@ -681,29 +681,29 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>26852.5</v>
+        <v>26772.5</v>
       </c>
       <c r="C4" t="n">
-        <v>26893.75</v>
+        <v>26827.5</v>
       </c>
       <c r="D4" t="n">
-        <v>165</v>
+        <v>220</v>
       </c>
       <c r="E4" t="n">
-        <v>26842.09</v>
+        <v>26834.78</v>
       </c>
       <c r="F4" t="n">
-        <v>5</v>
+        <v>60</v>
       </c>
       <c r="G4" t="n">
-        <v>1168</v>
+        <v>2171</v>
       </c>
       <c r="H4" t="n">
-        <v>-230</v>
+        <v>-541</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -711,19 +711,19 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>0.14</v>
+        <v>2.01</v>
       </c>
       <c r="K4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L4" t="n">
-        <v>26866.25</v>
+        <v>26772.5</v>
       </c>
       <c r="M4" t="n">
-        <v>26851.25</v>
+        <v>26757.5</v>
       </c>
       <c r="N4" t="n">
-        <v>26836.25</v>
+        <v>26742.5</v>
       </c>
       <c r="O4" t="n">
         <v>60</v>
@@ -732,7 +732,7 @@
         <v>60</v>
       </c>
       <c r="Q4" t="n">
-        <v>26836.25</v>
+        <v>26742.5</v>
       </c>
       <c r="R4" s="4" t="n">
         <v>60</v>
@@ -748,125 +748,117 @@
         </is>
       </c>
       <c r="U4" t="n">
+        <v>25</v>
+      </c>
+      <c r="V4" t="n">
+        <v>65</v>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-aplus-structure-export</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>09:31:00</t>
+        </is>
+      </c>
+      <c r="Y4" t="n">
+        <v>2310</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>29.832</v>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ4" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="AK4" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AN4" t="n">
         <v>0</v>
       </c>
-      <c r="V4" t="n">
-        <v>60</v>
-      </c>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t>score-exporter-2026-05-30-aplus-structure-export</t>
-        </is>
-      </c>
-      <c r="X4" t="inlineStr">
-        <is>
-          <t>09:32:00</t>
-        </is>
-      </c>
-      <c r="Y4" t="n">
-        <v>2311</v>
-      </c>
-      <c r="Z4" t="n">
-        <v>35.6594</v>
-      </c>
-      <c r="AA4" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AB4" t="inlineStr">
-        <is>
-          <t>A+ structure</t>
-        </is>
-      </c>
-      <c r="AC4" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AD4" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AE4" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AF4" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AG4" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AH4" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AI4" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AJ4" t="inlineStr">
-        <is>
-          <t>TP</t>
-        </is>
-      </c>
-      <c r="AK4" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AL4" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="AM4" t="n">
-        <v>26852.5</v>
-      </c>
-      <c r="AN4" t="n">
-        <v>3</v>
-      </c>
       <c r="AO4" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>29460</v>
+        <v>26852.5</v>
       </c>
       <c r="C5" t="n">
-        <v>29492.5</v>
+        <v>26893.75</v>
       </c>
       <c r="D5" t="n">
-        <v>130</v>
+        <v>165</v>
       </c>
       <c r="E5" t="n">
-        <v>29544.64</v>
+        <v>26842.08</v>
       </c>
       <c r="F5" t="n">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="G5" t="n">
-        <v>1620</v>
+        <v>1177</v>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>-233</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -874,19 +866,19 @@
         </is>
       </c>
       <c r="J5" t="n">
-        <v>1.89</v>
+        <v>0.28</v>
       </c>
       <c r="K5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L5" t="n">
-        <v>29487.5</v>
+        <v>26865</v>
       </c>
       <c r="M5" t="n">
-        <v>29502.5</v>
+        <v>26850</v>
       </c>
       <c r="N5" t="n">
-        <v>29517.5</v>
+        <v>26835</v>
       </c>
       <c r="O5" t="n">
         <v>60</v>
@@ -894,12 +886,15 @@
       <c r="P5" t="n">
         <v>60</v>
       </c>
+      <c r="Q5" t="n">
+        <v>26835</v>
+      </c>
       <c r="R5" s="4" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -911,7 +906,7 @@
         <v>0</v>
       </c>
       <c r="V5" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="W5" t="inlineStr">
         <is>
@@ -920,14 +915,14 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>09:31:00</t>
+          <t>09:32:00</t>
         </is>
       </c>
       <c r="Y5" t="n">
         <v>2311</v>
       </c>
       <c r="Z5" t="n">
-        <v>21.22</v>
+        <v>36.081</v>
       </c>
       <c r="AA5" t="inlineStr">
         <is>
@@ -956,7 +951,7 @@
       </c>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="AG5" t="inlineStr">
@@ -976,7 +971,7 @@
       </c>
       <c r="AJ5" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>TP</t>
         </is>
       </c>
       <c r="AK5" t="inlineStr">
@@ -986,11 +981,11 @@
       </c>
       <c r="AL5" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="AM5" t="n">
-        <v>29501.25</v>
+        <v>26852.5</v>
       </c>
       <c r="AN5" t="n">
         <v>3</v>
@@ -1002,64 +997,2847 @@
       </c>
     </row>
     <row r="6">
-      <c r="R6" s="4" t="n"/>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>26965</v>
+      </c>
+      <c r="C6" t="n">
+        <v>27016.25</v>
+      </c>
+      <c r="D6" t="n">
+        <v>205</v>
+      </c>
+      <c r="E6" t="n">
+        <v>26988.51</v>
+      </c>
+      <c r="F6" t="n">
+        <v>5</v>
+      </c>
+      <c r="G6" t="n">
+        <v>802</v>
+      </c>
+      <c r="H6" t="n">
+        <v>202</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>normal speed</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="K6" t="n">
+        <v>7</v>
+      </c>
+      <c r="L6" t="n">
+        <v>27002.5</v>
+      </c>
+      <c r="M6" t="n">
+        <v>27017.5</v>
+      </c>
+      <c r="N6" t="n">
+        <v>27032.5</v>
+      </c>
+      <c r="O6" t="n">
+        <v>60</v>
+      </c>
+      <c r="P6" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>27032.5</v>
+      </c>
+      <c r="R6" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>SCALP_NORMAL</t>
+        </is>
+      </c>
+      <c r="U6" t="n">
+        <v>25</v>
+      </c>
+      <c r="V6" t="n">
+        <v>60</v>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-aplus-structure-export</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>09:35:00</t>
+        </is>
+      </c>
+      <c r="Y6" t="n">
+        <v>2315</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>19.3289</v>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>A+ structure</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ6" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="AK6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AL6" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="AM6" t="n">
+        <v>27018.75</v>
+      </c>
+      <c r="AN6" t="n">
+        <v>3</v>
+      </c>
+      <c r="AO6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="R7" s="4" t="n"/>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>27176.25</v>
+      </c>
+      <c r="C7" t="n">
+        <v>27223.75</v>
+      </c>
+      <c r="D7" t="n">
+        <v>190</v>
+      </c>
+      <c r="E7" t="n">
+        <v>27208.53</v>
+      </c>
+      <c r="F7" t="n">
+        <v>50</v>
+      </c>
+      <c r="G7" t="n">
+        <v>803</v>
+      </c>
+      <c r="H7" t="n">
+        <v>109</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>normal speed</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>2.01</v>
+      </c>
+      <c r="K7" t="n">
+        <v>7</v>
+      </c>
+      <c r="L7" t="n">
+        <v>27222.5</v>
+      </c>
+      <c r="M7" t="n">
+        <v>27237.5</v>
+      </c>
+      <c r="N7" t="n">
+        <v>27252.5</v>
+      </c>
+      <c r="O7" t="n">
+        <v>60</v>
+      </c>
+      <c r="P7" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>27222.5</v>
+      </c>
+      <c r="R7" s="4" t="n">
+        <v>-60</v>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>SCALP_NORMAL</t>
+        </is>
+      </c>
+      <c r="U7" t="n">
+        <v>60</v>
+      </c>
+      <c r="V7" t="n">
+        <v>35</v>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-aplus-structure-export</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>09:34:00</t>
+        </is>
+      </c>
+      <c r="Y7" t="n">
+        <v>2314</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>24.9169</v>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE7" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF7" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG7" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH7" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI7" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ7" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="AK7" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AN7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO7" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="R8" s="4" t="n"/>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="R8" s="4" t="inlineStr">
+        <is>
+          <t>NO_CSV</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="R9" s="4" t="n"/>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>27082.5</v>
+      </c>
+      <c r="C9" t="n">
+        <v>27162.5</v>
+      </c>
+      <c r="D9" t="n">
+        <v>320</v>
+      </c>
+      <c r="E9" t="n">
+        <v>27189.24</v>
+      </c>
+      <c r="F9" t="n">
+        <v>15</v>
+      </c>
+      <c r="G9" t="n">
+        <v>1528</v>
+      </c>
+      <c r="H9" t="n">
+        <v>44</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>normal speed</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="K9" t="n">
+        <v>8</v>
+      </c>
+      <c r="L9" t="n">
+        <v>27162.5</v>
+      </c>
+      <c r="M9" t="n">
+        <v>27177.5</v>
+      </c>
+      <c r="N9" t="n">
+        <v>27192.5</v>
+      </c>
+      <c r="O9" t="n">
+        <v>60</v>
+      </c>
+      <c r="P9" t="n">
+        <v>60</v>
+      </c>
+      <c r="R9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>SCALP_NORMAL</t>
+        </is>
+      </c>
+      <c r="U9" t="n">
+        <v>0</v>
+      </c>
+      <c r="V9" t="n">
+        <v>0</v>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-aplus-structure-export</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>09:37:00</t>
+        </is>
+      </c>
+      <c r="Y9" t="n">
+        <v>2317</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>49.6574</v>
+      </c>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>A+ structure</t>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF9" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG9" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH9" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AI9" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ9" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="AK9" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AL9" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="AM9" t="n">
+        <v>27181.25</v>
+      </c>
+      <c r="AN9" t="n">
+        <v>3</v>
+      </c>
+      <c r="AO9" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="R10" s="4" t="n"/>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>27151.25</v>
+      </c>
+      <c r="C10" t="n">
+        <v>27218.75</v>
+      </c>
+      <c r="D10" t="n">
+        <v>270</v>
+      </c>
+      <c r="E10" t="n">
+        <v>27241.75</v>
+      </c>
+      <c r="F10" t="n">
+        <v>15</v>
+      </c>
+      <c r="G10" t="n">
+        <v>805</v>
+      </c>
+      <c r="H10" t="n">
+        <v>-89</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>normal speed</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="K10" t="n">
+        <v>8</v>
+      </c>
+      <c r="L10" t="n">
+        <v>27162.5</v>
+      </c>
+      <c r="M10" t="n">
+        <v>27147.5</v>
+      </c>
+      <c r="N10" t="n">
+        <v>27132.5</v>
+      </c>
+      <c r="O10" t="n">
+        <v>60</v>
+      </c>
+      <c r="P10" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>27162.5</v>
+      </c>
+      <c r="R10" s="4" t="n">
+        <v>-60</v>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>SCALP_NORMAL</t>
+        </is>
+      </c>
+      <c r="U10" t="n">
+        <v>60</v>
+      </c>
+      <c r="V10" t="n">
+        <v>40</v>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-aplus-structure-export</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>09:31:00</t>
+        </is>
+      </c>
+      <c r="Y10" t="n">
+        <v>2311</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>6.4496</v>
+      </c>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE10" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF10" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG10" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH10" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI10" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ10" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="AK10" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AN10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO10" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="R11" s="4" t="n"/>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>27422.5</v>
+      </c>
+      <c r="C11" t="n">
+        <v>27492.5</v>
+      </c>
+      <c r="D11" t="n">
+        <v>280</v>
+      </c>
+      <c r="E11" t="n">
+        <v>27385.42</v>
+      </c>
+      <c r="F11" t="n">
+        <v>30</v>
+      </c>
+      <c r="G11" t="n">
+        <v>984</v>
+      </c>
+      <c r="H11" t="n">
+        <v>-110</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>normal speed</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>2.55</v>
+      </c>
+      <c r="K11" t="n">
+        <v>6</v>
+      </c>
+      <c r="L11" t="n">
+        <v>27430</v>
+      </c>
+      <c r="M11" t="n">
+        <v>27415</v>
+      </c>
+      <c r="N11" t="n">
+        <v>27400</v>
+      </c>
+      <c r="O11" t="n">
+        <v>60</v>
+      </c>
+      <c r="P11" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>27400</v>
+      </c>
+      <c r="R11" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>SCALP_NORMAL</t>
+        </is>
+      </c>
+      <c r="U11" t="n">
+        <v>45</v>
+      </c>
+      <c r="V11" t="n">
+        <v>60</v>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-aplus-structure-export</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>09:31:00</t>
+        </is>
+      </c>
+      <c r="Y11" t="n">
+        <v>2311</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>11.7789</v>
+      </c>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE11" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF11" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG11" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH11" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AI11" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ11" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="AK11" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AN11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO11" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="R12" s="4" t="n"/>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>27618.75</v>
+      </c>
+      <c r="C12" t="n">
+        <v>27666.25</v>
+      </c>
+      <c r="D12" t="n">
+        <v>190</v>
+      </c>
+      <c r="E12" t="n">
+        <v>27598.31</v>
+      </c>
+      <c r="F12" t="n">
+        <v>20</v>
+      </c>
+      <c r="G12" t="n">
+        <v>854</v>
+      </c>
+      <c r="H12" t="n">
+        <v>254</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>normal speed</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>2.59</v>
+      </c>
+      <c r="K12" t="n">
+        <v>8</v>
+      </c>
+      <c r="L12" t="n">
+        <v>27656.25</v>
+      </c>
+      <c r="M12" t="n">
+        <v>27671.25</v>
+      </c>
+      <c r="N12" t="n">
+        <v>27686.25</v>
+      </c>
+      <c r="O12" t="n">
+        <v>60</v>
+      </c>
+      <c r="P12" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>27686.25</v>
+      </c>
+      <c r="R12" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>SCALP_NORMAL</t>
+        </is>
+      </c>
+      <c r="U12" t="n">
+        <v>5</v>
+      </c>
+      <c r="V12" t="n">
+        <v>60</v>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-aplus-structure-export</t>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>09:31:00</t>
+        </is>
+      </c>
+      <c r="Y12" t="n">
+        <v>2311</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>7.7202</v>
+      </c>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AB12" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE12" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF12" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG12" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH12" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI12" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ12" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="AK12" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AN12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO12" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="R13" s="4" t="n"/>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>27837.5</v>
+      </c>
+      <c r="C13" t="n">
+        <v>27875</v>
+      </c>
+      <c r="D13" t="n">
+        <v>150</v>
+      </c>
+      <c r="E13" t="n">
+        <v>27837.02</v>
+      </c>
+      <c r="F13" t="n">
+        <v>40</v>
+      </c>
+      <c r="G13" t="n">
+        <v>1284</v>
+      </c>
+      <c r="H13" t="n">
+        <v>10</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>normal speed</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>2.26</v>
+      </c>
+      <c r="K13" t="n">
+        <v>7</v>
+      </c>
+      <c r="L13" t="n">
+        <v>27842.5</v>
+      </c>
+      <c r="M13" t="n">
+        <v>27827.5</v>
+      </c>
+      <c r="N13" t="n">
+        <v>27812.5</v>
+      </c>
+      <c r="O13" t="n">
+        <v>60</v>
+      </c>
+      <c r="P13" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>27812.5</v>
+      </c>
+      <c r="R13" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>SCALP_NORMAL</t>
+        </is>
+      </c>
+      <c r="U13" t="n">
+        <v>10</v>
+      </c>
+      <c r="V13" t="n">
+        <v>60</v>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-aplus-structure-export</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>09:31:00</t>
+        </is>
+      </c>
+      <c r="Y13" t="n">
+        <v>2311</v>
+      </c>
+      <c r="Z13" t="n">
+        <v>17.7163</v>
+      </c>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AB13" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE13" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF13" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AG13" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH13" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI13" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ13" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="AK13" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AN13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO13" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="R14" s="4" t="n"/>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>27986.25</v>
+      </c>
+      <c r="C14" t="n">
+        <v>28023.75</v>
+      </c>
+      <c r="D14" t="n">
+        <v>150</v>
+      </c>
+      <c r="E14" t="n">
+        <v>27935.7</v>
+      </c>
+      <c r="F14" t="n">
+        <v>15</v>
+      </c>
+      <c r="G14" t="n">
+        <v>836</v>
+      </c>
+      <c r="H14" t="n">
+        <v>-136</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>normal speed</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="K14" t="n">
+        <v>6</v>
+      </c>
+      <c r="L14" t="n">
+        <v>27997.5</v>
+      </c>
+      <c r="M14" t="n">
+        <v>27982.5</v>
+      </c>
+      <c r="N14" t="n">
+        <v>27967.5</v>
+      </c>
+      <c r="O14" t="n">
+        <v>60</v>
+      </c>
+      <c r="P14" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>27997.5</v>
+      </c>
+      <c r="R14" s="4" t="n">
+        <v>-60</v>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>SCALP_NORMAL</t>
+        </is>
+      </c>
+      <c r="U14" t="n">
+        <v>60</v>
+      </c>
+      <c r="V14" t="n">
+        <v>45</v>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-aplus-structure-export</t>
+        </is>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>09:31:00</t>
+        </is>
+      </c>
+      <c r="Y14" t="n">
+        <v>2310</v>
+      </c>
+      <c r="Z14" t="n">
+        <v>5.4468</v>
+      </c>
+      <c r="AA14" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AB14" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE14" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF14" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG14" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH14" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AI14" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ14" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="AK14" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AN14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO14" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="R15" s="4" t="n"/>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>28336.25</v>
+      </c>
+      <c r="C15" t="n">
+        <v>28392.5</v>
+      </c>
+      <c r="D15" t="n">
+        <v>225</v>
+      </c>
+      <c r="E15" t="n">
+        <v>28455.83</v>
+      </c>
+      <c r="F15" t="n">
+        <v>25</v>
+      </c>
+      <c r="G15" t="n">
+        <v>835</v>
+      </c>
+      <c r="H15" t="n">
+        <v>27</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>normal speed</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="K15" t="n">
+        <v>6</v>
+      </c>
+      <c r="L15" t="n">
+        <v>28411.25</v>
+      </c>
+      <c r="M15" t="n">
+        <v>28426.25</v>
+      </c>
+      <c r="N15" t="n">
+        <v>28441.25</v>
+      </c>
+      <c r="O15" t="n">
+        <v>60</v>
+      </c>
+      <c r="P15" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>28411.25</v>
+      </c>
+      <c r="R15" s="4" t="n">
+        <v>-60</v>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>SCALP_NORMAL</t>
+        </is>
+      </c>
+      <c r="U15" t="n">
+        <v>60</v>
+      </c>
+      <c r="V15" t="n">
+        <v>0</v>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-aplus-structure-export</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>09:33:00</t>
+        </is>
+      </c>
+      <c r="Y15" t="n">
+        <v>2313</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>11.7309</v>
+      </c>
+      <c r="AA15" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AB15" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AC15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH15" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AI15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ15" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="AK15" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AN15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO15" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="R16" s="4" t="n"/>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>28730</v>
+      </c>
+      <c r="C16" t="n">
+        <v>28766.25</v>
+      </c>
+      <c r="D16" t="n">
+        <v>145</v>
+      </c>
+      <c r="E16" t="n">
+        <v>28744.56</v>
+      </c>
+      <c r="F16" t="n">
+        <v>40</v>
+      </c>
+      <c r="G16" t="n">
+        <v>1441</v>
+      </c>
+      <c r="H16" t="n">
+        <v>241</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>normal speed</t>
+        </is>
+      </c>
+      <c r="J16" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="K16" t="n">
+        <v>10</v>
+      </c>
+      <c r="L16" t="n">
+        <v>28761.25</v>
+      </c>
+      <c r="M16" t="n">
+        <v>28776.25</v>
+      </c>
+      <c r="N16" t="n">
+        <v>28791.25</v>
+      </c>
+      <c r="O16" t="n">
+        <v>60</v>
+      </c>
+      <c r="P16" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>28761.25</v>
+      </c>
+      <c r="R16" s="4" t="n">
+        <v>-60</v>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>SCALP_NORMAL</t>
+        </is>
+      </c>
+      <c r="U16" t="n">
+        <v>60</v>
+      </c>
+      <c r="V16" t="n">
+        <v>0</v>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-aplus-structure-export</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>09:38:00</t>
+        </is>
+      </c>
+      <c r="Y16" t="n">
+        <v>2318</v>
+      </c>
+      <c r="Z16" t="n">
+        <v>57.6084</v>
+      </c>
+      <c r="AA16" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AB16" t="inlineStr">
+        <is>
+          <t>A+ structure</t>
+        </is>
+      </c>
+      <c r="AC16" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD16" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE16" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF16" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG16" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH16" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI16" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ16" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="AK16" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AL16" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="AM16" t="n">
+        <v>28777.5</v>
+      </c>
+      <c r="AN16" t="n">
+        <v>3</v>
+      </c>
+      <c r="AO16" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="R17" s="4" t="n"/>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>28860</v>
+      </c>
+      <c r="C17" t="n">
+        <v>28903.75</v>
+      </c>
+      <c r="D17" t="n">
+        <v>175</v>
+      </c>
+      <c r="E17" t="n">
+        <v>28876.6</v>
+      </c>
+      <c r="F17" t="n">
+        <v>50</v>
+      </c>
+      <c r="G17" t="n">
+        <v>1573</v>
+      </c>
+      <c r="H17" t="n">
+        <v>209</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>normal speed</t>
+        </is>
+      </c>
+      <c r="J17" t="n">
+        <v>2.19</v>
+      </c>
+      <c r="K17" t="n">
+        <v>8</v>
+      </c>
+      <c r="L17" t="n">
+        <v>28901.25</v>
+      </c>
+      <c r="M17" t="n">
+        <v>28916.25</v>
+      </c>
+      <c r="N17" t="n">
+        <v>28931.25</v>
+      </c>
+      <c r="O17" t="n">
+        <v>60</v>
+      </c>
+      <c r="P17" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>28931.25</v>
+      </c>
+      <c r="R17" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>SCALP_NORMAL</t>
+        </is>
+      </c>
+      <c r="U17" t="n">
+        <v>45</v>
+      </c>
+      <c r="V17" t="n">
+        <v>65</v>
+      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-aplus-structure-export</t>
+        </is>
+      </c>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>09:31:00</t>
+        </is>
+      </c>
+      <c r="Y17" t="n">
+        <v>2311</v>
+      </c>
+      <c r="Z17" t="n">
+        <v>22.8326</v>
+      </c>
+      <c r="AA17" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AB17" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE17" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF17" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG17" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH17" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI17" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ17" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="AK17" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AN17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO17" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="R18" s="4" t="n"/>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>29282.5</v>
+      </c>
+      <c r="C18" t="n">
+        <v>29346.25</v>
+      </c>
+      <c r="D18" t="n">
+        <v>255</v>
+      </c>
+      <c r="E18" t="n">
+        <v>29316.62</v>
+      </c>
+      <c r="F18" t="n">
+        <v>75</v>
+      </c>
+      <c r="G18" t="n">
+        <v>817</v>
+      </c>
+      <c r="H18" t="n">
+        <v>137</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>A+ speed</t>
+        </is>
+      </c>
+      <c r="J18" t="n">
+        <v>10.68</v>
+      </c>
+      <c r="K18" t="n">
+        <v>9</v>
+      </c>
+      <c r="L18" t="n">
+        <v>29350</v>
+      </c>
+      <c r="M18" t="n">
+        <v>29365</v>
+      </c>
+      <c r="N18" t="n">
+        <v>29380</v>
+      </c>
+      <c r="O18" t="n">
+        <v>60</v>
+      </c>
+      <c r="P18" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>29380</v>
+      </c>
+      <c r="R18" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>POTENTIAL_RUNNER</t>
+        </is>
+      </c>
+      <c r="U18" t="n">
+        <v>15</v>
+      </c>
+      <c r="V18" t="n">
+        <v>60</v>
+      </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-aplus-structure-export</t>
+        </is>
+      </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>09:31:00</t>
+        </is>
+      </c>
+      <c r="Y18" t="n">
+        <v>2311</v>
+      </c>
+      <c r="Z18" t="n">
+        <v>7.0252</v>
+      </c>
+      <c r="AA18" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AB18" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AC18" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD18" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE18" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF18" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG18" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH18" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI18" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ18" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="AK18" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AN18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO18" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="R19" s="4" t="n"/>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="R19" s="4" t="inlineStr">
+        <is>
+          <t>NO_CSV</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="R20" s="4" t="n"/>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>29252.5</v>
+      </c>
+      <c r="C20" t="n">
+        <v>29288.75</v>
+      </c>
+      <c r="D20" t="n">
+        <v>145</v>
+      </c>
+      <c r="E20" t="n">
+        <v>29321.36</v>
+      </c>
+      <c r="F20" t="n">
+        <v>35</v>
+      </c>
+      <c r="G20" t="n">
+        <v>1113</v>
+      </c>
+      <c r="H20" t="n">
+        <v>-175</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>normal speed</t>
+        </is>
+      </c>
+      <c r="J20" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="K20" t="n">
+        <v>8</v>
+      </c>
+      <c r="L20" t="n">
+        <v>29258.75</v>
+      </c>
+      <c r="M20" t="n">
+        <v>29243.75</v>
+      </c>
+      <c r="N20" t="n">
+        <v>29228.75</v>
+      </c>
+      <c r="O20" t="n">
+        <v>60</v>
+      </c>
+      <c r="P20" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>29228.75</v>
+      </c>
+      <c r="R20" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>SCALP_NORMAL</t>
+        </is>
+      </c>
+      <c r="U20" t="n">
+        <v>0</v>
+      </c>
+      <c r="V20" t="n">
+        <v>60</v>
+      </c>
+      <c r="W20" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-aplus-structure-export</t>
+        </is>
+      </c>
+      <c r="X20" t="inlineStr">
+        <is>
+          <t>09:31:00</t>
+        </is>
+      </c>
+      <c r="Y20" t="n">
+        <v>2311</v>
+      </c>
+      <c r="Z20" t="n">
+        <v>16.8109</v>
+      </c>
+      <c r="AA20" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AB20" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AC20" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD20" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE20" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF20" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG20" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH20" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI20" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ20" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="AK20" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AN20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO20" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="R21" s="4" t="n"/>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>29460</v>
+      </c>
+      <c r="C21" t="n">
+        <v>29492.5</v>
+      </c>
+      <c r="D21" t="n">
+        <v>130</v>
+      </c>
+      <c r="E21" t="n">
+        <v>29544.64</v>
+      </c>
+      <c r="F21" t="n">
+        <v>40</v>
+      </c>
+      <c r="G21" t="n">
+        <v>1620</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>normal speed</t>
+        </is>
+      </c>
+      <c r="J21" t="n">
+        <v>1.89</v>
+      </c>
+      <c r="K21" t="n">
+        <v>7</v>
+      </c>
+      <c r="L21" t="n">
+        <v>29487.5</v>
+      </c>
+      <c r="M21" t="n">
+        <v>29502.5</v>
+      </c>
+      <c r="N21" t="n">
+        <v>29517.5</v>
+      </c>
+      <c r="O21" t="n">
+        <v>60</v>
+      </c>
+      <c r="P21" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>29487.5</v>
+      </c>
+      <c r="R21" s="4" t="n">
+        <v>-60</v>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>SCALP_NORMAL</t>
+        </is>
+      </c>
+      <c r="U21" t="n">
+        <v>60</v>
+      </c>
+      <c r="V21" t="n">
+        <v>10</v>
+      </c>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-aplus-structure-export</t>
+        </is>
+      </c>
+      <c r="X21" t="inlineStr">
+        <is>
+          <t>09:31:00</t>
+        </is>
+      </c>
+      <c r="Y21" t="n">
+        <v>2311</v>
+      </c>
+      <c r="Z21" t="n">
+        <v>21.22</v>
+      </c>
+      <c r="AA21" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AB21" t="inlineStr">
+        <is>
+          <t>A+ structure</t>
+        </is>
+      </c>
+      <c r="AC21" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD21" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE21" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF21" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AG21" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH21" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AI21" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ21" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="AK21" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AL21" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="AM21" t="n">
+        <v>29501.25</v>
+      </c>
+      <c r="AN21" t="n">
+        <v>3</v>
+      </c>
+      <c r="AO21" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="R22" s="4" t="n"/>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>29241.25</v>
+      </c>
+      <c r="C22" t="n">
+        <v>29291.25</v>
+      </c>
+      <c r="D22" t="n">
+        <v>200</v>
+      </c>
+      <c r="E22" t="n">
+        <v>29294.78</v>
+      </c>
+      <c r="F22" t="n">
+        <v>90</v>
+      </c>
+      <c r="G22" t="n">
+        <v>828</v>
+      </c>
+      <c r="H22" t="n">
+        <v>-354</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>A+ speed</t>
+        </is>
+      </c>
+      <c r="J22" t="n">
+        <v>17.36</v>
+      </c>
+      <c r="K22" t="n">
+        <v>9</v>
+      </c>
+      <c r="L22" t="n">
+        <v>29233.75</v>
+      </c>
+      <c r="M22" t="n">
+        <v>29218.75</v>
+      </c>
+      <c r="N22" t="n">
+        <v>29203.75</v>
+      </c>
+      <c r="O22" t="n">
+        <v>60</v>
+      </c>
+      <c r="P22" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>29203.75</v>
+      </c>
+      <c r="R22" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>POTENTIAL_RUNNER</t>
+        </is>
+      </c>
+      <c r="U22" t="n">
+        <v>25</v>
+      </c>
+      <c r="V22" t="n">
+        <v>60</v>
+      </c>
+      <c r="W22" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-aplus-structure-export</t>
+        </is>
+      </c>
+      <c r="X22" t="inlineStr">
+        <is>
+          <t>09:31:00</t>
+        </is>
+      </c>
+      <c r="Y22" t="n">
+        <v>2311</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>5.1835</v>
+      </c>
+      <c r="AA22" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AB22" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AC22" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD22" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE22" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF22" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG22" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH22" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI22" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ22" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="AK22" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AN22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO22" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="R23" s="4" t="n"/>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>29305</v>
+      </c>
+      <c r="C23" t="n">
+        <v>29356.25</v>
+      </c>
+      <c r="D23" t="n">
+        <v>205</v>
+      </c>
+      <c r="E23" t="n">
+        <v>29211.89</v>
+      </c>
+      <c r="F23" t="n">
+        <v>50</v>
+      </c>
+      <c r="G23" t="n">
+        <v>802</v>
+      </c>
+      <c r="H23" t="n">
+        <v>-158</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>normal speed</t>
+        </is>
+      </c>
+      <c r="J23" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="K23" t="n">
+        <v>6</v>
+      </c>
+      <c r="L23" t="n">
+        <v>29298.75</v>
+      </c>
+      <c r="M23" t="n">
+        <v>29283.75</v>
+      </c>
+      <c r="N23" t="n">
+        <v>29268.75</v>
+      </c>
+      <c r="O23" t="n">
+        <v>60</v>
+      </c>
+      <c r="P23" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>29298.75</v>
+      </c>
+      <c r="R23" s="4" t="n">
+        <v>-60</v>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>SCALP_NORMAL</t>
+        </is>
+      </c>
+      <c r="U23" t="n">
+        <v>60</v>
+      </c>
+      <c r="V23" t="n">
+        <v>5</v>
+      </c>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-aplus-structure-export</t>
+        </is>
+      </c>
+      <c r="X23" t="inlineStr">
+        <is>
+          <t>09:33:00</t>
+        </is>
+      </c>
+      <c r="Y23" t="n">
+        <v>2313</v>
+      </c>
+      <c r="Z23" t="n">
+        <v>12.8979</v>
+      </c>
+      <c r="AA23" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AB23" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AC23" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD23" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE23" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF23" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG23" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH23" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AI23" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ23" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="AK23" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AN23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO23" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="R24" s="4" t="n"/>
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>28851.25</v>
+      </c>
+      <c r="C24" t="n">
+        <v>28943.75</v>
+      </c>
+      <c r="D24" t="n">
+        <v>370</v>
+      </c>
+      <c r="E24" t="n">
+        <v>28925.15</v>
+      </c>
+      <c r="F24" t="n">
+        <v>40</v>
+      </c>
+      <c r="G24" t="n">
+        <v>848</v>
+      </c>
+      <c r="H24" t="n">
+        <v>126</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>normal speed</t>
+        </is>
+      </c>
+      <c r="J24" t="n">
+        <v>2.66</v>
+      </c>
+      <c r="K24" t="n">
+        <v>7</v>
+      </c>
+      <c r="L24" t="n">
+        <v>28938.75</v>
+      </c>
+      <c r="M24" t="n">
+        <v>28953.75</v>
+      </c>
+      <c r="N24" t="n">
+        <v>28968.75</v>
+      </c>
+      <c r="O24" t="n">
+        <v>60</v>
+      </c>
+      <c r="P24" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>28968.75</v>
+      </c>
+      <c r="R24" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>SCALP_NORMAL</t>
+        </is>
+      </c>
+      <c r="U24" t="n">
+        <v>0</v>
+      </c>
+      <c r="V24" t="n">
+        <v>65</v>
+      </c>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-aplus-structure-export</t>
+        </is>
+      </c>
+      <c r="X24" t="inlineStr">
+        <is>
+          <t>09:32:00</t>
+        </is>
+      </c>
+      <c r="Y24" t="n">
+        <v>2312</v>
+      </c>
+      <c r="Z24" t="n">
+        <v>15.0195</v>
+      </c>
+      <c r="AA24" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AB24" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AC24" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AD24" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE24" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF24" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG24" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH24" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI24" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ24" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="AK24" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AN24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO24" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
     </row>
     <row r="25">
-      <c r="R25" s="4" t="n"/>
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>29070</v>
+      </c>
+      <c r="C25" t="n">
+        <v>29122.5</v>
+      </c>
+      <c r="D25" t="n">
+        <v>210</v>
+      </c>
+      <c r="E25" t="n">
+        <v>29074.59</v>
+      </c>
+      <c r="F25" t="n">
+        <v>25</v>
+      </c>
+      <c r="G25" t="n">
+        <v>1130</v>
+      </c>
+      <c r="H25" t="n">
+        <v>184</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>normal speed</t>
+        </is>
+      </c>
+      <c r="J25" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="K25" t="n">
+        <v>8</v>
+      </c>
+      <c r="L25" t="n">
+        <v>29113.75</v>
+      </c>
+      <c r="M25" t="n">
+        <v>29128.75</v>
+      </c>
+      <c r="N25" t="n">
+        <v>29143.75</v>
+      </c>
+      <c r="O25" t="n">
+        <v>60</v>
+      </c>
+      <c r="P25" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>29113.75</v>
+      </c>
+      <c r="R25" s="4" t="n">
+        <v>-60</v>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>SCALP_NORMAL</t>
+        </is>
+      </c>
+      <c r="U25" t="n">
+        <v>60</v>
+      </c>
+      <c r="V25" t="n">
+        <v>30</v>
+      </c>
+      <c r="W25" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-aplus-structure-export</t>
+        </is>
+      </c>
+      <c r="X25" t="inlineStr">
+        <is>
+          <t>09:31:00</t>
+        </is>
+      </c>
+      <c r="Y25" t="n">
+        <v>2311</v>
+      </c>
+      <c r="Z25" t="n">
+        <v>8.0563</v>
+      </c>
+      <c r="AA25" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AB25" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AC25" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD25" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE25" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF25" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG25" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH25" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI25" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ25" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="AK25" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AN25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO25" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
falta corregir las absorciones el side trade de las absorciones, normal speed ya requiere 3 imbalances para activarse pero falta debug
</commit_message>
<xml_diff>
--- a/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
+++ b/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AO25"/>
+  <dimension ref="A1:AX25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -677,6 +677,51 @@
           <t>Speed_Ignored_By_Structure</t>
         </is>
       </c>
+      <c r="AP3" s="3" t="inlineStr">
+        <is>
+          <t>Previous_Volume</t>
+        </is>
+      </c>
+      <c r="AQ3" s="3" t="inlineStr">
+        <is>
+          <t>Previous_Delta</t>
+        </is>
+      </c>
+      <c r="AR3" s="3" t="inlineStr">
+        <is>
+          <t>Volume_Increasing</t>
+        </is>
+      </c>
+      <c r="AS3" s="3" t="inlineStr">
+        <is>
+          <t>Delta_Change</t>
+        </is>
+      </c>
+      <c r="AT3" s="3" t="inlineStr">
+        <is>
+          <t>Delta_With_Side</t>
+        </is>
+      </c>
+      <c r="AU3" s="3" t="inlineStr">
+        <is>
+          <t>Price_Accepted_After_Imbalance</t>
+        </is>
+      </c>
+      <c r="AV3" s="3" t="inlineStr">
+        <is>
+          <t>Signal_Source</t>
+        </is>
+      </c>
+      <c r="AW3" s="3" t="inlineStr">
+        <is>
+          <t>APlus_Absorption</t>
+        </is>
+      </c>
+      <c r="AX3" s="3" t="inlineStr">
+        <is>
+          <t>APlus_Speed</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -694,16 +739,16 @@
         <v>220</v>
       </c>
       <c r="E4" t="n">
-        <v>26834.78</v>
+        <v>26834.83</v>
       </c>
       <c r="F4" t="n">
         <v>60</v>
       </c>
       <c r="G4" t="n">
-        <v>2171</v>
+        <v>2118</v>
       </c>
       <c r="H4" t="n">
-        <v>-541</v>
+        <v>-548</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -711,7 +756,7 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>2.01</v>
+        <v>2.05</v>
       </c>
       <c r="K4" t="n">
         <v>8</v>
@@ -751,7 +796,7 @@
         <v>25</v>
       </c>
       <c r="V4" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="W4" t="inlineStr">
         <is>
@@ -767,7 +812,7 @@
         <v>2310</v>
       </c>
       <c r="Z4" t="n">
-        <v>29.832</v>
+        <v>29.2665</v>
       </c>
       <c r="AA4" t="inlineStr">
         <is>
@@ -828,6 +873,45 @@
         <v>0</v>
       </c>
       <c r="AO4" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AP4" t="n">
+        <v>5767</v>
+      </c>
+      <c r="AQ4" t="n">
+        <v>-1001</v>
+      </c>
+      <c r="AR4" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AS4" t="n">
+        <v>453</v>
+      </c>
+      <c r="AT4" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AU4" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AV4" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="AW4" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
@@ -849,16 +933,16 @@
         <v>165</v>
       </c>
       <c r="E5" t="n">
-        <v>26842.08</v>
+        <v>26842.09</v>
       </c>
       <c r="F5" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="G5" t="n">
-        <v>1177</v>
+        <v>1168</v>
       </c>
       <c r="H5" t="n">
-        <v>-233</v>
+        <v>-230</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -866,19 +950,19 @@
         </is>
       </c>
       <c r="J5" t="n">
-        <v>0.28</v>
+        <v>0.14</v>
       </c>
       <c r="K5" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L5" t="n">
-        <v>26865</v>
+        <v>26866.25</v>
       </c>
       <c r="M5" t="n">
-        <v>26850</v>
+        <v>26851.25</v>
       </c>
       <c r="N5" t="n">
-        <v>26835</v>
+        <v>26836.25</v>
       </c>
       <c r="O5" t="n">
         <v>60</v>
@@ -887,7 +971,7 @@
         <v>60</v>
       </c>
       <c r="Q5" t="n">
-        <v>26835</v>
+        <v>26836.25</v>
       </c>
       <c r="R5" s="4" t="n">
         <v>60</v>
@@ -922,7 +1006,7 @@
         <v>2311</v>
       </c>
       <c r="Z5" t="n">
-        <v>36.081</v>
+        <v>35.6594</v>
       </c>
       <c r="AA5" t="inlineStr">
         <is>
@@ -931,7 +1015,7 @@
       </c>
       <c r="AB5" t="inlineStr">
         <is>
-          <t>A+ structure</t>
+          <t>A+ ABSORTION</t>
         </is>
       </c>
       <c r="AC5" t="inlineStr">
@@ -941,7 +1025,7 @@
       </c>
       <c r="AD5" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="AE5" t="inlineStr">
@@ -993,6 +1077,45 @@
       <c r="AO5" t="inlineStr">
         <is>
           <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AP5" t="n">
+        <v>2019</v>
+      </c>
+      <c r="AQ5" t="n">
+        <v>17</v>
+      </c>
+      <c r="AR5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AS5" t="n">
+        <v>-247</v>
+      </c>
+      <c r="AT5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AU5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AV5" t="inlineStr">
+        <is>
+          <t>A+ ABSORTION</t>
+        </is>
+      </c>
+      <c r="AW5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -1094,7 +1217,7 @@
       </c>
       <c r="AB6" t="inlineStr">
         <is>
-          <t>A+ structure</t>
+          <t>A+ ABSORTION</t>
         </is>
       </c>
       <c r="AC6" t="inlineStr">
@@ -1156,6 +1279,45 @@
       <c r="AO6" t="inlineStr">
         <is>
           <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AP6" t="n">
+        <v>1280</v>
+      </c>
+      <c r="AQ6" t="n">
+        <v>-20</v>
+      </c>
+      <c r="AR6" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AS6" t="n">
+        <v>222</v>
+      </c>
+      <c r="AT6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AU6" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AV6" t="inlineStr">
+        <is>
+          <t>A+ ABSORTION</t>
+        </is>
+      </c>
+      <c r="AW6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -1175,16 +1337,16 @@
         <v>190</v>
       </c>
       <c r="E7" t="n">
-        <v>27208.53</v>
+        <v>27208.67</v>
       </c>
       <c r="F7" t="n">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="G7" t="n">
-        <v>803</v>
+        <v>1323</v>
       </c>
       <c r="H7" t="n">
-        <v>109</v>
+        <v>189</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -1192,19 +1354,19 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>2.01</v>
+        <v>2.02</v>
       </c>
       <c r="K7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L7" t="n">
-        <v>27222.5</v>
+        <v>27228.75</v>
       </c>
       <c r="M7" t="n">
-        <v>27237.5</v>
+        <v>27243.75</v>
       </c>
       <c r="N7" t="n">
-        <v>27252.5</v>
+        <v>27258.75</v>
       </c>
       <c r="O7" t="n">
         <v>60</v>
@@ -1213,7 +1375,7 @@
         <v>60</v>
       </c>
       <c r="Q7" t="n">
-        <v>27222.5</v>
+        <v>27228.75</v>
       </c>
       <c r="R7" s="4" t="n">
         <v>-60</v>
@@ -1232,7 +1394,7 @@
         <v>60</v>
       </c>
       <c r="V7" t="n">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="W7" t="inlineStr">
         <is>
@@ -1248,7 +1410,7 @@
         <v>2314</v>
       </c>
       <c r="Z7" t="n">
-        <v>24.9169</v>
+        <v>37.1674</v>
       </c>
       <c r="AA7" t="inlineStr">
         <is>
@@ -1309,6 +1471,45 @@
         <v>0</v>
       </c>
       <c r="AO7" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AP7" t="n">
+        <v>1678</v>
+      </c>
+      <c r="AQ7" t="n">
+        <v>136</v>
+      </c>
+      <c r="AR7" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AS7" t="n">
+        <v>53</v>
+      </c>
+      <c r="AT7" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AU7" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AV7" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="AW7" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AX7" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
@@ -1342,16 +1543,16 @@
         <v>320</v>
       </c>
       <c r="E9" t="n">
-        <v>27189.24</v>
+        <v>27189.23</v>
       </c>
       <c r="F9" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G9" t="n">
-        <v>1528</v>
+        <v>1544</v>
       </c>
       <c r="H9" t="n">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -1359,19 +1560,19 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="K9" t="n">
         <v>8</v>
       </c>
       <c r="L9" t="n">
-        <v>27162.5</v>
+        <v>27161.25</v>
       </c>
       <c r="M9" t="n">
-        <v>27177.5</v>
+        <v>27176.25</v>
       </c>
       <c r="N9" t="n">
-        <v>27192.5</v>
+        <v>27191.25</v>
       </c>
       <c r="O9" t="n">
         <v>60</v>
@@ -1412,7 +1613,7 @@
         <v>2317</v>
       </c>
       <c r="Z9" t="n">
-        <v>49.6574</v>
+        <v>50.074</v>
       </c>
       <c r="AA9" t="inlineStr">
         <is>
@@ -1421,7 +1622,7 @@
       </c>
       <c r="AB9" t="inlineStr">
         <is>
-          <t>A+ structure</t>
+          <t>A+ ABSORTION</t>
         </is>
       </c>
       <c r="AC9" t="inlineStr">
@@ -1483,6 +1684,45 @@
       <c r="AO9" t="inlineStr">
         <is>
           <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AP9" t="n">
+        <v>2441</v>
+      </c>
+      <c r="AQ9" t="n">
+        <v>-209</v>
+      </c>
+      <c r="AR9" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AS9" t="n">
+        <v>263</v>
+      </c>
+      <c r="AT9" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AU9" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AV9" t="inlineStr">
+        <is>
+          <t>A+ ABSORTION</t>
+        </is>
+      </c>
+      <c r="AW9" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AX9" t="inlineStr">
+        <is>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -1502,36 +1742,36 @@
         <v>270</v>
       </c>
       <c r="E10" t="n">
-        <v>27241.75</v>
+        <v>27241.62</v>
       </c>
       <c r="F10" t="n">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="G10" t="n">
-        <v>805</v>
+        <v>885</v>
       </c>
       <c r="H10" t="n">
-        <v>-89</v>
+        <v>-103</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>normal speed</t>
+          <t>A+ speed</t>
         </is>
       </c>
       <c r="J10" t="n">
-        <v>2.33</v>
+        <v>5.43</v>
       </c>
       <c r="K10" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="L10" t="n">
-        <v>27162.5</v>
+        <v>27156.25</v>
       </c>
       <c r="M10" t="n">
-        <v>27147.5</v>
+        <v>27141.25</v>
       </c>
       <c r="N10" t="n">
-        <v>27132.5</v>
+        <v>27126.25</v>
       </c>
       <c r="O10" t="n">
         <v>60</v>
@@ -1540,7 +1780,7 @@
         <v>60</v>
       </c>
       <c r="Q10" t="n">
-        <v>27162.5</v>
+        <v>27156.25</v>
       </c>
       <c r="R10" s="4" t="n">
         <v>-60</v>
@@ -1552,14 +1792,14 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>SCALP_NORMAL</t>
+          <t>POTENTIAL_RUNNER</t>
         </is>
       </c>
       <c r="U10" t="n">
         <v>60</v>
       </c>
       <c r="V10" t="n">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="W10" t="inlineStr">
         <is>
@@ -1575,7 +1815,7 @@
         <v>2311</v>
       </c>
       <c r="Z10" t="n">
-        <v>6.4496</v>
+        <v>7.3705</v>
       </c>
       <c r="AA10" t="inlineStr">
         <is>
@@ -1636,6 +1876,45 @@
         <v>0</v>
       </c>
       <c r="AO10" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AP10" t="n">
+        <v>5790</v>
+      </c>
+      <c r="AQ10" t="n">
+        <v>-614</v>
+      </c>
+      <c r="AR10" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AS10" t="n">
+        <v>511</v>
+      </c>
+      <c r="AT10" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AU10" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AV10" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="AW10" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AX10" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
@@ -1657,16 +1936,16 @@
         <v>280</v>
       </c>
       <c r="E11" t="n">
-        <v>27385.42</v>
+        <v>27386.14</v>
       </c>
       <c r="F11" t="n">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="G11" t="n">
-        <v>984</v>
+        <v>1973</v>
       </c>
       <c r="H11" t="n">
-        <v>-110</v>
+        <v>-251</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -1674,19 +1953,19 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>2.55</v>
+        <v>2.37</v>
       </c>
       <c r="K11" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L11" t="n">
-        <v>27430</v>
+        <v>27393.75</v>
       </c>
       <c r="M11" t="n">
-        <v>27415</v>
+        <v>27378.75</v>
       </c>
       <c r="N11" t="n">
-        <v>27400</v>
+        <v>27363.75</v>
       </c>
       <c r="O11" t="n">
         <v>60</v>
@@ -1695,7 +1974,7 @@
         <v>60</v>
       </c>
       <c r="Q11" t="n">
-        <v>27400</v>
+        <v>27363.75</v>
       </c>
       <c r="R11" s="4" t="n">
         <v>60</v>
@@ -1711,7 +1990,7 @@
         </is>
       </c>
       <c r="U11" t="n">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="V11" t="n">
         <v>60</v>
@@ -1723,14 +2002,14 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>09:31:00</t>
+          <t>09:33:00</t>
         </is>
       </c>
       <c r="Y11" t="n">
-        <v>2311</v>
+        <v>2313</v>
       </c>
       <c r="Z11" t="n">
-        <v>11.7789</v>
+        <v>38.0436</v>
       </c>
       <c r="AA11" t="inlineStr">
         <is>
@@ -1769,7 +2048,7 @@
       </c>
       <c r="AH11" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="AI11" t="inlineStr">
@@ -1791,6 +2070,45 @@
         <v>0</v>
       </c>
       <c r="AO11" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AP11" t="n">
+        <v>2815</v>
+      </c>
+      <c r="AQ11" t="n">
+        <v>67</v>
+      </c>
+      <c r="AR11" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AS11" t="n">
+        <v>-318</v>
+      </c>
+      <c r="AT11" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AU11" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AV11" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="AW11" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AX11" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
@@ -1812,36 +2130,36 @@
         <v>190</v>
       </c>
       <c r="E12" t="n">
-        <v>27598.31</v>
+        <v>27598.68</v>
       </c>
       <c r="F12" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="G12" t="n">
-        <v>854</v>
+        <v>1107</v>
       </c>
       <c r="H12" t="n">
-        <v>254</v>
+        <v>363</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>normal speed</t>
+          <t>A+ speed</t>
         </is>
       </c>
       <c r="J12" t="n">
-        <v>2.59</v>
+        <v>5.29</v>
       </c>
       <c r="K12" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="L12" t="n">
-        <v>27656.25</v>
+        <v>27663.75</v>
       </c>
       <c r="M12" t="n">
-        <v>27671.25</v>
+        <v>27678.75</v>
       </c>
       <c r="N12" t="n">
-        <v>27686.25</v>
+        <v>27693.75</v>
       </c>
       <c r="O12" t="n">
         <v>60</v>
@@ -1850,7 +2168,7 @@
         <v>60</v>
       </c>
       <c r="Q12" t="n">
-        <v>27686.25</v>
+        <v>27693.75</v>
       </c>
       <c r="R12" s="4" t="n">
         <v>60</v>
@@ -1862,11 +2180,11 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>SCALP_NORMAL</t>
+          <t>POTENTIAL_RUNNER</t>
         </is>
       </c>
       <c r="U12" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="V12" t="n">
         <v>60</v>
@@ -1885,7 +2203,7 @@
         <v>2311</v>
       </c>
       <c r="Z12" t="n">
-        <v>7.7202</v>
+        <v>9.459099999999999</v>
       </c>
       <c r="AA12" t="inlineStr">
         <is>
@@ -1946,6 +2264,45 @@
         <v>0</v>
       </c>
       <c r="AO12" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AP12" t="n">
+        <v>5714</v>
+      </c>
+      <c r="AQ12" t="n">
+        <v>256</v>
+      </c>
+      <c r="AR12" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AS12" t="n">
+        <v>107</v>
+      </c>
+      <c r="AT12" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AU12" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AV12" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="AW12" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AX12" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
@@ -1967,16 +2324,16 @@
         <v>150</v>
       </c>
       <c r="E13" t="n">
-        <v>27837.02</v>
+        <v>27836.93</v>
       </c>
       <c r="F13" t="n">
-        <v>40</v>
+        <v>75</v>
       </c>
       <c r="G13" t="n">
-        <v>1284</v>
+        <v>1732</v>
       </c>
       <c r="H13" t="n">
-        <v>10</v>
+        <v>-130</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -1984,19 +2341,19 @@
         </is>
       </c>
       <c r="J13" t="n">
-        <v>2.26</v>
+        <v>3.37</v>
       </c>
       <c r="K13" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L13" t="n">
-        <v>27842.5</v>
+        <v>27833.75</v>
       </c>
       <c r="M13" t="n">
-        <v>27827.5</v>
+        <v>27818.75</v>
       </c>
       <c r="N13" t="n">
-        <v>27812.5</v>
+        <v>27803.75</v>
       </c>
       <c r="O13" t="n">
         <v>60</v>
@@ -2005,10 +2362,10 @@
         <v>60</v>
       </c>
       <c r="Q13" t="n">
-        <v>27812.5</v>
+        <v>27833.75</v>
       </c>
       <c r="R13" s="4" t="n">
-        <v>60</v>
+        <v>-60</v>
       </c>
       <c r="S13" t="inlineStr">
         <is>
@@ -2021,10 +2378,10 @@
         </is>
       </c>
       <c r="U13" t="n">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="V13" t="n">
-        <v>60</v>
+        <v>35</v>
       </c>
       <c r="W13" t="inlineStr">
         <is>
@@ -2040,7 +2397,7 @@
         <v>2311</v>
       </c>
       <c r="Z13" t="n">
-        <v>17.7163</v>
+        <v>22.2559</v>
       </c>
       <c r="AA13" t="inlineStr">
         <is>
@@ -2069,7 +2426,7 @@
       </c>
       <c r="AF13" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="AG13" t="inlineStr">
@@ -2089,7 +2446,7 @@
       </c>
       <c r="AJ13" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>SL</t>
         </is>
       </c>
       <c r="AK13" t="inlineStr">
@@ -2101,6 +2458,45 @@
         <v>0</v>
       </c>
       <c r="AO13" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AP13" t="n">
+        <v>6092</v>
+      </c>
+      <c r="AQ13" t="n">
+        <v>120</v>
+      </c>
+      <c r="AR13" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AS13" t="n">
+        <v>-250</v>
+      </c>
+      <c r="AT13" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AU13" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AV13" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="AW13" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AX13" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
@@ -2260,6 +2656,45 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="AP14" t="n">
+        <v>5972</v>
+      </c>
+      <c r="AQ14" t="n">
+        <v>170</v>
+      </c>
+      <c r="AR14" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AS14" t="n">
+        <v>-306</v>
+      </c>
+      <c r="AT14" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AU14" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AV14" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="AW14" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AX14" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2277,16 +2712,16 @@
         <v>225</v>
       </c>
       <c r="E15" t="n">
-        <v>28455.83</v>
+        <v>28455.06</v>
       </c>
       <c r="F15" t="n">
-        <v>25</v>
+        <v>95</v>
       </c>
       <c r="G15" t="n">
-        <v>835</v>
+        <v>1845</v>
       </c>
       <c r="H15" t="n">
-        <v>27</v>
+        <v>163</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -2294,19 +2729,19 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>2.13</v>
+        <v>2.35</v>
       </c>
       <c r="K15" t="n">
         <v>6</v>
       </c>
       <c r="L15" t="n">
-        <v>28411.25</v>
+        <v>28420</v>
       </c>
       <c r="M15" t="n">
-        <v>28426.25</v>
+        <v>28435</v>
       </c>
       <c r="N15" t="n">
-        <v>28441.25</v>
+        <v>28450</v>
       </c>
       <c r="O15" t="n">
         <v>60</v>
@@ -2315,10 +2750,10 @@
         <v>60</v>
       </c>
       <c r="Q15" t="n">
-        <v>28411.25</v>
+        <v>28450</v>
       </c>
       <c r="R15" s="4" t="n">
-        <v>-60</v>
+        <v>60</v>
       </c>
       <c r="S15" t="inlineStr">
         <is>
@@ -2331,10 +2766,10 @@
         </is>
       </c>
       <c r="U15" t="n">
-        <v>60</v>
+        <v>5</v>
       </c>
       <c r="V15" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="W15" t="inlineStr">
         <is>
@@ -2343,14 +2778,14 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>09:33:00</t>
+          <t>09:34:00</t>
         </is>
       </c>
       <c r="Y15" t="n">
-        <v>2313</v>
+        <v>2314</v>
       </c>
       <c r="Z15" t="n">
-        <v>11.7309</v>
+        <v>40.4043</v>
       </c>
       <c r="AA15" t="inlineStr">
         <is>
@@ -2399,7 +2834,7 @@
       </c>
       <c r="AJ15" t="inlineStr">
         <is>
-          <t>SL</t>
+          <t>TP</t>
         </is>
       </c>
       <c r="AK15" t="inlineStr">
@@ -2411,6 +2846,45 @@
         <v>0</v>
       </c>
       <c r="AO15" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AP15" t="n">
+        <v>2487</v>
+      </c>
+      <c r="AQ15" t="n">
+        <v>-35</v>
+      </c>
+      <c r="AR15" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AS15" t="n">
+        <v>198</v>
+      </c>
+      <c r="AT15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AU15" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AV15" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="AW15" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AX15" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
@@ -2438,10 +2912,10 @@
         <v>40</v>
       </c>
       <c r="G16" t="n">
-        <v>1441</v>
+        <v>1442</v>
       </c>
       <c r="H16" t="n">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -2505,7 +2979,7 @@
         <v>2318</v>
       </c>
       <c r="Z16" t="n">
-        <v>57.6084</v>
+        <v>57.7433</v>
       </c>
       <c r="AA16" t="inlineStr">
         <is>
@@ -2514,7 +2988,7 @@
       </c>
       <c r="AB16" t="inlineStr">
         <is>
-          <t>A+ structure</t>
+          <t>A+ ABSORTION</t>
         </is>
       </c>
       <c r="AC16" t="inlineStr">
@@ -2576,6 +3050,45 @@
       <c r="AO16" t="inlineStr">
         <is>
           <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AP16" t="n">
+        <v>1647</v>
+      </c>
+      <c r="AQ16" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AR16" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AS16" t="n">
+        <v>243</v>
+      </c>
+      <c r="AT16" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AU16" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AV16" t="inlineStr">
+        <is>
+          <t>A+ ABSORTION</t>
+        </is>
+      </c>
+      <c r="AW16" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AX16" t="inlineStr">
+        <is>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -2595,16 +3108,16 @@
         <v>175</v>
       </c>
       <c r="E17" t="n">
-        <v>28876.6</v>
+        <v>28876.65</v>
       </c>
       <c r="F17" t="n">
         <v>50</v>
       </c>
       <c r="G17" t="n">
-        <v>1573</v>
+        <v>1703</v>
       </c>
       <c r="H17" t="n">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -2612,7 +3125,7 @@
         </is>
       </c>
       <c r="J17" t="n">
-        <v>2.19</v>
+        <v>2.05</v>
       </c>
       <c r="K17" t="n">
         <v>8</v>
@@ -2668,7 +3181,7 @@
         <v>2311</v>
       </c>
       <c r="Z17" t="n">
-        <v>22.8326</v>
+        <v>24.4185</v>
       </c>
       <c r="AA17" t="inlineStr">
         <is>
@@ -2729,6 +3242,45 @@
         <v>0</v>
       </c>
       <c r="AO17" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AP17" t="n">
+        <v>4730</v>
+      </c>
+      <c r="AQ17" t="n">
+        <v>170</v>
+      </c>
+      <c r="AR17" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AS17" t="n">
+        <v>43</v>
+      </c>
+      <c r="AT17" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AU17" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AV17" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="AW17" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AX17" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
@@ -2756,10 +3308,10 @@
         <v>75</v>
       </c>
       <c r="G18" t="n">
-        <v>817</v>
+        <v>812</v>
       </c>
       <c r="H18" t="n">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -2767,7 +3319,7 @@
         </is>
       </c>
       <c r="J18" t="n">
-        <v>10.68</v>
+        <v>10.73</v>
       </c>
       <c r="K18" t="n">
         <v>9</v>
@@ -2823,7 +3375,7 @@
         <v>2311</v>
       </c>
       <c r="Z18" t="n">
-        <v>7.0252</v>
+        <v>6.9889</v>
       </c>
       <c r="AA18" t="inlineStr">
         <is>
@@ -2884,6 +3436,45 @@
         <v>0</v>
       </c>
       <c r="AO18" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AP18" t="n">
+        <v>6846</v>
+      </c>
+      <c r="AQ18" t="n">
+        <v>296</v>
+      </c>
+      <c r="AR18" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AS18" t="n">
+        <v>-162</v>
+      </c>
+      <c r="AT18" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AU18" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AV18" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="AW18" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AX18" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
@@ -2917,16 +3508,16 @@
         <v>145</v>
       </c>
       <c r="E20" t="n">
-        <v>29321.36</v>
+        <v>29321.15</v>
       </c>
       <c r="F20" t="n">
-        <v>35</v>
+        <v>65</v>
       </c>
       <c r="G20" t="n">
-        <v>1113</v>
+        <v>1341</v>
       </c>
       <c r="H20" t="n">
-        <v>-175</v>
+        <v>-263</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -2934,19 +3525,19 @@
         </is>
       </c>
       <c r="J20" t="n">
-        <v>2.08</v>
+        <v>3.49</v>
       </c>
       <c r="K20" t="n">
         <v>8</v>
       </c>
       <c r="L20" t="n">
-        <v>29258.75</v>
+        <v>29251.25</v>
       </c>
       <c r="M20" t="n">
-        <v>29243.75</v>
+        <v>29236.25</v>
       </c>
       <c r="N20" t="n">
-        <v>29228.75</v>
+        <v>29221.25</v>
       </c>
       <c r="O20" t="n">
         <v>60</v>
@@ -2955,7 +3546,7 @@
         <v>60</v>
       </c>
       <c r="Q20" t="n">
-        <v>29228.75</v>
+        <v>29221.25</v>
       </c>
       <c r="R20" s="4" t="n">
         <v>60</v>
@@ -2971,7 +3562,7 @@
         </is>
       </c>
       <c r="U20" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="V20" t="n">
         <v>60</v>
@@ -2990,7 +3581,7 @@
         <v>2311</v>
       </c>
       <c r="Z20" t="n">
-        <v>16.8109</v>
+        <v>18.6189</v>
       </c>
       <c r="AA20" t="inlineStr">
         <is>
@@ -3051,6 +3642,45 @@
         <v>0</v>
       </c>
       <c r="AO20" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AP20" t="n">
+        <v>6047</v>
+      </c>
+      <c r="AQ20" t="n">
+        <v>-401</v>
+      </c>
+      <c r="AR20" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AS20" t="n">
+        <v>138</v>
+      </c>
+      <c r="AT20" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AU20" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AV20" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="AW20" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AX20" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
@@ -3078,10 +3708,10 @@
         <v>40</v>
       </c>
       <c r="G21" t="n">
-        <v>1620</v>
+        <v>1618</v>
       </c>
       <c r="H21" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -3145,7 +3775,7 @@
         <v>2311</v>
       </c>
       <c r="Z21" t="n">
-        <v>21.22</v>
+        <v>21.1943</v>
       </c>
       <c r="AA21" t="inlineStr">
         <is>
@@ -3154,7 +3784,7 @@
       </c>
       <c r="AB21" t="inlineStr">
         <is>
-          <t>A+ structure</t>
+          <t>A+ ABSORTION</t>
         </is>
       </c>
       <c r="AC21" t="inlineStr">
@@ -3216,6 +3846,45 @@
       <c r="AO21" t="inlineStr">
         <is>
           <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AP21" t="n">
+        <v>5632</v>
+      </c>
+      <c r="AQ21" t="n">
+        <v>-148</v>
+      </c>
+      <c r="AR21" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AS21" t="n">
+        <v>146</v>
+      </c>
+      <c r="AT21" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AU21" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AV21" t="inlineStr">
+        <is>
+          <t>A+ ABSORTION</t>
+        </is>
+      </c>
+      <c r="AW21" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AX21" t="inlineStr">
+        <is>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -3238,13 +3907,13 @@
         <v>29294.78</v>
       </c>
       <c r="F22" t="n">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="G22" t="n">
-        <v>828</v>
+        <v>818</v>
       </c>
       <c r="H22" t="n">
-        <v>-354</v>
+        <v>-356</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -3252,19 +3921,19 @@
         </is>
       </c>
       <c r="J22" t="n">
-        <v>17.36</v>
+        <v>16.9</v>
       </c>
       <c r="K22" t="n">
         <v>9</v>
       </c>
       <c r="L22" t="n">
-        <v>29233.75</v>
+        <v>29235</v>
       </c>
       <c r="M22" t="n">
-        <v>29218.75</v>
+        <v>29220</v>
       </c>
       <c r="N22" t="n">
-        <v>29203.75</v>
+        <v>29205</v>
       </c>
       <c r="O22" t="n">
         <v>60</v>
@@ -3273,7 +3942,7 @@
         <v>60</v>
       </c>
       <c r="Q22" t="n">
-        <v>29203.75</v>
+        <v>29205</v>
       </c>
       <c r="R22" s="4" t="n">
         <v>60</v>
@@ -3289,7 +3958,7 @@
         </is>
       </c>
       <c r="U22" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="V22" t="n">
         <v>60</v>
@@ -3308,7 +3977,7 @@
         <v>2311</v>
       </c>
       <c r="Z22" t="n">
-        <v>5.1835</v>
+        <v>5.0304</v>
       </c>
       <c r="AA22" t="inlineStr">
         <is>
@@ -3369,6 +4038,45 @@
         <v>0</v>
       </c>
       <c r="AO22" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AP22" t="n">
+        <v>7150</v>
+      </c>
+      <c r="AQ22" t="n">
+        <v>136</v>
+      </c>
+      <c r="AR22" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AS22" t="n">
+        <v>-492</v>
+      </c>
+      <c r="AT22" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AU22" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AV22" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="AW22" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AX22" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
@@ -3396,10 +4104,10 @@
         <v>50</v>
       </c>
       <c r="G23" t="n">
-        <v>802</v>
+        <v>809</v>
       </c>
       <c r="H23" t="n">
-        <v>-158</v>
+        <v>-159</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -3407,7 +4115,7 @@
         </is>
       </c>
       <c r="J23" t="n">
-        <v>3.88</v>
+        <v>3.82</v>
       </c>
       <c r="K23" t="n">
         <v>6</v>
@@ -3463,7 +4171,7 @@
         <v>2313</v>
       </c>
       <c r="Z23" t="n">
-        <v>12.8979</v>
+        <v>13.1022</v>
       </c>
       <c r="AA23" t="inlineStr">
         <is>
@@ -3524,6 +4232,45 @@
         <v>0</v>
       </c>
       <c r="AO23" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AP23" t="n">
+        <v>3452</v>
+      </c>
+      <c r="AQ23" t="n">
+        <v>-98</v>
+      </c>
+      <c r="AR23" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AS23" t="n">
+        <v>-61</v>
+      </c>
+      <c r="AT23" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AU23" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AV23" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="AW23" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AX23" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
@@ -3545,36 +4292,36 @@
         <v>370</v>
       </c>
       <c r="E24" t="n">
-        <v>28925.15</v>
+        <v>28925.32</v>
       </c>
       <c r="F24" t="n">
-        <v>40</v>
+        <v>95</v>
       </c>
       <c r="G24" t="n">
-        <v>848</v>
+        <v>1254</v>
       </c>
       <c r="H24" t="n">
-        <v>126</v>
+        <v>280</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>normal speed</t>
+          <t>A+ speed</t>
         </is>
       </c>
       <c r="J24" t="n">
-        <v>2.66</v>
+        <v>6.1</v>
       </c>
       <c r="K24" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L24" t="n">
-        <v>28938.75</v>
+        <v>28952.5</v>
       </c>
       <c r="M24" t="n">
-        <v>28953.75</v>
+        <v>28967.5</v>
       </c>
       <c r="N24" t="n">
-        <v>28968.75</v>
+        <v>28982.5</v>
       </c>
       <c r="O24" t="n">
         <v>60</v>
@@ -3583,7 +4330,7 @@
         <v>60</v>
       </c>
       <c r="Q24" t="n">
-        <v>28968.75</v>
+        <v>28982.5</v>
       </c>
       <c r="R24" s="4" t="n">
         <v>60</v>
@@ -3595,14 +4342,14 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>SCALP_NORMAL</t>
+          <t>POTENTIAL_RUNNER</t>
         </is>
       </c>
       <c r="U24" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="V24" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="W24" t="inlineStr">
         <is>
@@ -3618,7 +4365,7 @@
         <v>2312</v>
       </c>
       <c r="Z24" t="n">
-        <v>15.0195</v>
+        <v>15.5645</v>
       </c>
       <c r="AA24" t="inlineStr">
         <is>
@@ -3679,6 +4426,45 @@
         <v>0</v>
       </c>
       <c r="AO24" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AP24" t="n">
+        <v>4358</v>
+      </c>
+      <c r="AQ24" t="n">
+        <v>-32</v>
+      </c>
+      <c r="AR24" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AS24" t="n">
+        <v>312</v>
+      </c>
+      <c r="AT24" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AU24" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AV24" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="AW24" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AX24" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
@@ -3700,16 +4486,16 @@
         <v>210</v>
       </c>
       <c r="E25" t="n">
-        <v>29074.59</v>
+        <v>29074.6</v>
       </c>
       <c r="F25" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="G25" t="n">
-        <v>1130</v>
+        <v>1158</v>
       </c>
       <c r="H25" t="n">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
@@ -3717,19 +4503,19 @@
         </is>
       </c>
       <c r="J25" t="n">
-        <v>3.1</v>
+        <v>2.4</v>
       </c>
       <c r="K25" t="n">
         <v>8</v>
       </c>
       <c r="L25" t="n">
-        <v>29113.75</v>
+        <v>29112.5</v>
       </c>
       <c r="M25" t="n">
-        <v>29128.75</v>
+        <v>29127.5</v>
       </c>
       <c r="N25" t="n">
-        <v>29143.75</v>
+        <v>29142.5</v>
       </c>
       <c r="O25" t="n">
         <v>60</v>
@@ -3738,7 +4524,7 @@
         <v>60</v>
       </c>
       <c r="Q25" t="n">
-        <v>29113.75</v>
+        <v>29112.5</v>
       </c>
       <c r="R25" s="4" t="n">
         <v>-60</v>
@@ -3757,7 +4543,7 @@
         <v>60</v>
       </c>
       <c r="V25" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="W25" t="inlineStr">
         <is>
@@ -3773,7 +4559,7 @@
         <v>2311</v>
       </c>
       <c r="Z25" t="n">
-        <v>8.0563</v>
+        <v>8.349399999999999</v>
       </c>
       <c r="AA25" t="inlineStr">
         <is>
@@ -3834,6 +4620,45 @@
         <v>0</v>
       </c>
       <c r="AO25" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AP25" t="n">
+        <v>5619</v>
+      </c>
+      <c r="AQ25" t="n">
+        <v>211</v>
+      </c>
+      <c r="AR25" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AS25" t="n">
+        <v>-15</v>
+      </c>
+      <c r="AT25" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AU25" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AV25" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="AW25" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AX25" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>

</xml_diff>

<commit_message>
LAS FECHAS NO CSV YA GENERAN EXCEL
</commit_message>
<xml_diff>
--- a/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
+++ b/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
@@ -739,16 +739,16 @@
         <v>220</v>
       </c>
       <c r="E4" t="n">
-        <v>26834.83</v>
+        <v>26835.37</v>
       </c>
       <c r="F4" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="G4" t="n">
-        <v>2118</v>
+        <v>1633</v>
       </c>
       <c r="H4" t="n">
-        <v>-548</v>
+        <v>-385</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -762,13 +762,13 @@
         <v>8</v>
       </c>
       <c r="L4" t="n">
-        <v>26772.5</v>
+        <v>26775</v>
       </c>
       <c r="M4" t="n">
-        <v>26757.5</v>
+        <v>26760</v>
       </c>
       <c r="N4" t="n">
-        <v>26742.5</v>
+        <v>26745</v>
       </c>
       <c r="O4" t="n">
         <v>60</v>
@@ -777,7 +777,7 @@
         <v>60</v>
       </c>
       <c r="Q4" t="n">
-        <v>26742.5</v>
+        <v>26745</v>
       </c>
       <c r="R4" s="4" t="n">
         <v>60</v>
@@ -793,7 +793,7 @@
         </is>
       </c>
       <c r="U4" t="n">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="V4" t="n">
         <v>60</v>
@@ -812,7 +812,7 @@
         <v>2310</v>
       </c>
       <c r="Z4" t="n">
-        <v>29.2665</v>
+        <v>24.3957</v>
       </c>
       <c r="AA4" t="inlineStr">
         <is>
@@ -889,7 +889,7 @@
         </is>
       </c>
       <c r="AS4" t="n">
-        <v>453</v>
+        <v>616</v>
       </c>
       <c r="AT4" t="inlineStr">
         <is>
@@ -933,16 +933,16 @@
         <v>165</v>
       </c>
       <c r="E5" t="n">
-        <v>26842.09</v>
+        <v>26842.08</v>
       </c>
       <c r="F5" t="n">
         <v>5</v>
       </c>
       <c r="G5" t="n">
-        <v>1168</v>
+        <v>1151</v>
       </c>
       <c r="H5" t="n">
-        <v>-230</v>
+        <v>-229</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -1006,7 +1006,7 @@
         <v>2311</v>
       </c>
       <c r="Z5" t="n">
-        <v>35.6594</v>
+        <v>35.3264</v>
       </c>
       <c r="AA5" t="inlineStr">
         <is>
@@ -1015,7 +1015,7 @@
       </c>
       <c r="AB5" t="inlineStr">
         <is>
-          <t>A+ ABSORTION</t>
+          <t>A+ STRUCTURE</t>
         </is>
       </c>
       <c r="AC5" t="inlineStr">
@@ -1091,7 +1091,7 @@
         </is>
       </c>
       <c r="AS5" t="n">
-        <v>-247</v>
+        <v>-246</v>
       </c>
       <c r="AT5" t="inlineStr">
         <is>
@@ -1105,12 +1105,12 @@
       </c>
       <c r="AV5" t="inlineStr">
         <is>
-          <t>A+ ABSORTION</t>
+          <t>A+ STRUCTURE</t>
         </is>
       </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
@@ -1337,16 +1337,16 @@
         <v>190</v>
       </c>
       <c r="E7" t="n">
-        <v>27208.67</v>
+        <v>27208.61</v>
       </c>
       <c r="F7" t="n">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="G7" t="n">
-        <v>1323</v>
+        <v>1128</v>
       </c>
       <c r="H7" t="n">
-        <v>189</v>
+        <v>158</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -1354,19 +1354,19 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>2.02</v>
+        <v>1.96</v>
       </c>
       <c r="K7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="L7" t="n">
-        <v>27228.75</v>
+        <v>27226.25</v>
       </c>
       <c r="M7" t="n">
-        <v>27243.75</v>
+        <v>27241.25</v>
       </c>
       <c r="N7" t="n">
-        <v>27258.75</v>
+        <v>27256.25</v>
       </c>
       <c r="O7" t="n">
         <v>60</v>
@@ -1375,7 +1375,7 @@
         <v>60</v>
       </c>
       <c r="Q7" t="n">
-        <v>27228.75</v>
+        <v>27226.25</v>
       </c>
       <c r="R7" s="4" t="n">
         <v>-60</v>
@@ -1391,10 +1391,10 @@
         </is>
       </c>
       <c r="U7" t="n">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="V7" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="W7" t="inlineStr">
         <is>
@@ -1410,7 +1410,7 @@
         <v>2314</v>
       </c>
       <c r="Z7" t="n">
-        <v>37.1674</v>
+        <v>33.0902</v>
       </c>
       <c r="AA7" t="inlineStr">
         <is>
@@ -1419,7 +1419,7 @@
       </c>
       <c r="AB7" t="inlineStr">
         <is>
-          <t>LastTime</t>
+          <t>A+ ABSORTION</t>
         </is>
       </c>
       <c r="AC7" t="inlineStr">
@@ -1464,15 +1464,23 @@
       </c>
       <c r="AK7" t="inlineStr">
         <is>
-          <t>FALSE</t>
-        </is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AL7" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="AM7" t="n">
+        <v>27241.25</v>
       </c>
       <c r="AN7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AO7" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="AP7" t="n">
@@ -1487,7 +1495,7 @@
         </is>
       </c>
       <c r="AS7" t="n">
-        <v>53</v>
+        <v>22</v>
       </c>
       <c r="AT7" t="inlineStr">
         <is>
@@ -1501,12 +1509,12 @@
       </c>
       <c r="AV7" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>A+ ABSORTION</t>
         </is>
       </c>
       <c r="AW7" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="AX7" t="inlineStr">
@@ -1521,9 +1529,199 @@
           <t>2026-04-27</t>
         </is>
       </c>
-      <c r="R8" s="4" t="inlineStr">
-        <is>
-          <t>NO_CSV</t>
+      <c r="B8" t="n">
+        <v>27363.75</v>
+      </c>
+      <c r="C8" t="n">
+        <v>27435</v>
+      </c>
+      <c r="D8" t="n">
+        <v>285</v>
+      </c>
+      <c r="E8" t="n">
+        <v>27430.74</v>
+      </c>
+      <c r="F8" t="n">
+        <v>30</v>
+      </c>
+      <c r="G8" t="n">
+        <v>873</v>
+      </c>
+      <c r="H8" t="n">
+        <v>-197</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>normal speed</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="K8" t="n">
+        <v>8</v>
+      </c>
+      <c r="L8" t="n">
+        <v>27371.25</v>
+      </c>
+      <c r="M8" t="n">
+        <v>27356.25</v>
+      </c>
+      <c r="N8" t="n">
+        <v>27341.25</v>
+      </c>
+      <c r="O8" t="n">
+        <v>60</v>
+      </c>
+      <c r="P8" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>27371.25</v>
+      </c>
+      <c r="R8" s="4" t="n">
+        <v>-60</v>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>SCALP_NORMAL</t>
+        </is>
+      </c>
+      <c r="U8" t="n">
+        <v>60</v>
+      </c>
+      <c r="V8" t="n">
+        <v>5</v>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-aplus-structure-export</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>09:36:00</t>
+        </is>
+      </c>
+      <c r="Y8" t="n">
+        <v>2316</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>17.4596</v>
+      </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>A+ STRUCTURE</t>
+        </is>
+      </c>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ8" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="AK8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AL8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="AM8" t="n">
+        <v>27362.5</v>
+      </c>
+      <c r="AN8" t="n">
+        <v>3</v>
+      </c>
+      <c r="AO8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AP8" t="n">
+        <v>2041</v>
+      </c>
+      <c r="AQ8" t="n">
+        <v>-123</v>
+      </c>
+      <c r="AR8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AS8" t="n">
+        <v>-74</v>
+      </c>
+      <c r="AT8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AU8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AV8" t="inlineStr">
+        <is>
+          <t>A+ STRUCTURE</t>
+        </is>
+      </c>
+      <c r="AW8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AX8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
@@ -1543,36 +1741,36 @@
         <v>320</v>
       </c>
       <c r="E9" t="n">
-        <v>27189.23</v>
+        <v>27194.37</v>
       </c>
       <c r="F9" t="n">
+        <v>20</v>
+      </c>
+      <c r="G9" t="n">
+        <v>3003</v>
+      </c>
+      <c r="H9" t="n">
+        <v>-83</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>normal speed</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="K9" t="n">
         <v>10</v>
       </c>
-      <c r="G9" t="n">
-        <v>1544</v>
-      </c>
-      <c r="H9" t="n">
-        <v>54</v>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>normal speed</t>
-        </is>
-      </c>
-      <c r="J9" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="K9" t="n">
-        <v>8</v>
-      </c>
       <c r="L9" t="n">
-        <v>27161.25</v>
+        <v>27092.5</v>
       </c>
       <c r="M9" t="n">
-        <v>27176.25</v>
+        <v>27077.5</v>
       </c>
       <c r="N9" t="n">
-        <v>27191.25</v>
+        <v>27062.5</v>
       </c>
       <c r="O9" t="n">
         <v>60</v>
@@ -1580,12 +1778,15 @@
       <c r="P9" t="n">
         <v>60</v>
       </c>
+      <c r="Q9" t="n">
+        <v>27092.5</v>
+      </c>
       <c r="R9" s="4" t="n">
-        <v>0</v>
+        <v>-60</v>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
@@ -1594,10 +1795,10 @@
         </is>
       </c>
       <c r="U9" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="V9" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="W9" t="inlineStr">
         <is>
@@ -1606,14 +1807,14 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>09:37:00</t>
+          <t>09:31:00</t>
         </is>
       </c>
       <c r="Y9" t="n">
-        <v>2317</v>
+        <v>2311</v>
       </c>
       <c r="Z9" t="n">
-        <v>50.074</v>
+        <v>36.3744</v>
       </c>
       <c r="AA9" t="inlineStr">
         <is>
@@ -1652,7 +1853,7 @@
       </c>
       <c r="AH9" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="AI9" t="inlineStr">
@@ -1662,7 +1863,7 @@
       </c>
       <c r="AJ9" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>SL</t>
         </is>
       </c>
       <c r="AK9" t="inlineStr">
@@ -1672,11 +1873,11 @@
       </c>
       <c r="AL9" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="AM9" t="n">
-        <v>27181.25</v>
+        <v>27080</v>
       </c>
       <c r="AN9" t="n">
         <v>3</v>
@@ -1687,10 +1888,10 @@
         </is>
       </c>
       <c r="AP9" t="n">
-        <v>2441</v>
+        <v>7642</v>
       </c>
       <c r="AQ9" t="n">
-        <v>-209</v>
+        <v>-672</v>
       </c>
       <c r="AR9" t="inlineStr">
         <is>
@@ -1698,16 +1899,16 @@
         </is>
       </c>
       <c r="AS9" t="n">
-        <v>263</v>
+        <v>589</v>
       </c>
       <c r="AT9" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="AU9" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="AV9" t="inlineStr">
@@ -1742,16 +1943,16 @@
         <v>270</v>
       </c>
       <c r="E10" t="n">
-        <v>27241.62</v>
+        <v>27241.68</v>
       </c>
       <c r="F10" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="G10" t="n">
-        <v>885</v>
+        <v>841</v>
       </c>
       <c r="H10" t="n">
-        <v>-103</v>
+        <v>-91</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -1759,19 +1960,19 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>5.43</v>
+        <v>5.03</v>
       </c>
       <c r="K10" t="n">
         <v>9</v>
       </c>
       <c r="L10" t="n">
-        <v>27156.25</v>
+        <v>27157.5</v>
       </c>
       <c r="M10" t="n">
-        <v>27141.25</v>
+        <v>27142.5</v>
       </c>
       <c r="N10" t="n">
-        <v>27126.25</v>
+        <v>27127.5</v>
       </c>
       <c r="O10" t="n">
         <v>60</v>
@@ -1780,7 +1981,7 @@
         <v>60</v>
       </c>
       <c r="Q10" t="n">
-        <v>27156.25</v>
+        <v>27157.5</v>
       </c>
       <c r="R10" s="4" t="n">
         <v>-60</v>
@@ -1799,7 +2000,7 @@
         <v>60</v>
       </c>
       <c r="V10" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="W10" t="inlineStr">
         <is>
@@ -1815,7 +2016,7 @@
         <v>2311</v>
       </c>
       <c r="Z10" t="n">
-        <v>7.3705</v>
+        <v>6.9635</v>
       </c>
       <c r="AA10" t="inlineStr">
         <is>
@@ -1869,11 +2070,19 @@
       </c>
       <c r="AK10" t="inlineStr">
         <is>
-          <t>FALSE</t>
-        </is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AL10" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="AM10" t="n">
+        <v>27150</v>
       </c>
       <c r="AN10" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AO10" t="inlineStr">
         <is>
@@ -1892,7 +2101,7 @@
         </is>
       </c>
       <c r="AS10" t="n">
-        <v>511</v>
+        <v>523</v>
       </c>
       <c r="AT10" t="inlineStr">
         <is>
@@ -1901,17 +2110,17 @@
       </c>
       <c r="AU10" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="AV10" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>A+ ABSORTION</t>
         </is>
       </c>
       <c r="AW10" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="AX10" t="inlineStr">
@@ -1936,16 +2145,16 @@
         <v>280</v>
       </c>
       <c r="E11" t="n">
-        <v>27386.14</v>
+        <v>27385.42</v>
       </c>
       <c r="F11" t="n">
-        <v>90</v>
+        <v>25</v>
       </c>
       <c r="G11" t="n">
-        <v>1973</v>
+        <v>970</v>
       </c>
       <c r="H11" t="n">
-        <v>-251</v>
+        <v>-110</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -1953,19 +2162,19 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>2.37</v>
+        <v>2.13</v>
       </c>
       <c r="K11" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L11" t="n">
-        <v>27393.75</v>
+        <v>27431.25</v>
       </c>
       <c r="M11" t="n">
-        <v>27378.75</v>
+        <v>27416.25</v>
       </c>
       <c r="N11" t="n">
-        <v>27363.75</v>
+        <v>27401.25</v>
       </c>
       <c r="O11" t="n">
         <v>60</v>
@@ -1974,7 +2183,7 @@
         <v>60</v>
       </c>
       <c r="Q11" t="n">
-        <v>27363.75</v>
+        <v>27401.25</v>
       </c>
       <c r="R11" s="4" t="n">
         <v>60</v>
@@ -1990,7 +2199,7 @@
         </is>
       </c>
       <c r="U11" t="n">
-        <v>15</v>
+        <v>45</v>
       </c>
       <c r="V11" t="n">
         <v>60</v>
@@ -2002,14 +2211,14 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>09:33:00</t>
+          <t>09:31:00</t>
         </is>
       </c>
       <c r="Y11" t="n">
-        <v>2313</v>
+        <v>2311</v>
       </c>
       <c r="Z11" t="n">
-        <v>38.0436</v>
+        <v>11.723</v>
       </c>
       <c r="AA11" t="inlineStr">
         <is>
@@ -2048,7 +2257,7 @@
       </c>
       <c r="AH11" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="AI11" t="inlineStr">
@@ -2075,10 +2284,10 @@
         </is>
       </c>
       <c r="AP11" t="n">
-        <v>2815</v>
+        <v>6340</v>
       </c>
       <c r="AQ11" t="n">
-        <v>67</v>
+        <v>-568</v>
       </c>
       <c r="AR11" t="inlineStr">
         <is>
@@ -2086,11 +2295,11 @@
         </is>
       </c>
       <c r="AS11" t="n">
-        <v>-318</v>
+        <v>458</v>
       </c>
       <c r="AT11" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="AU11" t="inlineStr">
@@ -2130,36 +2339,36 @@
         <v>190</v>
       </c>
       <c r="E12" t="n">
-        <v>27598.68</v>
+        <v>27598.27</v>
       </c>
       <c r="F12" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="G12" t="n">
-        <v>1107</v>
+        <v>807</v>
       </c>
       <c r="H12" t="n">
-        <v>363</v>
+        <v>239</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>A+ speed</t>
+          <t>normal speed</t>
         </is>
       </c>
       <c r="J12" t="n">
-        <v>5.29</v>
+        <v>3.3</v>
       </c>
       <c r="K12" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="L12" t="n">
-        <v>27663.75</v>
+        <v>27657.5</v>
       </c>
       <c r="M12" t="n">
-        <v>27678.75</v>
+        <v>27672.5</v>
       </c>
       <c r="N12" t="n">
-        <v>27693.75</v>
+        <v>27687.5</v>
       </c>
       <c r="O12" t="n">
         <v>60</v>
@@ -2168,7 +2377,7 @@
         <v>60</v>
       </c>
       <c r="Q12" t="n">
-        <v>27693.75</v>
+        <v>27687.5</v>
       </c>
       <c r="R12" s="4" t="n">
         <v>60</v>
@@ -2180,7 +2389,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>POTENTIAL_RUNNER</t>
+          <t>SCALP_NORMAL</t>
         </is>
       </c>
       <c r="U12" t="n">
@@ -2203,7 +2412,7 @@
         <v>2311</v>
       </c>
       <c r="Z12" t="n">
-        <v>9.459099999999999</v>
+        <v>7.575</v>
       </c>
       <c r="AA12" t="inlineStr">
         <is>
@@ -2280,11 +2489,11 @@
         </is>
       </c>
       <c r="AS12" t="n">
-        <v>107</v>
+        <v>-17</v>
       </c>
       <c r="AT12" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="AU12" t="inlineStr">
@@ -2324,16 +2533,16 @@
         <v>150</v>
       </c>
       <c r="E13" t="n">
-        <v>27836.93</v>
+        <v>27837.01</v>
       </c>
       <c r="F13" t="n">
-        <v>75</v>
+        <v>40</v>
       </c>
       <c r="G13" t="n">
-        <v>1732</v>
+        <v>1330</v>
       </c>
       <c r="H13" t="n">
-        <v>-130</v>
+        <v>-24</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -2341,19 +2550,19 @@
         </is>
       </c>
       <c r="J13" t="n">
-        <v>3.37</v>
+        <v>2.25</v>
       </c>
       <c r="K13" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L13" t="n">
-        <v>27833.75</v>
+        <v>27842.5</v>
       </c>
       <c r="M13" t="n">
-        <v>27818.75</v>
+        <v>27827.5</v>
       </c>
       <c r="N13" t="n">
-        <v>27803.75</v>
+        <v>27812.5</v>
       </c>
       <c r="O13" t="n">
         <v>60</v>
@@ -2362,10 +2571,10 @@
         <v>60</v>
       </c>
       <c r="Q13" t="n">
-        <v>27833.75</v>
+        <v>27812.5</v>
       </c>
       <c r="R13" s="4" t="n">
-        <v>-60</v>
+        <v>60</v>
       </c>
       <c r="S13" t="inlineStr">
         <is>
@@ -2378,10 +2587,10 @@
         </is>
       </c>
       <c r="U13" t="n">
-        <v>60</v>
+        <v>10</v>
       </c>
       <c r="V13" t="n">
-        <v>35</v>
+        <v>60</v>
       </c>
       <c r="W13" t="inlineStr">
         <is>
@@ -2397,7 +2606,7 @@
         <v>2311</v>
       </c>
       <c r="Z13" t="n">
-        <v>22.2559</v>
+        <v>17.7671</v>
       </c>
       <c r="AA13" t="inlineStr">
         <is>
@@ -2426,7 +2635,7 @@
       </c>
       <c r="AF13" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="AG13" t="inlineStr">
@@ -2446,7 +2655,7 @@
       </c>
       <c r="AJ13" t="inlineStr">
         <is>
-          <t>SL</t>
+          <t>TP</t>
         </is>
       </c>
       <c r="AK13" t="inlineStr">
@@ -2474,7 +2683,7 @@
         </is>
       </c>
       <c r="AS13" t="n">
-        <v>-250</v>
+        <v>-144</v>
       </c>
       <c r="AT13" t="inlineStr">
         <is>
@@ -2518,16 +2727,16 @@
         <v>150</v>
       </c>
       <c r="E14" t="n">
-        <v>27935.7</v>
+        <v>27935.68</v>
       </c>
       <c r="F14" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G14" t="n">
-        <v>836</v>
+        <v>801</v>
       </c>
       <c r="H14" t="n">
-        <v>-136</v>
+        <v>-135</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -2535,19 +2744,19 @@
         </is>
       </c>
       <c r="J14" t="n">
-        <v>2.75</v>
+        <v>1.99</v>
       </c>
       <c r="K14" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L14" t="n">
-        <v>27997.5</v>
+        <v>27998.75</v>
       </c>
       <c r="M14" t="n">
-        <v>27982.5</v>
+        <v>27983.75</v>
       </c>
       <c r="N14" t="n">
-        <v>27967.5</v>
+        <v>27968.75</v>
       </c>
       <c r="O14" t="n">
         <v>60</v>
@@ -2556,7 +2765,7 @@
         <v>60</v>
       </c>
       <c r="Q14" t="n">
-        <v>27997.5</v>
+        <v>27998.75</v>
       </c>
       <c r="R14" s="4" t="n">
         <v>-60</v>
@@ -2572,10 +2781,10 @@
         </is>
       </c>
       <c r="U14" t="n">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="V14" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="W14" t="inlineStr">
         <is>
@@ -2591,7 +2800,7 @@
         <v>2310</v>
       </c>
       <c r="Z14" t="n">
-        <v>5.4468</v>
+        <v>5.021</v>
       </c>
       <c r="AA14" t="inlineStr">
         <is>
@@ -2600,7 +2809,7 @@
       </c>
       <c r="AB14" t="inlineStr">
         <is>
-          <t>LastTime</t>
+          <t>A+ STRUCTURE</t>
         </is>
       </c>
       <c r="AC14" t="inlineStr">
@@ -2645,15 +2854,23 @@
       </c>
       <c r="AK14" t="inlineStr">
         <is>
-          <t>FALSE</t>
-        </is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AL14" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="AM14" t="n">
+        <v>27993.75</v>
       </c>
       <c r="AN14" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AO14" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="AP14" t="n">
@@ -2668,7 +2885,7 @@
         </is>
       </c>
       <c r="AS14" t="n">
-        <v>-306</v>
+        <v>-305</v>
       </c>
       <c r="AT14" t="inlineStr">
         <is>
@@ -2677,12 +2894,12 @@
       </c>
       <c r="AU14" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="AV14" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>A+ STRUCTURE</t>
         </is>
       </c>
       <c r="AW14" t="inlineStr">
@@ -2712,16 +2929,16 @@
         <v>225</v>
       </c>
       <c r="E15" t="n">
-        <v>28455.06</v>
+        <v>28456.38</v>
       </c>
       <c r="F15" t="n">
-        <v>95</v>
+        <v>5</v>
       </c>
       <c r="G15" t="n">
-        <v>1845</v>
+        <v>1408</v>
       </c>
       <c r="H15" t="n">
-        <v>163</v>
+        <v>150</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -2729,19 +2946,19 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>2.35</v>
+        <v>0.16</v>
       </c>
       <c r="K15" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L15" t="n">
-        <v>28420</v>
+        <v>28378.75</v>
       </c>
       <c r="M15" t="n">
-        <v>28435</v>
+        <v>28393.75</v>
       </c>
       <c r="N15" t="n">
-        <v>28450</v>
+        <v>28408.75</v>
       </c>
       <c r="O15" t="n">
         <v>60</v>
@@ -2750,7 +2967,7 @@
         <v>60</v>
       </c>
       <c r="Q15" t="n">
-        <v>28450</v>
+        <v>28408.75</v>
       </c>
       <c r="R15" s="4" t="n">
         <v>60</v>
@@ -2769,7 +2986,7 @@
         <v>5</v>
       </c>
       <c r="V15" t="n">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="W15" t="inlineStr">
         <is>
@@ -2778,14 +2995,14 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>09:34:00</t>
+          <t>09:32:00</t>
         </is>
       </c>
       <c r="Y15" t="n">
-        <v>2314</v>
+        <v>2312</v>
       </c>
       <c r="Z15" t="n">
-        <v>40.4043</v>
+        <v>31.1546</v>
       </c>
       <c r="AA15" t="inlineStr">
         <is>
@@ -2794,7 +3011,7 @@
       </c>
       <c r="AB15" t="inlineStr">
         <is>
-          <t>LastTime</t>
+          <t>A+ ABSORTION</t>
         </is>
       </c>
       <c r="AC15" t="inlineStr">
@@ -2804,7 +3021,7 @@
       </c>
       <c r="AD15" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="AE15" t="inlineStr">
@@ -2839,22 +3056,30 @@
       </c>
       <c r="AK15" t="inlineStr">
         <is>
-          <t>FALSE</t>
-        </is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AL15" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="AM15" t="n">
+        <v>28397.5</v>
       </c>
       <c r="AN15" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AO15" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="AP15" t="n">
-        <v>2487</v>
+        <v>3447</v>
       </c>
       <c r="AQ15" t="n">
-        <v>-35</v>
+        <v>195</v>
       </c>
       <c r="AR15" t="inlineStr">
         <is>
@@ -2862,11 +3087,11 @@
         </is>
       </c>
       <c r="AS15" t="n">
-        <v>198</v>
+        <v>-45</v>
       </c>
       <c r="AT15" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="AU15" t="inlineStr">
@@ -2876,12 +3101,12 @@
       </c>
       <c r="AV15" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>A+ ABSORTION</t>
         </is>
       </c>
       <c r="AW15" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="AX15" t="inlineStr">
@@ -2906,16 +3131,16 @@
         <v>145</v>
       </c>
       <c r="E16" t="n">
-        <v>28744.56</v>
+        <v>28742.46</v>
       </c>
       <c r="F16" t="n">
-        <v>40</v>
+        <v>5</v>
       </c>
       <c r="G16" t="n">
-        <v>1442</v>
+        <v>907</v>
       </c>
       <c r="H16" t="n">
-        <v>242</v>
+        <v>-45</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -2923,19 +3148,19 @@
         </is>
       </c>
       <c r="J16" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.24</v>
       </c>
       <c r="K16" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="L16" t="n">
-        <v>28761.25</v>
+        <v>28743.75</v>
       </c>
       <c r="M16" t="n">
-        <v>28776.25</v>
+        <v>28728.75</v>
       </c>
       <c r="N16" t="n">
-        <v>28791.25</v>
+        <v>28713.75</v>
       </c>
       <c r="O16" t="n">
         <v>60</v>
@@ -2944,14 +3169,14 @@
         <v>60</v>
       </c>
       <c r="Q16" t="n">
-        <v>28761.25</v>
+        <v>28743.75</v>
       </c>
       <c r="R16" s="4" t="n">
         <v>-60</v>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
@@ -2972,14 +3197,14 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>09:38:00</t>
+          <t>09:32:00</t>
         </is>
       </c>
       <c r="Y16" t="n">
-        <v>2318</v>
+        <v>2312</v>
       </c>
       <c r="Z16" t="n">
-        <v>57.7433</v>
+        <v>21.2575</v>
       </c>
       <c r="AA16" t="inlineStr">
         <is>
@@ -2998,7 +3223,7 @@
       </c>
       <c r="AD16" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="AE16" t="inlineStr">
@@ -3038,11 +3263,11 @@
       </c>
       <c r="AL16" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="AM16" t="n">
-        <v>28777.5</v>
+        <v>28732.5</v>
       </c>
       <c r="AN16" t="n">
         <v>3</v>
@@ -3053,10 +3278,10 @@
         </is>
       </c>
       <c r="AP16" t="n">
-        <v>1647</v>
+        <v>3146</v>
       </c>
       <c r="AQ16" t="n">
-        <v>-1</v>
+        <v>-88</v>
       </c>
       <c r="AR16" t="inlineStr">
         <is>
@@ -3064,16 +3289,16 @@
         </is>
       </c>
       <c r="AS16" t="n">
-        <v>243</v>
+        <v>43</v>
       </c>
       <c r="AT16" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="AU16" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="AV16" t="inlineStr">
@@ -3098,191 +3323,9 @@
           <t>2026-05-08</t>
         </is>
       </c>
-      <c r="B17" t="n">
-        <v>28860</v>
-      </c>
-      <c r="C17" t="n">
-        <v>28903.75</v>
-      </c>
-      <c r="D17" t="n">
-        <v>175</v>
-      </c>
-      <c r="E17" t="n">
-        <v>28876.65</v>
-      </c>
-      <c r="F17" t="n">
-        <v>50</v>
-      </c>
-      <c r="G17" t="n">
-        <v>1703</v>
-      </c>
-      <c r="H17" t="n">
-        <v>213</v>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>normal speed</t>
-        </is>
-      </c>
-      <c r="J17" t="n">
-        <v>2.05</v>
-      </c>
-      <c r="K17" t="n">
-        <v>8</v>
-      </c>
-      <c r="L17" t="n">
-        <v>28901.25</v>
-      </c>
-      <c r="M17" t="n">
-        <v>28916.25</v>
-      </c>
-      <c r="N17" t="n">
-        <v>28931.25</v>
-      </c>
-      <c r="O17" t="n">
-        <v>60</v>
-      </c>
-      <c r="P17" t="n">
-        <v>60</v>
-      </c>
-      <c r="Q17" t="n">
-        <v>28931.25</v>
-      </c>
-      <c r="R17" s="4" t="n">
-        <v>60</v>
-      </c>
-      <c r="S17" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="T17" t="inlineStr">
-        <is>
-          <t>SCALP_NORMAL</t>
-        </is>
-      </c>
-      <c r="U17" t="n">
-        <v>45</v>
-      </c>
-      <c r="V17" t="n">
-        <v>65</v>
-      </c>
-      <c r="W17" t="inlineStr">
-        <is>
-          <t>score-exporter-2026-05-30-aplus-structure-export</t>
-        </is>
-      </c>
-      <c r="X17" t="inlineStr">
-        <is>
-          <t>09:31:00</t>
-        </is>
-      </c>
-      <c r="Y17" t="n">
-        <v>2311</v>
-      </c>
-      <c r="Z17" t="n">
-        <v>24.4185</v>
-      </c>
-      <c r="AA17" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AB17" t="inlineStr">
-        <is>
-          <t>LastTime</t>
-        </is>
-      </c>
-      <c r="AC17" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AD17" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AE17" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AF17" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AG17" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AH17" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AI17" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AJ17" t="inlineStr">
-        <is>
-          <t>TP</t>
-        </is>
-      </c>
-      <c r="AK17" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AN17" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO17" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AP17" t="n">
-        <v>4730</v>
-      </c>
-      <c r="AQ17" t="n">
-        <v>170</v>
-      </c>
-      <c r="AR17" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AS17" t="n">
-        <v>43</v>
-      </c>
-      <c r="AT17" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AU17" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AV17" t="inlineStr">
-        <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="AW17" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AX17" t="inlineStr">
-        <is>
-          <t>FALSE</t>
+      <c r="R17" s="4" t="inlineStr">
+        <is>
+          <t>NO_CSV</t>
         </is>
       </c>
     </row>
@@ -3308,10 +3351,10 @@
         <v>75</v>
       </c>
       <c r="G18" t="n">
-        <v>812</v>
+        <v>816</v>
       </c>
       <c r="H18" t="n">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -3319,7 +3362,7 @@
         </is>
       </c>
       <c r="J18" t="n">
-        <v>10.73</v>
+        <v>10.7</v>
       </c>
       <c r="K18" t="n">
         <v>9</v>
@@ -3375,7 +3418,7 @@
         <v>2311</v>
       </c>
       <c r="Z18" t="n">
-        <v>6.9889</v>
+        <v>7.0112</v>
       </c>
       <c r="AA18" t="inlineStr">
         <is>
@@ -3452,7 +3495,7 @@
         </is>
       </c>
       <c r="AS18" t="n">
-        <v>-162</v>
+        <v>-158</v>
       </c>
       <c r="AT18" t="inlineStr">
         <is>
@@ -3508,64 +3551,64 @@
         <v>145</v>
       </c>
       <c r="E20" t="n">
-        <v>29321.15</v>
+        <v>29321.56</v>
       </c>
       <c r="F20" t="n">
+        <v>20</v>
+      </c>
+      <c r="G20" t="n">
+        <v>843</v>
+      </c>
+      <c r="H20" t="n">
+        <v>-131</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>normal speed</t>
+        </is>
+      </c>
+      <c r="J20" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="K20" t="n">
+        <v>10</v>
+      </c>
+      <c r="L20" t="n">
+        <v>29262.5</v>
+      </c>
+      <c r="M20" t="n">
+        <v>29247.5</v>
+      </c>
+      <c r="N20" t="n">
+        <v>29232.5</v>
+      </c>
+      <c r="O20" t="n">
+        <v>60</v>
+      </c>
+      <c r="P20" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>29232.5</v>
+      </c>
+      <c r="R20" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>SCALP_NORMAL</t>
+        </is>
+      </c>
+      <c r="U20" t="n">
+        <v>30</v>
+      </c>
+      <c r="V20" t="n">
         <v>65</v>
-      </c>
-      <c r="G20" t="n">
-        <v>1341</v>
-      </c>
-      <c r="H20" t="n">
-        <v>-263</v>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>normal speed</t>
-        </is>
-      </c>
-      <c r="J20" t="n">
-        <v>3.49</v>
-      </c>
-      <c r="K20" t="n">
-        <v>8</v>
-      </c>
-      <c r="L20" t="n">
-        <v>29251.25</v>
-      </c>
-      <c r="M20" t="n">
-        <v>29236.25</v>
-      </c>
-      <c r="N20" t="n">
-        <v>29221.25</v>
-      </c>
-      <c r="O20" t="n">
-        <v>60</v>
-      </c>
-      <c r="P20" t="n">
-        <v>60</v>
-      </c>
-      <c r="Q20" t="n">
-        <v>29221.25</v>
-      </c>
-      <c r="R20" s="4" t="n">
-        <v>60</v>
-      </c>
-      <c r="S20" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="T20" t="inlineStr">
-        <is>
-          <t>SCALP_NORMAL</t>
-        </is>
-      </c>
-      <c r="U20" t="n">
-        <v>15</v>
-      </c>
-      <c r="V20" t="n">
-        <v>60</v>
       </c>
       <c r="W20" t="inlineStr">
         <is>
@@ -3581,7 +3624,7 @@
         <v>2311</v>
       </c>
       <c r="Z20" t="n">
-        <v>18.6189</v>
+        <v>12.517</v>
       </c>
       <c r="AA20" t="inlineStr">
         <is>
@@ -3590,7 +3633,7 @@
       </c>
       <c r="AB20" t="inlineStr">
         <is>
-          <t>LastTime</t>
+          <t>A+ ABSORTION</t>
         </is>
       </c>
       <c r="AC20" t="inlineStr">
@@ -3635,15 +3678,23 @@
       </c>
       <c r="AK20" t="inlineStr">
         <is>
-          <t>FALSE</t>
-        </is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AL20" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="AM20" t="n">
+        <v>29247.5</v>
       </c>
       <c r="AN20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AO20" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="AP20" t="n">
@@ -3658,7 +3709,7 @@
         </is>
       </c>
       <c r="AS20" t="n">
-        <v>138</v>
+        <v>270</v>
       </c>
       <c r="AT20" t="inlineStr">
         <is>
@@ -3672,12 +3723,12 @@
       </c>
       <c r="AV20" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>A+ ABSORTION</t>
         </is>
       </c>
       <c r="AW20" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="AX20" t="inlineStr">
@@ -3708,10 +3759,10 @@
         <v>40</v>
       </c>
       <c r="G21" t="n">
-        <v>1618</v>
+        <v>1620</v>
       </c>
       <c r="H21" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -3775,7 +3826,7 @@
         <v>2311</v>
       </c>
       <c r="Z21" t="n">
-        <v>21.1943</v>
+        <v>21.22</v>
       </c>
       <c r="AA21" t="inlineStr">
         <is>
@@ -3860,7 +3911,7 @@
         </is>
       </c>
       <c r="AS21" t="n">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="AT21" t="inlineStr">
         <is>
@@ -3907,13 +3958,13 @@
         <v>29294.78</v>
       </c>
       <c r="F22" t="n">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="G22" t="n">
-        <v>818</v>
+        <v>814</v>
       </c>
       <c r="H22" t="n">
-        <v>-356</v>
+        <v>-358</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -3921,19 +3972,19 @@
         </is>
       </c>
       <c r="J22" t="n">
-        <v>16.9</v>
+        <v>18.05</v>
       </c>
       <c r="K22" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="L22" t="n">
-        <v>29235</v>
+        <v>29233.75</v>
       </c>
       <c r="M22" t="n">
-        <v>29220</v>
+        <v>29218.75</v>
       </c>
       <c r="N22" t="n">
-        <v>29205</v>
+        <v>29203.75</v>
       </c>
       <c r="O22" t="n">
         <v>60</v>
@@ -3942,7 +3993,7 @@
         <v>60</v>
       </c>
       <c r="Q22" t="n">
-        <v>29205</v>
+        <v>29203.75</v>
       </c>
       <c r="R22" s="4" t="n">
         <v>60</v>
@@ -3958,7 +4009,7 @@
         </is>
       </c>
       <c r="U22" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="V22" t="n">
         <v>60</v>
@@ -3977,7 +4028,7 @@
         <v>2311</v>
       </c>
       <c r="Z22" t="n">
-        <v>5.0304</v>
+        <v>4.9856</v>
       </c>
       <c r="AA22" t="inlineStr">
         <is>
@@ -4031,11 +4082,19 @@
       </c>
       <c r="AK22" t="inlineStr">
         <is>
-          <t>FALSE</t>
-        </is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AL22" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="AM22" t="n">
+        <v>29251.25</v>
       </c>
       <c r="AN22" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AO22" t="inlineStr">
         <is>
@@ -4054,7 +4113,7 @@
         </is>
       </c>
       <c r="AS22" t="n">
-        <v>-492</v>
+        <v>-494</v>
       </c>
       <c r="AT22" t="inlineStr">
         <is>
@@ -4063,12 +4122,12 @@
       </c>
       <c r="AU22" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="AV22" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>A+ STRUCTURE</t>
         </is>
       </c>
       <c r="AW22" t="inlineStr">
@@ -4088,191 +4147,9 @@
           <t>2026-05-18</t>
         </is>
       </c>
-      <c r="B23" t="n">
-        <v>29305</v>
-      </c>
-      <c r="C23" t="n">
-        <v>29356.25</v>
-      </c>
-      <c r="D23" t="n">
-        <v>205</v>
-      </c>
-      <c r="E23" t="n">
-        <v>29211.89</v>
-      </c>
-      <c r="F23" t="n">
-        <v>50</v>
-      </c>
-      <c r="G23" t="n">
-        <v>809</v>
-      </c>
-      <c r="H23" t="n">
-        <v>-159</v>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>normal speed</t>
-        </is>
-      </c>
-      <c r="J23" t="n">
-        <v>3.82</v>
-      </c>
-      <c r="K23" t="n">
-        <v>6</v>
-      </c>
-      <c r="L23" t="n">
-        <v>29298.75</v>
-      </c>
-      <c r="M23" t="n">
-        <v>29283.75</v>
-      </c>
-      <c r="N23" t="n">
-        <v>29268.75</v>
-      </c>
-      <c r="O23" t="n">
-        <v>60</v>
-      </c>
-      <c r="P23" t="n">
-        <v>60</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>29298.75</v>
-      </c>
-      <c r="R23" s="4" t="n">
-        <v>-60</v>
-      </c>
-      <c r="S23" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="T23" t="inlineStr">
-        <is>
-          <t>SCALP_NORMAL</t>
-        </is>
-      </c>
-      <c r="U23" t="n">
-        <v>60</v>
-      </c>
-      <c r="V23" t="n">
-        <v>5</v>
-      </c>
-      <c r="W23" t="inlineStr">
-        <is>
-          <t>score-exporter-2026-05-30-aplus-structure-export</t>
-        </is>
-      </c>
-      <c r="X23" t="inlineStr">
-        <is>
-          <t>09:33:00</t>
-        </is>
-      </c>
-      <c r="Y23" t="n">
-        <v>2313</v>
-      </c>
-      <c r="Z23" t="n">
-        <v>13.1022</v>
-      </c>
-      <c r="AA23" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AB23" t="inlineStr">
-        <is>
-          <t>LastTime</t>
-        </is>
-      </c>
-      <c r="AC23" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AD23" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AE23" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AF23" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AG23" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AH23" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AI23" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AJ23" t="inlineStr">
-        <is>
-          <t>SL</t>
-        </is>
-      </c>
-      <c r="AK23" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AN23" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO23" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AP23" t="n">
-        <v>3452</v>
-      </c>
-      <c r="AQ23" t="n">
-        <v>-98</v>
-      </c>
-      <c r="AR23" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AS23" t="n">
-        <v>-61</v>
-      </c>
-      <c r="AT23" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AU23" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AV23" t="inlineStr">
-        <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="AW23" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AX23" t="inlineStr">
-        <is>
-          <t>FALSE</t>
+      <c r="R23" s="4" t="inlineStr">
+        <is>
+          <t>NO_CSV</t>
         </is>
       </c>
     </row>
@@ -4292,36 +4169,36 @@
         <v>370</v>
       </c>
       <c r="E24" t="n">
-        <v>28925.32</v>
+        <v>28924.85</v>
       </c>
       <c r="F24" t="n">
-        <v>95</v>
+        <v>5</v>
       </c>
       <c r="G24" t="n">
-        <v>1254</v>
+        <v>2634</v>
       </c>
       <c r="H24" t="n">
-        <v>280</v>
+        <v>150</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>A+ speed</t>
+          <t>normal speed</t>
         </is>
       </c>
       <c r="J24" t="n">
-        <v>6.1</v>
+        <v>0.14</v>
       </c>
       <c r="K24" t="n">
         <v>8</v>
       </c>
       <c r="L24" t="n">
-        <v>28952.5</v>
+        <v>28930</v>
       </c>
       <c r="M24" t="n">
-        <v>28967.5</v>
+        <v>28945</v>
       </c>
       <c r="N24" t="n">
-        <v>28982.5</v>
+        <v>28960</v>
       </c>
       <c r="O24" t="n">
         <v>60</v>
@@ -4330,7 +4207,7 @@
         <v>60</v>
       </c>
       <c r="Q24" t="n">
-        <v>28982.5</v>
+        <v>28960</v>
       </c>
       <c r="R24" s="4" t="n">
         <v>60</v>
@@ -4342,11 +4219,11 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>POTENTIAL_RUNNER</t>
+          <t>SCALP_NORMAL</t>
         </is>
       </c>
       <c r="U24" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="V24" t="n">
         <v>60</v>
@@ -4358,14 +4235,14 @@
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>09:32:00</t>
+          <t>09:31:00</t>
         </is>
       </c>
       <c r="Y24" t="n">
-        <v>2312</v>
+        <v>2311</v>
       </c>
       <c r="Z24" t="n">
-        <v>15.5645</v>
+        <v>35.7781</v>
       </c>
       <c r="AA24" t="inlineStr">
         <is>
@@ -4374,7 +4251,7 @@
       </c>
       <c r="AB24" t="inlineStr">
         <is>
-          <t>LastTime</t>
+          <t>A+ ABSORTION</t>
         </is>
       </c>
       <c r="AC24" t="inlineStr">
@@ -4384,7 +4261,7 @@
       </c>
       <c r="AD24" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="AE24" t="inlineStr">
@@ -4419,22 +4296,30 @@
       </c>
       <c r="AK24" t="inlineStr">
         <is>
-          <t>FALSE</t>
-        </is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AL24" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="AM24" t="n">
+        <v>28933.75</v>
       </c>
       <c r="AN24" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AO24" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="AP24" t="n">
-        <v>4358</v>
+        <v>8651</v>
       </c>
       <c r="AQ24" t="n">
-        <v>-32</v>
+        <v>405</v>
       </c>
       <c r="AR24" t="inlineStr">
         <is>
@@ -4442,26 +4327,26 @@
         </is>
       </c>
       <c r="AS24" t="n">
-        <v>312</v>
+        <v>-255</v>
       </c>
       <c r="AT24" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="AU24" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="AV24" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>A+ ABSORTION</t>
         </is>
       </c>
       <c r="AW24" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="AX24" t="inlineStr">
@@ -4476,191 +4361,9 @@
           <t>2026-05-20</t>
         </is>
       </c>
-      <c r="B25" t="n">
-        <v>29070</v>
-      </c>
-      <c r="C25" t="n">
-        <v>29122.5</v>
-      </c>
-      <c r="D25" t="n">
-        <v>210</v>
-      </c>
-      <c r="E25" t="n">
-        <v>29074.6</v>
-      </c>
-      <c r="F25" t="n">
-        <v>20</v>
-      </c>
-      <c r="G25" t="n">
-        <v>1158</v>
-      </c>
-      <c r="H25" t="n">
-        <v>196</v>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>normal speed</t>
-        </is>
-      </c>
-      <c r="J25" t="n">
-        <v>2.4</v>
-      </c>
-      <c r="K25" t="n">
-        <v>8</v>
-      </c>
-      <c r="L25" t="n">
-        <v>29112.5</v>
-      </c>
-      <c r="M25" t="n">
-        <v>29127.5</v>
-      </c>
-      <c r="N25" t="n">
-        <v>29142.5</v>
-      </c>
-      <c r="O25" t="n">
-        <v>60</v>
-      </c>
-      <c r="P25" t="n">
-        <v>60</v>
-      </c>
-      <c r="Q25" t="n">
-        <v>29112.5</v>
-      </c>
-      <c r="R25" s="4" t="n">
-        <v>-60</v>
-      </c>
-      <c r="S25" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="T25" t="inlineStr">
-        <is>
-          <t>SCALP_NORMAL</t>
-        </is>
-      </c>
-      <c r="U25" t="n">
-        <v>60</v>
-      </c>
-      <c r="V25" t="n">
-        <v>35</v>
-      </c>
-      <c r="W25" t="inlineStr">
-        <is>
-          <t>score-exporter-2026-05-30-aplus-structure-export</t>
-        </is>
-      </c>
-      <c r="X25" t="inlineStr">
-        <is>
-          <t>09:31:00</t>
-        </is>
-      </c>
-      <c r="Y25" t="n">
-        <v>2311</v>
-      </c>
-      <c r="Z25" t="n">
-        <v>8.349399999999999</v>
-      </c>
-      <c r="AA25" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AB25" t="inlineStr">
-        <is>
-          <t>LastTime</t>
-        </is>
-      </c>
-      <c r="AC25" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AD25" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AE25" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AF25" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AG25" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AH25" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AI25" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AJ25" t="inlineStr">
-        <is>
-          <t>SL</t>
-        </is>
-      </c>
-      <c r="AK25" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AN25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO25" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AP25" t="n">
-        <v>5619</v>
-      </c>
-      <c r="AQ25" t="n">
-        <v>211</v>
-      </c>
-      <c r="AR25" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AS25" t="n">
-        <v>-15</v>
-      </c>
-      <c r="AT25" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AU25" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AV25" t="inlineStr">
-        <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="AW25" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AX25" t="inlineStr">
-        <is>
-          <t>FALSE</t>
+      <c r="R25" s="4" t="inlineStr">
+        <is>
+          <t>NO_CSV</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
added Cummulative Volume Delta y Delta Change
</commit_message>
<xml_diff>
--- a/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
+++ b/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX25"/>
+  <dimension ref="A1:AZ25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -722,6 +722,16 @@
           <t>APlus_Speed</t>
         </is>
       </c>
+      <c r="AY3" s="3" t="inlineStr">
+        <is>
+          <t>Cumulative_Delta_entry</t>
+        </is>
+      </c>
+      <c r="AZ3" s="3" t="inlineStr">
+        <is>
+          <t>Cumulative_Delta_Source</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -739,16 +749,16 @@
         <v>175</v>
       </c>
       <c r="E4" t="n">
-        <v>28876.35</v>
+        <v>28876.34</v>
       </c>
       <c r="F4" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G4" t="n">
-        <v>1044</v>
+        <v>1035</v>
       </c>
       <c r="H4" t="n">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -756,19 +766,19 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>0.97</v>
+        <v>0.65</v>
       </c>
       <c r="K4" t="n">
         <v>10</v>
       </c>
       <c r="L4" t="n">
-        <v>28892.5</v>
+        <v>28891.25</v>
       </c>
       <c r="M4" t="n">
-        <v>28907.5</v>
+        <v>28906.25</v>
       </c>
       <c r="N4" t="n">
-        <v>28922.5</v>
+        <v>28921.25</v>
       </c>
       <c r="O4" t="n">
         <v>60</v>
@@ -777,7 +787,7 @@
         <v>60</v>
       </c>
       <c r="Q4" t="n">
-        <v>28922.5</v>
+        <v>28921.25</v>
       </c>
       <c r="R4" s="4" t="n">
         <v>60</v>
@@ -793,7 +803,7 @@
         </is>
       </c>
       <c r="U4" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="V4" t="n">
         <v>60</v>
@@ -812,7 +822,7 @@
         <v>2311</v>
       </c>
       <c r="Z4" t="n">
-        <v>15.4393</v>
+        <v>15.3696</v>
       </c>
       <c r="AA4" t="inlineStr">
         <is>
@@ -897,7 +907,7 @@
         </is>
       </c>
       <c r="AS4" t="n">
-        <v>-112</v>
+        <v>-115</v>
       </c>
       <c r="AT4" t="inlineStr">
         <is>
@@ -906,7 +916,7 @@
       </c>
       <c r="AU4" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="AV4" t="inlineStr">
@@ -922,6 +932,14 @@
       <c r="AX4" t="inlineStr">
         <is>
           <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AY4" t="n">
+        <v>1381</v>
+      </c>
+      <c r="AZ4" t="inlineStr">
+        <is>
+          <t>SessionDeltaSum</t>
         </is>
       </c>
     </row>
@@ -947,7 +965,7 @@
         <v>5</v>
       </c>
       <c r="G5" t="n">
-        <v>2829</v>
+        <v>2827</v>
       </c>
       <c r="H5" t="n">
         <v>-245</v>
@@ -1014,7 +1032,7 @@
         <v>2315</v>
       </c>
       <c r="Z5" t="n">
-        <v>57.0282</v>
+        <v>56.9984</v>
       </c>
       <c r="AA5" t="inlineStr">
         <is>
@@ -1126,6 +1144,14 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="AY5" t="n">
+        <v>-1836</v>
+      </c>
+      <c r="AZ5" t="inlineStr">
+        <is>
+          <t>SessionDeltaSum</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1143,16 +1169,16 @@
         <v>205</v>
       </c>
       <c r="E6" t="n">
-        <v>29211.89</v>
+        <v>29211.08</v>
       </c>
       <c r="F6" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="G6" t="n">
-        <v>800</v>
+        <v>2599</v>
       </c>
       <c r="H6" t="n">
-        <v>-160</v>
+        <v>-217</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -1160,19 +1186,19 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>4.69</v>
+        <v>1.1</v>
       </c>
       <c r="K6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L6" t="n">
-        <v>29296.25</v>
+        <v>29307.5</v>
       </c>
       <c r="M6" t="n">
-        <v>29281.25</v>
+        <v>29292.5</v>
       </c>
       <c r="N6" t="n">
-        <v>29266.25</v>
+        <v>29277.5</v>
       </c>
       <c r="O6" t="n">
         <v>60</v>
@@ -1181,10 +1207,10 @@
         <v>60</v>
       </c>
       <c r="Q6" t="n">
-        <v>29296.25</v>
+        <v>29277.5</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>-60</v>
+        <v>60</v>
       </c>
       <c r="S6" t="inlineStr">
         <is>
@@ -1197,10 +1223,10 @@
         </is>
       </c>
       <c r="U6" t="n">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="V6" t="n">
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="W6" t="inlineStr">
         <is>
@@ -1209,14 +1235,14 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>09:33:00</t>
+          <t>09:32:00</t>
         </is>
       </c>
       <c r="Y6" t="n">
-        <v>2313</v>
+        <v>2312</v>
       </c>
       <c r="Z6" t="n">
-        <v>12.781</v>
+        <v>45.6277</v>
       </c>
       <c r="AA6" t="inlineStr">
         <is>
@@ -1225,7 +1251,7 @@
       </c>
       <c r="AB6" t="inlineStr">
         <is>
-          <t>LastTime</t>
+          <t>A+ STRUCTURE</t>
         </is>
       </c>
       <c r="AC6" t="inlineStr">
@@ -1265,27 +1291,35 @@
       </c>
       <c r="AJ6" t="inlineStr">
         <is>
-          <t>SL</t>
+          <t>TP</t>
         </is>
       </c>
       <c r="AK6" t="inlineStr">
         <is>
-          <t>FALSE</t>
-        </is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AL6" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="AM6" t="n">
+        <v>29295</v>
       </c>
       <c r="AN6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AO6" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="AP6" t="n">
-        <v>3452</v>
+        <v>4070</v>
       </c>
       <c r="AQ6" t="n">
-        <v>-98</v>
+        <v>134</v>
       </c>
       <c r="AR6" t="inlineStr">
         <is>
@@ -1293,7 +1327,7 @@
         </is>
       </c>
       <c r="AS6" t="n">
-        <v>-62</v>
+        <v>-351</v>
       </c>
       <c r="AT6" t="inlineStr">
         <is>
@@ -1302,12 +1336,12 @@
       </c>
       <c r="AU6" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="AV6" t="inlineStr">
         <is>
-          <t>BREAKOUT</t>
+          <t>A+ STRUCTURE</t>
         </is>
       </c>
       <c r="AW6" t="inlineStr">
@@ -1318,6 +1352,14 @@
       <c r="AX6" t="inlineStr">
         <is>
           <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AY6" t="n">
+        <v>2242</v>
+      </c>
+      <c r="AZ6" t="inlineStr">
+        <is>
+          <t>SessionDeltaSum</t>
         </is>
       </c>
     </row>
@@ -1337,16 +1379,16 @@
         <v>210</v>
       </c>
       <c r="E7" t="n">
-        <v>29074.6</v>
+        <v>29074.59</v>
       </c>
       <c r="F7" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="G7" t="n">
-        <v>1137</v>
+        <v>1131</v>
       </c>
       <c r="H7" t="n">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -1354,19 +1396,19 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>3.03</v>
+        <v>2.48</v>
       </c>
       <c r="K7" t="n">
         <v>8</v>
       </c>
       <c r="L7" t="n">
-        <v>29113.75</v>
+        <v>29112.5</v>
       </c>
       <c r="M7" t="n">
-        <v>29128.75</v>
+        <v>29127.5</v>
       </c>
       <c r="N7" t="n">
-        <v>29143.75</v>
+        <v>29142.5</v>
       </c>
       <c r="O7" t="n">
         <v>60</v>
@@ -1375,7 +1417,7 @@
         <v>60</v>
       </c>
       <c r="Q7" t="n">
-        <v>29113.75</v>
+        <v>29112.5</v>
       </c>
       <c r="R7" s="4" t="n">
         <v>-60</v>
@@ -1394,7 +1436,7 @@
         <v>60</v>
       </c>
       <c r="V7" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="W7" t="inlineStr">
         <is>
@@ -1410,7 +1452,7 @@
         <v>2311</v>
       </c>
       <c r="Z7" t="n">
-        <v>8.241400000000001</v>
+        <v>8.072800000000001</v>
       </c>
       <c r="AA7" t="inlineStr">
         <is>
@@ -1487,7 +1529,7 @@
         </is>
       </c>
       <c r="AS7" t="n">
-        <v>-30</v>
+        <v>-28</v>
       </c>
       <c r="AT7" t="inlineStr">
         <is>
@@ -1512,6 +1554,14 @@
       <c r="AX7" t="inlineStr">
         <is>
           <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AY7" t="n">
+        <v>1157</v>
+      </c>
+      <c r="AZ7" t="inlineStr">
+        <is>
+          <t>SessionDeltaSum</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
normal speed permitida solo para A+ ABSORTION  y A+ STRUCTURE
</commit_message>
<xml_diff>
--- a/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
+++ b/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AZ25"/>
+  <dimension ref="A1:BD25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -463,11 +463,11 @@
     </row>
     <row r="2">
       <c r="A2" s="1">
-        <f>IF((COUNTIF(R4:R7,"&gt;0")+COUNTIF(R4:R7,"&lt;0"))=0,"",COUNTIF(R4:R7,"&gt;0")/(COUNTIF(R4:R7,"&gt;0")+COUNTIF(R4:R7,"&lt;0")))</f>
+        <f>IF((COUNTIF(R4:R15,"&gt;0")+COUNTIF(R4:R15,"&lt;0"))=0,"",COUNTIF(R4:R15,"&gt;0")/(COUNTIF(R4:R15,"&gt;0")+COUNTIF(R4:R15,"&lt;0")))</f>
         <v/>
       </c>
       <c r="B2" s="2">
-        <f>IF(ABS(SUMIF(R4:R7,"&lt;0",R4:R7))=0,IF(SUMIF(R4:R7,"&gt;0",R4:R7)&gt;0,"INF",""),SUMIF(R4:R7,"&gt;0",R4:R7)/ABS(SUMIF(R4:R7,"&lt;0",R4:R7)))</f>
+        <f>IF(ABS(SUMIF(R4:R15,"&lt;0",R4:R15))=0,IF(SUMIF(R4:R15,"&gt;0",R4:R15)&gt;0,"INF",""),SUMIF(R4:R15,"&gt;0",R4:R15)/ABS(SUMIF(R4:R15,"&lt;0",R4:R15)))</f>
         <v/>
       </c>
     </row>
@@ -732,53 +732,73 @@
           <t>Cumulative_Delta_Source</t>
         </is>
       </c>
+      <c r="BA3" s="3" t="inlineStr">
+        <is>
+          <t>Cvd_Peak</t>
+        </is>
+      </c>
+      <c r="BB3" s="3" t="inlineStr">
+        <is>
+          <t>Cvd_Current</t>
+        </is>
+      </c>
+      <c r="BC3" s="3" t="inlineStr">
+        <is>
+          <t>Cvd_Pullback_Pct</t>
+        </is>
+      </c>
+      <c r="BD3" s="3" t="inlineStr">
+        <is>
+          <t>Cvd_Pullback_Label</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>28860</v>
+        <v>29305</v>
       </c>
       <c r="C4" t="n">
-        <v>28903.75</v>
+        <v>29356.25</v>
       </c>
       <c r="D4" t="n">
-        <v>175</v>
+        <v>205</v>
       </c>
       <c r="E4" t="n">
-        <v>28876.34</v>
+        <v>29215.95</v>
       </c>
       <c r="F4" t="n">
-        <v>10</v>
+        <v>150</v>
       </c>
       <c r="G4" t="n">
-        <v>1035</v>
+        <v>1001</v>
       </c>
       <c r="H4" t="n">
-        <v>55</v>
+        <v>-199</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>normal speed</t>
+          <t>A+ speed</t>
         </is>
       </c>
       <c r="J4" t="n">
-        <v>0.65</v>
+        <v>8.449999999999999</v>
       </c>
       <c r="K4" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="L4" t="n">
-        <v>28891.25</v>
+        <v>29273.75</v>
       </c>
       <c r="M4" t="n">
-        <v>28906.25</v>
+        <v>29258.75</v>
       </c>
       <c r="N4" t="n">
-        <v>28921.25</v>
+        <v>29243.75</v>
       </c>
       <c r="O4" t="n">
         <v>60</v>
@@ -787,23 +807,23 @@
         <v>60</v>
       </c>
       <c r="Q4" t="n">
-        <v>28921.25</v>
+        <v>29243.75</v>
       </c>
       <c r="R4" s="4" t="n">
         <v>60</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>SCALP_NORMAL</t>
+          <t>POTENTIAL_RUNNER</t>
         </is>
       </c>
       <c r="U4" t="n">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="V4" t="n">
         <v>60</v>
@@ -815,14 +835,14 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>09:31:00</t>
+          <t>09:36:00</t>
         </is>
       </c>
       <c r="Y4" t="n">
-        <v>2311</v>
+        <v>2316</v>
       </c>
       <c r="Z4" t="n">
-        <v>15.3696</v>
+        <v>17.7459</v>
       </c>
       <c r="AA4" t="inlineStr">
         <is>
@@ -831,7 +851,7 @@
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>A+ ABSORTION</t>
+          <t>LastTime</t>
         </is>
       </c>
       <c r="AC4" t="inlineStr">
@@ -861,7 +881,7 @@
       </c>
       <c r="AH4" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="AI4" t="inlineStr">
@@ -876,30 +896,22 @@
       </c>
       <c r="AK4" t="inlineStr">
         <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AL4" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="AM4" t="n">
-        <v>28906.25</v>
+          <t>FALSE</t>
+        </is>
       </c>
       <c r="AN4" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AO4" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="AP4" t="n">
-        <v>4730</v>
+        <v>2804</v>
       </c>
       <c r="AQ4" t="n">
-        <v>170</v>
+        <v>-58</v>
       </c>
       <c r="AR4" t="inlineStr">
         <is>
@@ -907,11 +919,11 @@
         </is>
       </c>
       <c r="AS4" t="n">
-        <v>-115</v>
+        <v>-141</v>
       </c>
       <c r="AT4" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="AU4" t="inlineStr">
@@ -921,12 +933,12 @@
       </c>
       <c r="AV4" t="inlineStr">
         <is>
-          <t>A+ ABSORTION</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
@@ -935,60 +947,74 @@
         </is>
       </c>
       <c r="AY4" t="n">
-        <v>1381</v>
+        <v>2215</v>
       </c>
       <c r="AZ4" t="inlineStr">
         <is>
           <t>SessionDeltaSum</t>
+        </is>
+      </c>
+      <c r="BA4" t="n">
+        <v>2135</v>
+      </c>
+      <c r="BB4" t="n">
+        <v>2215</v>
+      </c>
+      <c r="BC4" t="n">
+        <v>5.33</v>
+      </c>
+      <c r="BD4" t="inlineStr">
+        <is>
+          <t>Riesgo de reversion</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>29146.25</v>
+        <v>28851.25</v>
       </c>
       <c r="C5" t="n">
-        <v>29227.5</v>
+        <v>28943.75</v>
       </c>
       <c r="D5" t="n">
-        <v>325</v>
+        <v>370</v>
       </c>
       <c r="E5" t="n">
-        <v>29203.49</v>
+        <v>28925.31</v>
       </c>
       <c r="F5" t="n">
-        <v>5</v>
+        <v>90</v>
       </c>
       <c r="G5" t="n">
-        <v>2827</v>
+        <v>1259</v>
       </c>
       <c r="H5" t="n">
-        <v>-245</v>
+        <v>281</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>normal speed</t>
+          <t>A+ speed</t>
         </is>
       </c>
       <c r="J5" t="n">
-        <v>0.09</v>
+        <v>5.76</v>
       </c>
       <c r="K5" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="L5" t="n">
-        <v>29160</v>
+        <v>28951.25</v>
       </c>
       <c r="M5" t="n">
-        <v>29145</v>
+        <v>28966.25</v>
       </c>
       <c r="N5" t="n">
-        <v>29130</v>
+        <v>28981.25</v>
       </c>
       <c r="O5" t="n">
         <v>60</v>
@@ -997,127 +1023,119 @@
         <v>60</v>
       </c>
       <c r="Q5" t="n">
-        <v>29160</v>
+        <v>28981.25</v>
       </c>
       <c r="R5" s="4" t="n">
-        <v>-60</v>
+        <v>60</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>SCALP_NORMAL</t>
+          <t>POTENTIAL_RUNNER</t>
         </is>
       </c>
       <c r="U5" t="n">
-        <v>60</v>
+        <v>5</v>
       </c>
       <c r="V5" t="n">
+        <v>65</v>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-aplus-structure-export</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>09:32:00</t>
+        </is>
+      </c>
+      <c r="Y5" t="n">
+        <v>2312</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>15.635</v>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ5" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="AK5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AN5" t="n">
         <v>0</v>
       </c>
-      <c r="W5" t="inlineStr">
-        <is>
-          <t>score-exporter-2026-05-30-aplus-structure-export</t>
-        </is>
-      </c>
-      <c r="X5" t="inlineStr">
-        <is>
-          <t>09:35:00</t>
-        </is>
-      </c>
-      <c r="Y5" t="n">
-        <v>2315</v>
-      </c>
-      <c r="Z5" t="n">
-        <v>56.9984</v>
-      </c>
-      <c r="AA5" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AB5" t="inlineStr">
-        <is>
-          <t>A+ STRUCTURE</t>
-        </is>
-      </c>
-      <c r="AC5" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AD5" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AE5" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AF5" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AG5" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AH5" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AI5" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AJ5" t="inlineStr">
-        <is>
-          <t>SL</t>
-        </is>
-      </c>
-      <c r="AK5" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AL5" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="AM5" t="n">
-        <v>29146.25</v>
-      </c>
-      <c r="AN5" t="n">
-        <v>3</v>
-      </c>
       <c r="AO5" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="AP5" t="n">
-        <v>2738</v>
+        <v>4358</v>
       </c>
       <c r="AQ5" t="n">
-        <v>52</v>
+        <v>-32</v>
       </c>
       <c r="AR5" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="AS5" t="n">
-        <v>-297</v>
+        <v>313</v>
       </c>
       <c r="AT5" t="inlineStr">
         <is>
@@ -1126,12 +1144,12 @@
       </c>
       <c r="AU5" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="AV5" t="inlineStr">
         <is>
-          <t>A+ STRUCTURE</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="AW5" t="inlineStr">
@@ -1145,60 +1163,74 @@
         </is>
       </c>
       <c r="AY5" t="n">
-        <v>-1836</v>
+        <v>473</v>
       </c>
       <c r="AZ5" t="inlineStr">
         <is>
           <t>SessionDeltaSum</t>
+        </is>
+      </c>
+      <c r="BA5" t="n">
+        <v>473</v>
+      </c>
+      <c r="BB5" t="n">
+        <v>473</v>
+      </c>
+      <c r="BC5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD5" t="inlineStr">
+        <is>
+          <t>Excelente</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>29305</v>
+        <v>29070</v>
       </c>
       <c r="C6" t="n">
-        <v>29356.25</v>
+        <v>29122.5</v>
       </c>
       <c r="D6" t="n">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="E6" t="n">
-        <v>29211.08</v>
+        <v>29081.21</v>
       </c>
       <c r="F6" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="G6" t="n">
-        <v>2599</v>
+        <v>811</v>
       </c>
       <c r="H6" t="n">
-        <v>-217</v>
+        <v>-181</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>normal speed</t>
+          <t>A+ speed</t>
         </is>
       </c>
       <c r="J6" t="n">
-        <v>1.1</v>
+        <v>9.75</v>
       </c>
       <c r="K6" t="n">
         <v>8</v>
       </c>
       <c r="L6" t="n">
-        <v>29307.5</v>
+        <v>29071.25</v>
       </c>
       <c r="M6" t="n">
-        <v>29292.5</v>
+        <v>29056.25</v>
       </c>
       <c r="N6" t="n">
-        <v>29277.5</v>
+        <v>29041.25</v>
       </c>
       <c r="O6" t="n">
         <v>60</v>
@@ -1207,10 +1239,10 @@
         <v>60</v>
       </c>
       <c r="Q6" t="n">
-        <v>29277.5</v>
+        <v>29071.25</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>60</v>
+        <v>-60</v>
       </c>
       <c r="S6" t="inlineStr">
         <is>
@@ -1219,14 +1251,14 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>SCALP_NORMAL</t>
+          <t>POTENTIAL_RUNNER</t>
         </is>
       </c>
       <c r="U6" t="n">
-        <v>45</v>
+        <v>65</v>
       </c>
       <c r="V6" t="n">
-        <v>65</v>
+        <v>25</v>
       </c>
       <c r="W6" t="inlineStr">
         <is>
@@ -1235,14 +1267,14 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>09:32:00</t>
+          <t>09:36:00</t>
         </is>
       </c>
       <c r="Y6" t="n">
-        <v>2312</v>
+        <v>2316</v>
       </c>
       <c r="Z6" t="n">
-        <v>45.6277</v>
+        <v>4.614</v>
       </c>
       <c r="AA6" t="inlineStr">
         <is>
@@ -1251,7 +1283,7 @@
       </c>
       <c r="AB6" t="inlineStr">
         <is>
-          <t>A+ STRUCTURE</t>
+          <t>LastTime</t>
         </is>
       </c>
       <c r="AC6" t="inlineStr">
@@ -1281,7 +1313,7 @@
       </c>
       <c r="AH6" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="AI6" t="inlineStr">
@@ -1291,35 +1323,27 @@
       </c>
       <c r="AJ6" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>SL</t>
         </is>
       </c>
       <c r="AK6" t="inlineStr">
         <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AL6" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="AM6" t="n">
-        <v>29295</v>
+          <t>FALSE</t>
+        </is>
       </c>
       <c r="AN6" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AO6" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="AP6" t="n">
-        <v>4070</v>
+        <v>3478</v>
       </c>
       <c r="AQ6" t="n">
-        <v>134</v>
+        <v>-486</v>
       </c>
       <c r="AR6" t="inlineStr">
         <is>
@@ -1327,21 +1351,21 @@
         </is>
       </c>
       <c r="AS6" t="n">
-        <v>-351</v>
+        <v>305</v>
       </c>
       <c r="AT6" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="AU6" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="AV6" t="inlineStr">
         <is>
-          <t>A+ STRUCTURE</t>
+          <t>BREAKOUT</t>
         </is>
       </c>
       <c r="AW6" t="inlineStr">
@@ -1355,88 +1379,83 @@
         </is>
       </c>
       <c r="AY6" t="n">
-        <v>2242</v>
+        <v>714</v>
       </c>
       <c r="AZ6" t="inlineStr">
         <is>
           <t>SessionDeltaSum</t>
+        </is>
+      </c>
+      <c r="BA6" t="n">
+        <v>639</v>
+      </c>
+      <c r="BB6" t="n">
+        <v>714</v>
+      </c>
+      <c r="BC6" t="n">
+        <v>15</v>
+      </c>
+      <c r="BD6" t="inlineStr">
+        <is>
+          <t>Riesgo de reversion</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>29070</v>
+        <v>29193.75</v>
       </c>
       <c r="C7" t="n">
-        <v>29122.5</v>
+        <v>29250</v>
       </c>
       <c r="D7" t="n">
-        <v>210</v>
+        <v>225</v>
       </c>
       <c r="E7" t="n">
-        <v>29074.59</v>
+        <v>29287.16</v>
       </c>
       <c r="F7" t="n">
-        <v>20</v>
+        <v>65</v>
       </c>
       <c r="G7" t="n">
-        <v>1131</v>
+        <v>3617</v>
       </c>
       <c r="H7" t="n">
-        <v>183</v>
+        <v>-71</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>normal speed</t>
+          <t>invalid speed</t>
         </is>
       </c>
       <c r="J7" t="n">
-        <v>2.48</v>
+        <v>1.1</v>
       </c>
       <c r="K7" t="n">
-        <v>8</v>
-      </c>
-      <c r="L7" t="n">
-        <v>29112.5</v>
+        <v>7</v>
       </c>
       <c r="M7" t="n">
-        <v>29127.5</v>
-      </c>
-      <c r="N7" t="n">
-        <v>29142.5</v>
-      </c>
-      <c r="O7" t="n">
-        <v>60</v>
-      </c>
-      <c r="P7" t="n">
-        <v>60</v>
-      </c>
-      <c r="Q7" t="n">
-        <v>29112.5</v>
-      </c>
-      <c r="R7" s="4" t="n">
-        <v>-60</v>
+        <v>29177.5</v>
+      </c>
+      <c r="R7" s="4" t="inlineStr">
+        <is>
+          <t>NO_PROFILE</t>
+        </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>SCALP_NORMAL</t>
-        </is>
-      </c>
-      <c r="U7" t="n">
-        <v>60</v>
-      </c>
-      <c r="V7" t="n">
-        <v>35</v>
+          <t>UNCLASSIFIED</t>
+        </is>
       </c>
       <c r="W7" t="inlineStr">
         <is>
@@ -1452,7 +1471,7 @@
         <v>2311</v>
       </c>
       <c r="Z7" t="n">
-        <v>8.072800000000001</v>
+        <v>58.8622</v>
       </c>
       <c r="AA7" t="inlineStr">
         <is>
@@ -1496,12 +1515,12 @@
       </c>
       <c r="AI7" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="AJ7" t="inlineStr">
         <is>
-          <t>SL</t>
+          <t>NO_PROFILE</t>
         </is>
       </c>
       <c r="AK7" t="inlineStr">
@@ -1518,10 +1537,10 @@
         </is>
       </c>
       <c r="AP7" t="n">
-        <v>5619</v>
+        <v>6819</v>
       </c>
       <c r="AQ7" t="n">
-        <v>211</v>
+        <v>41</v>
       </c>
       <c r="AR7" t="inlineStr">
         <is>
@@ -1529,11 +1548,11 @@
         </is>
       </c>
       <c r="AS7" t="n">
-        <v>-28</v>
+        <v>-112</v>
       </c>
       <c r="AT7" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="AU7" t="inlineStr">
@@ -1557,37 +1576,1668 @@
         </is>
       </c>
       <c r="AY7" t="n">
-        <v>1157</v>
+        <v>-993</v>
       </c>
       <c r="AZ7" t="inlineStr">
         <is>
           <t>SessionDeltaSum</t>
+        </is>
+      </c>
+      <c r="BA7" t="n">
+        <v>-993</v>
+      </c>
+      <c r="BB7" t="n">
+        <v>-993</v>
+      </c>
+      <c r="BC7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD7" t="inlineStr">
+        <is>
+          <t>Excelente</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="R8" s="4" t="n"/>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>29551.25</v>
+      </c>
+      <c r="C8" t="n">
+        <v>29620</v>
+      </c>
+      <c r="D8" t="n">
+        <v>275</v>
+      </c>
+      <c r="E8" t="n">
+        <v>29570.71</v>
+      </c>
+      <c r="F8" t="n">
+        <v>115</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1319</v>
+      </c>
+      <c r="H8" t="n">
+        <v>437</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>A+ speed</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>5.53</v>
+      </c>
+      <c r="K8" t="n">
+        <v>9</v>
+      </c>
+      <c r="M8" t="n">
+        <v>29680</v>
+      </c>
+      <c r="R8" s="4" t="inlineStr">
+        <is>
+          <t>NO_PROFILE</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>POTENTIAL_RUNNER</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-aplus-structure-export</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>09:37:00</t>
+        </is>
+      </c>
+      <c r="Y8" t="n">
+        <v>2317</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>20.7972</v>
+      </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ8" t="inlineStr">
+        <is>
+          <t>NO_PROFILE</t>
+        </is>
+      </c>
+      <c r="AK8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AN8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AP8" t="n">
+        <v>1695</v>
+      </c>
+      <c r="AQ8" t="n">
+        <v>133</v>
+      </c>
+      <c r="AR8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AS8" t="n">
+        <v>304</v>
+      </c>
+      <c r="AT8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AU8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AV8" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="AW8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AX8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AY8" t="n">
+        <v>1205</v>
+      </c>
+      <c r="AZ8" t="inlineStr">
+        <is>
+          <t>SessionDeltaSum</t>
+        </is>
+      </c>
+      <c r="BA8" t="n">
+        <v>1205</v>
+      </c>
+      <c r="BB8" t="n">
+        <v>1205</v>
+      </c>
+      <c r="BC8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD8" t="inlineStr">
+        <is>
+          <t>Excelente</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="R9" s="4" t="n"/>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>29940</v>
+      </c>
+      <c r="C9" t="n">
+        <v>29948.75</v>
+      </c>
+      <c r="D9" t="n">
+        <v>35</v>
+      </c>
+      <c r="E9" t="n">
+        <v>29958.9</v>
+      </c>
+      <c r="F9" t="n">
+        <v>15</v>
+      </c>
+      <c r="G9" t="n">
+        <v>55</v>
+      </c>
+      <c r="H9" t="n">
+        <v>37</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>normal speed</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v>2.11</v>
+      </c>
+      <c r="K9" t="n">
+        <v>5</v>
+      </c>
+      <c r="M9" t="n">
+        <v>29966.25</v>
+      </c>
+      <c r="R9" s="4" t="inlineStr">
+        <is>
+          <t>NO_PROFILE</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>SCALP_NORMAL</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-aplus-structure-export</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>09:37:00</t>
+        </is>
+      </c>
+      <c r="Y9" t="n">
+        <v>2317</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>7.1191</v>
+      </c>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AF9" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG9" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH9" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI9" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ9" t="inlineStr">
+        <is>
+          <t>NO_PROFILE</t>
+        </is>
+      </c>
+      <c r="AK9" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AN9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO9" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AP9" t="n">
+        <v>232</v>
+      </c>
+      <c r="AQ9" t="n">
+        <v>-32</v>
+      </c>
+      <c r="AR9" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AS9" t="n">
+        <v>69</v>
+      </c>
+      <c r="AT9" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AU9" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AV9" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="AW9" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AX9" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AY9" t="n">
+        <v>-44</v>
+      </c>
+      <c r="AZ9" t="inlineStr">
+        <is>
+          <t>SessionDeltaSum</t>
+        </is>
+      </c>
+      <c r="BA9" t="n">
+        <v>-44</v>
+      </c>
+      <c r="BB9" t="n">
+        <v>-44</v>
+      </c>
+      <c r="BC9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD9" t="inlineStr">
+        <is>
+          <t>Excelente</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="R10" s="4" t="n"/>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>29880</v>
+      </c>
+      <c r="C10" t="n">
+        <v>29935</v>
+      </c>
+      <c r="D10" t="n">
+        <v>220</v>
+      </c>
+      <c r="E10" t="n">
+        <v>29859.58</v>
+      </c>
+      <c r="F10" t="n">
+        <v>65</v>
+      </c>
+      <c r="G10" t="n">
+        <v>907</v>
+      </c>
+      <c r="H10" t="n">
+        <v>-95</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>A+ speed</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>5.03</v>
+      </c>
+      <c r="K10" t="n">
+        <v>8</v>
+      </c>
+      <c r="L10" t="n">
+        <v>29852.5</v>
+      </c>
+      <c r="M10" t="n">
+        <v>29837.5</v>
+      </c>
+      <c r="N10" t="n">
+        <v>29822.5</v>
+      </c>
+      <c r="O10" t="n">
+        <v>60</v>
+      </c>
+      <c r="P10" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>29852.5</v>
+      </c>
+      <c r="R10" s="4" t="n">
+        <v>-60</v>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>POTENTIAL_RUNNER</t>
+        </is>
+      </c>
+      <c r="U10" t="n">
+        <v>60</v>
+      </c>
+      <c r="V10" t="n">
+        <v>40</v>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-aplus-structure-export</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>09:35:00</t>
+        </is>
+      </c>
+      <c r="Y10" t="n">
+        <v>2075</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>12.9344</v>
+      </c>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE10" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF10" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG10" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH10" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI10" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ10" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="AK10" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AN10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO10" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AP10" t="n">
+        <v>2999</v>
+      </c>
+      <c r="AQ10" t="n">
+        <v>-267</v>
+      </c>
+      <c r="AR10" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AS10" t="n">
+        <v>172</v>
+      </c>
+      <c r="AT10" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AU10" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AV10" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="AW10" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AX10" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AY10" t="n">
+        <v>32</v>
+      </c>
+      <c r="AZ10" t="inlineStr">
+        <is>
+          <t>SessionDeltaSum</t>
+        </is>
+      </c>
+      <c r="BA10" t="n">
+        <v>-213</v>
+      </c>
+      <c r="BB10" t="n">
+        <v>32</v>
+      </c>
+      <c r="BC10" t="n">
+        <v>2.78</v>
+      </c>
+      <c r="BD10" t="inlineStr">
+        <is>
+          <t>Riesgo de reversion</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="R11" s="4" t="n"/>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>30133.75</v>
+      </c>
+      <c r="C11" t="n">
+        <v>30192.5</v>
+      </c>
+      <c r="D11" t="n">
+        <v>235</v>
+      </c>
+      <c r="E11" t="n">
+        <v>30205.97</v>
+      </c>
+      <c r="F11" t="n">
+        <v>90</v>
+      </c>
+      <c r="G11" t="n">
+        <v>3218</v>
+      </c>
+      <c r="H11" t="n">
+        <v>-986</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>normal speed</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="K11" t="n">
+        <v>8</v>
+      </c>
+      <c r="L11" t="n">
+        <v>30126.25</v>
+      </c>
+      <c r="M11" t="n">
+        <v>30111.25</v>
+      </c>
+      <c r="N11" t="n">
+        <v>30096.25</v>
+      </c>
+      <c r="O11" t="n">
+        <v>60</v>
+      </c>
+      <c r="P11" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>30126.25</v>
+      </c>
+      <c r="R11" s="4" t="n">
+        <v>-60</v>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>SCALP_NORMAL</t>
+        </is>
+      </c>
+      <c r="U11" t="n">
+        <v>60</v>
+      </c>
+      <c r="V11" t="n">
+        <v>25</v>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-aplus-structure-export</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>09:35:00</t>
+        </is>
+      </c>
+      <c r="Y11" t="n">
+        <v>2315</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>39.9795</v>
+      </c>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE11" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF11" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG11" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH11" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI11" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ11" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="AK11" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AN11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO11" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AP11" t="n">
+        <v>2162</v>
+      </c>
+      <c r="AQ11" t="n">
+        <v>-116</v>
+      </c>
+      <c r="AR11" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AS11" t="n">
+        <v>-870</v>
+      </c>
+      <c r="AT11" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AU11" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AV11" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="AW11" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AX11" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AY11" t="n">
+        <v>-2475</v>
+      </c>
+      <c r="AZ11" t="inlineStr">
+        <is>
+          <t>SessionDeltaSum</t>
+        </is>
+      </c>
+      <c r="BA11" t="n">
+        <v>-2658</v>
+      </c>
+      <c r="BB11" t="n">
+        <v>-2475</v>
+      </c>
+      <c r="BC11" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="BD11" t="inlineStr">
+        <is>
+          <t>Riesgo de reversion</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="R12" s="4" t="n"/>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>30052.5</v>
+      </c>
+      <c r="C12" t="n">
+        <v>30107.5</v>
+      </c>
+      <c r="D12" t="n">
+        <v>220</v>
+      </c>
+      <c r="E12" t="n">
+        <v>29947.54</v>
+      </c>
+      <c r="F12" t="n">
+        <v>10</v>
+      </c>
+      <c r="G12" t="n">
+        <v>1996</v>
+      </c>
+      <c r="H12" t="n">
+        <v>196</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>invalid speed</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="K12" t="n">
+        <v>7</v>
+      </c>
+      <c r="M12" t="n">
+        <v>30110</v>
+      </c>
+      <c r="R12" s="4" t="inlineStr">
+        <is>
+          <t>NO_PROFILE</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>UNCLASSIFIED</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-aplus-structure-export</t>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>09:31:00</t>
+        </is>
+      </c>
+      <c r="Y12" t="n">
+        <v>2311</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>33.384</v>
+      </c>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AB12" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE12" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF12" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG12" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH12" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI12" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AJ12" t="inlineStr">
+        <is>
+          <t>NO_PROFILE</t>
+        </is>
+      </c>
+      <c r="AK12" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AN12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO12" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AP12" t="n">
+        <v>6970</v>
+      </c>
+      <c r="AQ12" t="n">
+        <v>426</v>
+      </c>
+      <c r="AR12" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AS12" t="n">
+        <v>-230</v>
+      </c>
+      <c r="AT12" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AU12" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AV12" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="AW12" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AX12" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AY12" t="n">
+        <v>1139</v>
+      </c>
+      <c r="AZ12" t="inlineStr">
+        <is>
+          <t>SessionDeltaSum</t>
+        </is>
+      </c>
+      <c r="BA12" t="n">
+        <v>1139</v>
+      </c>
+      <c r="BB12" t="n">
+        <v>1139</v>
+      </c>
+      <c r="BC12" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD12" t="inlineStr">
+        <is>
+          <t>Excelente</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="R13" s="4" t="n"/>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>30365</v>
+      </c>
+      <c r="C13" t="n">
+        <v>30405</v>
+      </c>
+      <c r="D13" t="n">
+        <v>160</v>
+      </c>
+      <c r="E13" t="n">
+        <v>30336.94</v>
+      </c>
+      <c r="F13" t="n">
+        <v>30</v>
+      </c>
+      <c r="G13" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H13" t="n">
+        <v>492</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>A+ speed</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>6.13</v>
+      </c>
+      <c r="K13" t="n">
+        <v>11</v>
+      </c>
+      <c r="L13" t="n">
+        <v>30438.75</v>
+      </c>
+      <c r="M13" t="n">
+        <v>30423.75</v>
+      </c>
+      <c r="N13" t="n">
+        <v>30408.75</v>
+      </c>
+      <c r="O13" t="n">
+        <v>60</v>
+      </c>
+      <c r="P13" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>30408.75</v>
+      </c>
+      <c r="R13" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>POTENTIAL_RUNNER</t>
+        </is>
+      </c>
+      <c r="U13" t="n">
+        <v>0</v>
+      </c>
+      <c r="V13" t="n">
+        <v>60</v>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-aplus-structure-export</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>09:32:00</t>
+        </is>
+      </c>
+      <c r="Y13" t="n">
+        <v>2312</v>
+      </c>
+      <c r="Z13" t="n">
+        <v>4.8927</v>
+      </c>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AB13" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE13" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF13" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG13" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH13" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI13" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ13" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="AK13" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AL13" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="AM13" t="n">
+        <v>30425</v>
+      </c>
+      <c r="AN13" t="n">
+        <v>3</v>
+      </c>
+      <c r="AO13" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AP13" t="n">
+        <v>3724</v>
+      </c>
+      <c r="AQ13" t="n">
+        <v>166</v>
+      </c>
+      <c r="AR13" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AS13" t="n">
+        <v>326</v>
+      </c>
+      <c r="AT13" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AU13" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AV13" t="inlineStr">
+        <is>
+          <t>A+ ABSORTION</t>
+        </is>
+      </c>
+      <c r="AW13" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AX13" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AY13" t="n">
+        <v>2920</v>
+      </c>
+      <c r="AZ13" t="inlineStr">
+        <is>
+          <t>SessionDeltaSum</t>
+        </is>
+      </c>
+      <c r="BA13" t="n">
+        <v>2916</v>
+      </c>
+      <c r="BB13" t="n">
+        <v>2920</v>
+      </c>
+      <c r="BC13" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="BD13" t="inlineStr">
+        <is>
+          <t>Excelente</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="R14" s="4" t="n"/>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>30311.25</v>
+      </c>
+      <c r="C14" t="n">
+        <v>30370</v>
+      </c>
+      <c r="D14" t="n">
+        <v>235</v>
+      </c>
+      <c r="E14" t="n">
+        <v>30440.72</v>
+      </c>
+      <c r="F14" t="n">
+        <v>95</v>
+      </c>
+      <c r="G14" t="n">
+        <v>1793</v>
+      </c>
+      <c r="H14" t="n">
+        <v>179</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>normal speed</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="K14" t="n">
+        <v>8</v>
+      </c>
+      <c r="M14" t="n">
+        <v>30443.75</v>
+      </c>
+      <c r="R14" s="4" t="inlineStr">
+        <is>
+          <t>NO_PROFILE</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>SCALP_NORMAL</t>
+        </is>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-aplus-structure-export</t>
+        </is>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>09:37:00</t>
+        </is>
+      </c>
+      <c r="Y14" t="n">
+        <v>2317</v>
+      </c>
+      <c r="Z14" t="n">
+        <v>44.7</v>
+      </c>
+      <c r="AA14" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AB14" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE14" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF14" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG14" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH14" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI14" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ14" t="inlineStr">
+        <is>
+          <t>NO_PROFILE</t>
+        </is>
+      </c>
+      <c r="AK14" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AN14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO14" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AP14" t="n">
+        <v>3604</v>
+      </c>
+      <c r="AQ14" t="n">
+        <v>-250</v>
+      </c>
+      <c r="AR14" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AS14" t="n">
+        <v>429</v>
+      </c>
+      <c r="AT14" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AU14" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AV14" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="AW14" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AX14" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AY14" t="n">
+        <v>-115</v>
+      </c>
+      <c r="AZ14" t="inlineStr">
+        <is>
+          <t>SessionDeltaSum</t>
+        </is>
+      </c>
+      <c r="BA14" t="n">
+        <v>-115</v>
+      </c>
+      <c r="BB14" t="n">
+        <v>-115</v>
+      </c>
+      <c r="BC14" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD14" t="inlineStr">
+        <is>
+          <t>Excelente</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="R15" s="4" t="n"/>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>30497.5</v>
+      </c>
+      <c r="C15" t="n">
+        <v>30568.75</v>
+      </c>
+      <c r="D15" t="n">
+        <v>285</v>
+      </c>
+      <c r="E15" t="n">
+        <v>30515.37</v>
+      </c>
+      <c r="F15" t="n">
+        <v>55</v>
+      </c>
+      <c r="G15" t="n">
+        <v>1210</v>
+      </c>
+      <c r="H15" t="n">
+        <v>-372</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>normal speed</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>2.29</v>
+      </c>
+      <c r="K15" t="n">
+        <v>8</v>
+      </c>
+      <c r="M15" t="n">
+        <v>30473.75</v>
+      </c>
+      <c r="R15" s="4" t="inlineStr">
+        <is>
+          <t>NO_PROFILE</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>SCALP_NORMAL</t>
+        </is>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-aplus-structure-export</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>09:34:00</t>
+        </is>
+      </c>
+      <c r="Y15" t="n">
+        <v>2314</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>23.9661</v>
+      </c>
+      <c r="AA15" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AB15" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AC15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AG15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AH15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AJ15" t="inlineStr">
+        <is>
+          <t>NO_PROFILE</t>
+        </is>
+      </c>
+      <c r="AK15" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AN15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO15" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AP15" t="n">
+        <v>2104</v>
+      </c>
+      <c r="AQ15" t="n">
+        <v>48</v>
+      </c>
+      <c r="AR15" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AS15" t="n">
+        <v>-420</v>
+      </c>
+      <c r="AT15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AU15" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AV15" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="AW15" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AX15" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AY15" t="n">
+        <v>1988</v>
+      </c>
+      <c r="AZ15" t="inlineStr">
+        <is>
+          <t>SessionDeltaSum</t>
+        </is>
+      </c>
+      <c r="BA15" t="n">
+        <v>1988</v>
+      </c>
+      <c r="BB15" t="n">
+        <v>1988</v>
+      </c>
+      <c r="BC15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD15" t="inlineStr">
+        <is>
+          <t>Excelente</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="R16" s="4" t="n"/>

</xml_diff>

<commit_message>
A+ SPEED diferencia de A+ ABSORTION fechas 27-05-2026-2026
</commit_message>
<xml_diff>
--- a/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
+++ b/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AZ25"/>
+  <dimension ref="A1:BD25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -463,11 +463,11 @@
     </row>
     <row r="2">
       <c r="A2" s="1">
-        <f>IF((COUNTIF(R4:R7,"&gt;0")+COUNTIF(R4:R7,"&lt;0"))=0,"",COUNTIF(R4:R7,"&gt;0")/(COUNTIF(R4:R7,"&gt;0")+COUNTIF(R4:R7,"&lt;0")))</f>
+        <f>IF((COUNTIF(R4:R5,"&gt;0")+COUNTIF(R4:R5,"&lt;0"))=0,"",COUNTIF(R4:R5,"&gt;0")/(COUNTIF(R4:R5,"&gt;0")+COUNTIF(R4:R5,"&lt;0")))</f>
         <v/>
       </c>
       <c r="B2" s="2">
-        <f>IF(ABS(SUMIF(R4:R7,"&lt;0",R4:R7))=0,IF(SUMIF(R4:R7,"&gt;0",R4:R7)&gt;0,"INF",""),SUMIF(R4:R7,"&gt;0",R4:R7)/ABS(SUMIF(R4:R7,"&lt;0",R4:R7)))</f>
+        <f>IF(ABS(SUMIF(R4:R5,"&lt;0",R4:R5))=0,IF(SUMIF(R4:R5,"&gt;0",R4:R5)&gt;0,"INF",""),SUMIF(R4:R5,"&gt;0",R4:R5)/ABS(SUMIF(R4:R5,"&lt;0",R4:R5)))</f>
         <v/>
       </c>
     </row>
@@ -732,33 +732,53 @@
           <t>Cumulative_Delta_Source</t>
         </is>
       </c>
+      <c r="BA3" s="3" t="inlineStr">
+        <is>
+          <t>Cvd_Peak</t>
+        </is>
+      </c>
+      <c r="BB3" s="3" t="inlineStr">
+        <is>
+          <t>Cvd_Current</t>
+        </is>
+      </c>
+      <c r="BC3" s="3" t="inlineStr">
+        <is>
+          <t>Cvd_Pullback_Pct</t>
+        </is>
+      </c>
+      <c r="BD3" s="3" t="inlineStr">
+        <is>
+          <t>Cvd_Pullback_Label</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>28860</v>
+        <v>30133.75</v>
       </c>
       <c r="C4" t="n">
-        <v>28903.75</v>
+        <v>30192.5</v>
       </c>
       <c r="D4" t="n">
-        <v>175</v>
+        <v>235</v>
       </c>
       <c r="E4" t="n">
-        <v>28876.34</v>
+        <v>30206.02</v>
       </c>
       <c r="F4" t="n">
-        <v>10</v>
+        <v>85</v>
       </c>
       <c r="G4" t="n">
-        <v>1035</v>
+        <v>3179</v>
       </c>
       <c r="H4" t="n">
-        <v>55</v>
+        <v>-971</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -766,35 +786,35 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>0.65</v>
+        <v>2.13</v>
       </c>
       <c r="K4" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="L4" t="n">
-        <v>28891.25</v>
+        <v>30133.75</v>
       </c>
       <c r="M4" t="n">
-        <v>28906.25</v>
+        <v>30112.5</v>
       </c>
       <c r="N4" t="n">
-        <v>28921.25</v>
+        <v>30091.25</v>
       </c>
       <c r="O4" t="n">
-        <v>60</v>
+        <v>85</v>
       </c>
       <c r="P4" t="n">
-        <v>60</v>
+        <v>85</v>
       </c>
       <c r="Q4" t="n">
-        <v>28921.25</v>
+        <v>30091.25</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>60</v>
+        <v>85</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -803,10 +823,10 @@
         </is>
       </c>
       <c r="U4" t="n">
-        <v>10</v>
+        <v>75</v>
       </c>
       <c r="V4" t="n">
-        <v>60</v>
+        <v>85</v>
       </c>
       <c r="W4" t="inlineStr">
         <is>
@@ -815,14 +835,14 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>09:31:00</t>
+          <t>09:35:00</t>
         </is>
       </c>
       <c r="Y4" t="n">
-        <v>2311</v>
+        <v>2315</v>
       </c>
       <c r="Z4" t="n">
-        <v>15.3696</v>
+        <v>39.9452</v>
       </c>
       <c r="AA4" t="inlineStr">
         <is>
@@ -831,7 +851,7 @@
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>A+ ABSORTION</t>
+          <t>LastTime</t>
         </is>
       </c>
       <c r="AC4" t="inlineStr">
@@ -876,119 +896,125 @@
       </c>
       <c r="AK4" t="inlineStr">
         <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AL4" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="AM4" t="n">
-        <v>28906.25</v>
+          <t>FALSE</t>
+        </is>
       </c>
       <c r="AN4" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AO4" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="AP4" t="n">
-        <v>4730</v>
+        <v>2162</v>
       </c>
       <c r="AQ4" t="n">
-        <v>170</v>
+        <v>-116</v>
       </c>
       <c r="AR4" t="inlineStr">
         <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AS4" t="n">
+        <v>-855</v>
+      </c>
+      <c r="AT4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AU4" t="inlineStr">
+        <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="AS4" t="n">
-        <v>-115</v>
-      </c>
-      <c r="AT4" t="inlineStr">
+      <c r="AV4" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="AW4" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="AU4" t="inlineStr">
+      <c r="AX4" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="AV4" t="inlineStr">
-        <is>
-          <t>A+ ABSORTION</t>
-        </is>
-      </c>
-      <c r="AW4" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AX4" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
       <c r="AY4" t="n">
-        <v>1381</v>
+        <v>-2787</v>
       </c>
       <c r="AZ4" t="inlineStr">
         <is>
           <t>SessionDeltaSum</t>
+        </is>
+      </c>
+      <c r="BA4" t="n">
+        <v>-2787</v>
+      </c>
+      <c r="BB4" t="n">
+        <v>-2787</v>
+      </c>
+      <c r="BC4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD4" t="inlineStr">
+        <is>
+          <t>Excelente</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>29146.25</v>
+        <v>30365</v>
       </c>
       <c r="C5" t="n">
-        <v>29227.5</v>
+        <v>30405</v>
       </c>
       <c r="D5" t="n">
-        <v>325</v>
+        <v>160</v>
       </c>
       <c r="E5" t="n">
-        <v>29203.49</v>
+        <v>30336.94</v>
       </c>
       <c r="F5" t="n">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="G5" t="n">
-        <v>2827</v>
+        <v>1000</v>
       </c>
       <c r="H5" t="n">
-        <v>-245</v>
+        <v>492</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>normal speed</t>
+          <t>A+ speed</t>
         </is>
       </c>
       <c r="J5" t="n">
-        <v>0.09</v>
+        <v>6.13</v>
       </c>
       <c r="K5" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="L5" t="n">
-        <v>29160</v>
+        <v>30438.75</v>
       </c>
       <c r="M5" t="n">
-        <v>29145</v>
+        <v>30423.75</v>
       </c>
       <c r="N5" t="n">
-        <v>29130</v>
+        <v>30408.75</v>
       </c>
       <c r="O5" t="n">
         <v>60</v>
@@ -997,10 +1023,10 @@
         <v>60</v>
       </c>
       <c r="Q5" t="n">
-        <v>29160</v>
+        <v>30408.75</v>
       </c>
       <c r="R5" s="4" t="n">
-        <v>-60</v>
+        <v>60</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
@@ -1009,15 +1035,15 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>SCALP_NORMAL</t>
+          <t>POTENTIAL_RUNNER</t>
         </is>
       </c>
       <c r="U5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V5" t="n">
         <v>60</v>
       </c>
-      <c r="V5" t="n">
-        <v>0</v>
-      </c>
       <c r="W5" t="inlineStr">
         <is>
           <t>score-exporter-2026-05-30-aplus-structure-export</t>
@@ -1025,14 +1051,14 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>09:35:00</t>
+          <t>09:32:00</t>
         </is>
       </c>
       <c r="Y5" t="n">
-        <v>2315</v>
+        <v>2312</v>
       </c>
       <c r="Z5" t="n">
-        <v>56.9984</v>
+        <v>4.8927</v>
       </c>
       <c r="AA5" t="inlineStr">
         <is>
@@ -1041,7 +1067,7 @@
       </c>
       <c r="AB5" t="inlineStr">
         <is>
-          <t>A+ STRUCTURE</t>
+          <t>LastTime</t>
         </is>
       </c>
       <c r="AC5" t="inlineStr">
@@ -1051,7 +1077,7 @@
       </c>
       <c r="AD5" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="AE5" t="inlineStr">
@@ -1081,7 +1107,7 @@
       </c>
       <c r="AJ5" t="inlineStr">
         <is>
-          <t>SL</t>
+          <t>TP</t>
         </is>
       </c>
       <c r="AK5" t="inlineStr">
@@ -1091,33 +1117,33 @@
       </c>
       <c r="AL5" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="AM5" t="n">
-        <v>29146.25</v>
+        <v>30425</v>
       </c>
       <c r="AN5" t="n">
         <v>3</v>
       </c>
       <c r="AO5" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="AP5" t="n">
-        <v>2738</v>
+        <v>3724</v>
       </c>
       <c r="AQ5" t="n">
-        <v>52</v>
+        <v>166</v>
       </c>
       <c r="AR5" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="AS5" t="n">
-        <v>-297</v>
+        <v>326</v>
       </c>
       <c r="AT5" t="inlineStr">
         <is>
@@ -1126,444 +1152,52 @@
       </c>
       <c r="AU5" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="AV5" t="inlineStr">
         <is>
-          <t>A+ STRUCTURE</t>
+          <t>A+ ABSORTION</t>
         </is>
       </c>
       <c r="AW5" t="inlineStr">
         <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="AX5" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
       <c r="AY5" t="n">
-        <v>-1836</v>
+        <v>2920</v>
       </c>
       <c r="AZ5" t="inlineStr">
         <is>
           <t>SessionDeltaSum</t>
         </is>
       </c>
+      <c r="BA5" t="n">
+        <v>2917</v>
+      </c>
+      <c r="BB5" t="n">
+        <v>2920</v>
+      </c>
+      <c r="BC5" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="BD5" t="inlineStr">
+        <is>
+          <t>Excelente</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2026-05-18</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>29305</v>
-      </c>
-      <c r="C6" t="n">
-        <v>29356.25</v>
-      </c>
-      <c r="D6" t="n">
-        <v>205</v>
-      </c>
-      <c r="E6" t="n">
-        <v>29211.08</v>
-      </c>
-      <c r="F6" t="n">
-        <v>50</v>
-      </c>
-      <c r="G6" t="n">
-        <v>2599</v>
-      </c>
-      <c r="H6" t="n">
-        <v>-217</v>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>normal speed</t>
-        </is>
-      </c>
-      <c r="J6" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="K6" t="n">
-        <v>8</v>
-      </c>
-      <c r="L6" t="n">
-        <v>29307.5</v>
-      </c>
-      <c r="M6" t="n">
-        <v>29292.5</v>
-      </c>
-      <c r="N6" t="n">
-        <v>29277.5</v>
-      </c>
-      <c r="O6" t="n">
-        <v>60</v>
-      </c>
-      <c r="P6" t="n">
-        <v>60</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>29277.5</v>
-      </c>
-      <c r="R6" s="4" t="n">
-        <v>60</v>
-      </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="T6" t="inlineStr">
-        <is>
-          <t>SCALP_NORMAL</t>
-        </is>
-      </c>
-      <c r="U6" t="n">
-        <v>45</v>
-      </c>
-      <c r="V6" t="n">
-        <v>65</v>
-      </c>
-      <c r="W6" t="inlineStr">
-        <is>
-          <t>score-exporter-2026-05-30-aplus-structure-export</t>
-        </is>
-      </c>
-      <c r="X6" t="inlineStr">
-        <is>
-          <t>09:32:00</t>
-        </is>
-      </c>
-      <c r="Y6" t="n">
-        <v>2312</v>
-      </c>
-      <c r="Z6" t="n">
-        <v>45.6277</v>
-      </c>
-      <c r="AA6" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AB6" t="inlineStr">
-        <is>
-          <t>A+ STRUCTURE</t>
-        </is>
-      </c>
-      <c r="AC6" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AD6" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AE6" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AF6" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AG6" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AH6" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AI6" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AJ6" t="inlineStr">
-        <is>
-          <t>TP</t>
-        </is>
-      </c>
-      <c r="AK6" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AL6" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="AM6" t="n">
-        <v>29295</v>
-      </c>
-      <c r="AN6" t="n">
-        <v>3</v>
-      </c>
-      <c r="AO6" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AP6" t="n">
-        <v>4070</v>
-      </c>
-      <c r="AQ6" t="n">
-        <v>134</v>
-      </c>
-      <c r="AR6" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AS6" t="n">
-        <v>-351</v>
-      </c>
-      <c r="AT6" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AU6" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AV6" t="inlineStr">
-        <is>
-          <t>A+ STRUCTURE</t>
-        </is>
-      </c>
-      <c r="AW6" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AX6" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AY6" t="n">
-        <v>2242</v>
-      </c>
-      <c r="AZ6" t="inlineStr">
-        <is>
-          <t>SessionDeltaSum</t>
-        </is>
-      </c>
+      <c r="R6" s="4" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2026-05-20</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>29070</v>
-      </c>
-      <c r="C7" t="n">
-        <v>29122.5</v>
-      </c>
-      <c r="D7" t="n">
-        <v>210</v>
-      </c>
-      <c r="E7" t="n">
-        <v>29074.59</v>
-      </c>
-      <c r="F7" t="n">
-        <v>20</v>
-      </c>
-      <c r="G7" t="n">
-        <v>1131</v>
-      </c>
-      <c r="H7" t="n">
-        <v>183</v>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>normal speed</t>
-        </is>
-      </c>
-      <c r="J7" t="n">
-        <v>2.48</v>
-      </c>
-      <c r="K7" t="n">
-        <v>8</v>
-      </c>
-      <c r="L7" t="n">
-        <v>29112.5</v>
-      </c>
-      <c r="M7" t="n">
-        <v>29127.5</v>
-      </c>
-      <c r="N7" t="n">
-        <v>29142.5</v>
-      </c>
-      <c r="O7" t="n">
-        <v>60</v>
-      </c>
-      <c r="P7" t="n">
-        <v>60</v>
-      </c>
-      <c r="Q7" t="n">
-        <v>29112.5</v>
-      </c>
-      <c r="R7" s="4" t="n">
-        <v>-60</v>
-      </c>
-      <c r="S7" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="T7" t="inlineStr">
-        <is>
-          <t>SCALP_NORMAL</t>
-        </is>
-      </c>
-      <c r="U7" t="n">
-        <v>60</v>
-      </c>
-      <c r="V7" t="n">
-        <v>35</v>
-      </c>
-      <c r="W7" t="inlineStr">
-        <is>
-          <t>score-exporter-2026-05-30-aplus-structure-export</t>
-        </is>
-      </c>
-      <c r="X7" t="inlineStr">
-        <is>
-          <t>09:31:00</t>
-        </is>
-      </c>
-      <c r="Y7" t="n">
-        <v>2311</v>
-      </c>
-      <c r="Z7" t="n">
-        <v>8.072800000000001</v>
-      </c>
-      <c r="AA7" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AB7" t="inlineStr">
-        <is>
-          <t>LastTime</t>
-        </is>
-      </c>
-      <c r="AC7" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AD7" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AE7" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AF7" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AG7" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AH7" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AI7" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AJ7" t="inlineStr">
-        <is>
-          <t>SL</t>
-        </is>
-      </c>
-      <c r="AK7" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AN7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO7" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AP7" t="n">
-        <v>5619</v>
-      </c>
-      <c r="AQ7" t="n">
-        <v>211</v>
-      </c>
-      <c r="AR7" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AS7" t="n">
-        <v>-28</v>
-      </c>
-      <c r="AT7" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AU7" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AV7" t="inlineStr">
-        <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="AW7" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AX7" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AY7" t="n">
-        <v>1157</v>
-      </c>
-      <c r="AZ7" t="inlineStr">
-        <is>
-          <t>SessionDeltaSum</t>
-        </is>
-      </c>
+      <c r="R7" s="4" t="n"/>
     </row>
     <row r="8">
       <c r="R8" s="4" t="n"/>

</xml_diff>

<commit_message>
Linea EXIT al 50% si hay CVD risk
</commit_message>
<xml_diff>
--- a/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
+++ b/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BD5"/>
+  <dimension ref="A1:BD7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -463,11 +463,11 @@
     </row>
     <row r="2">
       <c r="A2" s="1">
-        <f>IF((COUNTIF(R4:R5,"&gt;0")+COUNTIF(R4:R5,"&lt;0"))=0,"",COUNTIF(R4:R5,"&gt;0")/(COUNTIF(R4:R5,"&gt;0")+COUNTIF(R4:R5,"&lt;0")))</f>
+        <f>IF((COUNTIF(R4:R7,"&gt;0")+COUNTIF(R4:R7,"&lt;0"))=0,"",COUNTIF(R4:R7,"&gt;0")/(COUNTIF(R4:R7,"&gt;0")+COUNTIF(R4:R7,"&lt;0")))</f>
         <v/>
       </c>
       <c r="B2" s="2">
-        <f>IF(ABS(SUMIF(R4:R5,"&lt;0",R4:R5))=0,IF(SUMIF(R4:R5,"&gt;0",R4:R5)&gt;0,"INF",""),SUMIF(R4:R5,"&gt;0",R4:R5)/ABS(SUMIF(R4:R5,"&lt;0",R4:R5)))</f>
+        <f>IF(ABS(SUMIF(R4:R7,"&lt;0",R4:R7))=0,IF(SUMIF(R4:R7,"&gt;0",R4:R7)&gt;0,"INF",""),SUMIF(R4:R7,"&gt;0",R4:R7)/ABS(SUMIF(R4:R7,"&lt;0",R4:R7)))</f>
         <v/>
       </c>
     </row>
@@ -807,10 +807,10 @@
         <v>50</v>
       </c>
       <c r="Q4" t="n">
-        <v>29525</v>
+        <v>29510</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
@@ -823,10 +823,10 @@
         </is>
       </c>
       <c r="U4" t="n">
+        <v>10</v>
+      </c>
+      <c r="V4" t="n">
         <v>0</v>
-      </c>
-      <c r="V4" t="n">
-        <v>70</v>
       </c>
       <c r="W4" t="inlineStr">
         <is>
@@ -842,7 +842,7 @@
         <v>2312</v>
       </c>
       <c r="Z4" t="n">
-        <v>-1877</v>
+        <v>-2026</v>
       </c>
       <c r="AA4" t="inlineStr">
         <is>
@@ -850,17 +850,17 @@
         </is>
       </c>
       <c r="AB4" t="n">
-        <v>-1877</v>
+        <v>-2020</v>
       </c>
       <c r="AC4" t="n">
-        <v>-1877</v>
+        <v>-2026</v>
       </c>
       <c r="AD4" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AE4" t="inlineStr">
         <is>
-          <t>Excelente</t>
+          <t>Riesgo de reversion</t>
         </is>
       </c>
       <c r="AF4" t="n">
@@ -942,7 +942,7 @@
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>EXIT</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
@@ -975,213 +975,33 @@
           <t>2026-05-15</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>29241.25</v>
-      </c>
-      <c r="C5" t="n">
-        <v>29291.25</v>
-      </c>
-      <c r="D5" t="n">
-        <v>200</v>
-      </c>
-      <c r="E5" t="n">
-        <v>29294.78</v>
-      </c>
-      <c r="F5" t="n">
-        <v>75</v>
-      </c>
-      <c r="G5" t="n">
-        <v>833</v>
-      </c>
-      <c r="H5" t="n">
-        <v>-349</v>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>A+ speed</t>
-        </is>
-      </c>
-      <c r="J5" t="n">
-        <v>14.2</v>
-      </c>
-      <c r="K5" t="n">
-        <v>8</v>
-      </c>
-      <c r="L5" t="n">
-        <v>29252.5</v>
-      </c>
-      <c r="M5" t="n">
-        <v>29222.5</v>
-      </c>
-      <c r="N5" t="n">
-        <v>29192.5</v>
-      </c>
-      <c r="O5" t="n">
-        <v>120</v>
-      </c>
-      <c r="P5" t="n">
-        <v>120</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>29252.5</v>
-      </c>
-      <c r="R5" s="4" t="n">
-        <v>-120</v>
-      </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>POTENTIAL_RUNNER</t>
-        </is>
-      </c>
-      <c r="U5" t="n">
-        <v>125</v>
-      </c>
-      <c r="V5" t="n">
-        <v>75</v>
-      </c>
-      <c r="W5" t="inlineStr">
-        <is>
-          <t>score-exporter-2026-05-30-aplus-structure-export</t>
-        </is>
-      </c>
-      <c r="X5" t="inlineStr">
-        <is>
-          <t>09:31:00</t>
-        </is>
-      </c>
-      <c r="Y5" t="n">
-        <v>2311</v>
-      </c>
-      <c r="Z5" t="n">
-        <v>-1779</v>
-      </c>
-      <c r="AA5" t="inlineStr">
-        <is>
-          <t>SessionDeltaSum</t>
-        </is>
-      </c>
-      <c r="AB5" t="n">
-        <v>-2026</v>
-      </c>
-      <c r="AC5" t="n">
-        <v>-1779</v>
-      </c>
-      <c r="AD5" t="n">
-        <v>1.93</v>
-      </c>
-      <c r="AE5" t="inlineStr">
-        <is>
-          <t>Riesgo de reversion</t>
-        </is>
-      </c>
-      <c r="AF5" t="n">
-        <v>7150</v>
-      </c>
-      <c r="AG5" t="n">
-        <v>136</v>
-      </c>
-      <c r="AH5" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AI5" t="n">
-        <v>-485</v>
-      </c>
-      <c r="AJ5" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AK5" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AL5" t="n">
-        <v>5.2831</v>
-      </c>
-      <c r="AM5" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AN5" t="inlineStr">
-        <is>
-          <t>LastTime</t>
-        </is>
-      </c>
-      <c r="AO5" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AP5" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AQ5" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AR5" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AS5" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AT5" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AU5" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AV5" t="inlineStr">
-        <is>
-          <t>BREAKOUT</t>
-        </is>
-      </c>
-      <c r="AW5" t="inlineStr">
-        <is>
-          <t>SL</t>
-        </is>
-      </c>
-      <c r="AX5" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AY5" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AZ5" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="BC5" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD5" t="inlineStr">
-        <is>
-          <t>FALSE</t>
+      <c r="R5" s="4" t="inlineStr">
+        <is>
+          <t>NO_CSV</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="R6" s="4" t="inlineStr">
+        <is>
+          <t>NO_CSV</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="R7" s="4" t="inlineStr">
+        <is>
+          <t>NO_CSV</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Imprime correctamente los segundos de la entrada al trade
</commit_message>
<xml_diff>
--- a/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
+++ b/EddiewareOpeningRangeSetup/EddiewareOpeningRangeSetup/Score_indicator_results_updated.xlsx
@@ -56,12 +56,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -427,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BD7"/>
+  <dimension ref="A1:BE27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -447,6 +449,8 @@
     <col width="10" customWidth="1" min="15" max="15"/>
     <col width="10" customWidth="1" min="16" max="16"/>
     <col width="10" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="24" max="24"/>
+    <col width="14" customWidth="1" min="57" max="57"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -752,6 +756,11 @@
           <t>Speed_Ignored_By_Structure</t>
         </is>
       </c>
+      <c r="BE3" s="3" t="inlineStr">
+        <is>
+          <t>EntrySecond_NY</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -807,10 +816,10 @@
         <v>50</v>
       </c>
       <c r="Q4" t="n">
-        <v>29510</v>
+        <v>29525</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
@@ -823,26 +832,26 @@
         </is>
       </c>
       <c r="U4" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="V4" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="W4" t="inlineStr">
         <is>
           <t>score-exporter-2026-05-30-aplus-structure-export</t>
         </is>
       </c>
-      <c r="X4" t="inlineStr">
-        <is>
-          <t>09:32:00</t>
+      <c r="X4" s="5" t="inlineStr">
+        <is>
+          <t>09:32:06</t>
         </is>
       </c>
       <c r="Y4" t="n">
         <v>2312</v>
       </c>
       <c r="Z4" t="n">
-        <v>-2026</v>
+        <v>-1934</v>
       </c>
       <c r="AA4" t="inlineStr">
         <is>
@@ -850,17 +859,17 @@
         </is>
       </c>
       <c r="AB4" t="n">
-        <v>-2020</v>
+        <v>-1934</v>
       </c>
       <c r="AC4" t="n">
-        <v>-2026</v>
+        <v>-1934</v>
       </c>
       <c r="AD4" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AE4" t="inlineStr">
         <is>
-          <t>Riesgo de reversion</t>
+          <t>Excelente</t>
         </is>
       </c>
       <c r="AF4" t="n">
@@ -942,7 +951,7 @@
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>EXIT</t>
+          <t>TP</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
@@ -968,6 +977,9 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="BE4" s="6" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -975,10 +987,217 @@
           <t>2026-05-15</t>
         </is>
       </c>
-      <c r="R5" s="4" t="inlineStr">
-        <is>
-          <t>NO_CSV</t>
-        </is>
+      <c r="B5" t="n">
+        <v>29241.25</v>
+      </c>
+      <c r="C5" t="n">
+        <v>29291.25</v>
+      </c>
+      <c r="D5" t="n">
+        <v>200</v>
+      </c>
+      <c r="E5" t="n">
+        <v>29294.78</v>
+      </c>
+      <c r="F5" t="n">
+        <v>70</v>
+      </c>
+      <c r="G5" t="n">
+        <v>836</v>
+      </c>
+      <c r="H5" t="n">
+        <v>-350</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>A+ speed</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>13.19</v>
+      </c>
+      <c r="K5" t="n">
+        <v>8</v>
+      </c>
+      <c r="L5" t="n">
+        <v>29252.5</v>
+      </c>
+      <c r="M5" t="n">
+        <v>29223.75</v>
+      </c>
+      <c r="N5" t="n">
+        <v>29195</v>
+      </c>
+      <c r="O5" t="n">
+        <v>115</v>
+      </c>
+      <c r="P5" t="n">
+        <v>115</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>29220</v>
+      </c>
+      <c r="R5" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>POTENTIAL_RUNNER</t>
+        </is>
+      </c>
+      <c r="U5" t="n">
+        <v>5</v>
+      </c>
+      <c r="V5" t="n">
+        <v>80</v>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-aplus-structure-export</t>
+        </is>
+      </c>
+      <c r="X5" s="5" t="inlineStr">
+        <is>
+          <t>09:31:05</t>
+        </is>
+      </c>
+      <c r="Y5" t="n">
+        <v>2311</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>-1927</v>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>SessionDeltaSum</t>
+        </is>
+      </c>
+      <c r="AB5" t="n">
+        <v>-2027</v>
+      </c>
+      <c r="AC5" t="n">
+        <v>-1927</v>
+      </c>
+      <c r="AD5" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>Riesgo de reversion</t>
+        </is>
+      </c>
+      <c r="AF5" t="n">
+        <v>7150</v>
+      </c>
+      <c r="AG5" t="n">
+        <v>136</v>
+      </c>
+      <c r="AH5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AI5" t="n">
+        <v>-486</v>
+      </c>
+      <c r="AJ5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AK5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AL5" t="n">
+        <v>5.3081</v>
+      </c>
+      <c r="AM5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AN5" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AO5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AP5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AQ5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AR5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AS5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AT5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AU5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AV5" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="AW5" t="inlineStr">
+        <is>
+          <t>EXIT</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AY5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AZ5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="BC5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="BE5" s="6" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="6">
@@ -987,10 +1206,217 @@
           <t>2026-05-20</t>
         </is>
       </c>
-      <c r="R6" s="4" t="inlineStr">
-        <is>
-          <t>NO_CSV</t>
-        </is>
+      <c r="B6" t="n">
+        <v>29070</v>
+      </c>
+      <c r="C6" t="n">
+        <v>29122.5</v>
+      </c>
+      <c r="D6" t="n">
+        <v>210</v>
+      </c>
+      <c r="E6" t="n">
+        <v>29081.21</v>
+      </c>
+      <c r="F6" t="n">
+        <v>40</v>
+      </c>
+      <c r="G6" t="n">
+        <v>806</v>
+      </c>
+      <c r="H6" t="n">
+        <v>-178</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>A+ speed</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>8.82</v>
+      </c>
+      <c r="K6" t="n">
+        <v>8</v>
+      </c>
+      <c r="L6" t="n">
+        <v>29067.5</v>
+      </c>
+      <c r="M6" t="n">
+        <v>29057.5</v>
+      </c>
+      <c r="N6" t="n">
+        <v>29047.5</v>
+      </c>
+      <c r="O6" t="n">
+        <v>40</v>
+      </c>
+      <c r="P6" t="n">
+        <v>40</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>29057.5</v>
+      </c>
+      <c r="R6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>POTENTIAL_RUNNER</t>
+        </is>
+      </c>
+      <c r="U6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V6" t="n">
+        <v>20</v>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-aplus-structure-export</t>
+        </is>
+      </c>
+      <c r="X6" s="5" t="inlineStr">
+        <is>
+          <t>09:36:04</t>
+        </is>
+      </c>
+      <c r="Y6" t="n">
+        <v>2316</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>650</v>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>SessionDeltaSum</t>
+        </is>
+      </c>
+      <c r="AB6" t="n">
+        <v>632</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>650</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="AE6" t="inlineStr">
+        <is>
+          <t>Riesgo de reversion</t>
+        </is>
+      </c>
+      <c r="AF6" t="n">
+        <v>3478</v>
+      </c>
+      <c r="AG6" t="n">
+        <v>-486</v>
+      </c>
+      <c r="AH6" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AI6" t="n">
+        <v>308</v>
+      </c>
+      <c r="AJ6" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AK6" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AL6" t="n">
+        <v>4.5359</v>
+      </c>
+      <c r="AM6" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AN6" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AO6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AP6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AQ6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AR6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AS6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AT6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AU6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AV6" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="AW6" t="inlineStr">
+        <is>
+          <t>EXIT</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AY6" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AZ6" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="BC6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD6" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="BE6" s="6" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="7">
@@ -999,11 +1425,278 @@
           <t>2026-05-26</t>
         </is>
       </c>
-      <c r="R7" s="4" t="inlineStr">
-        <is>
-          <t>NO_CSV</t>
-        </is>
-      </c>
+      <c r="B7" t="n">
+        <v>29880</v>
+      </c>
+      <c r="C7" t="n">
+        <v>29935</v>
+      </c>
+      <c r="D7" t="n">
+        <v>220</v>
+      </c>
+      <c r="E7" t="n">
+        <v>29859.58</v>
+      </c>
+      <c r="F7" t="n">
+        <v>65</v>
+      </c>
+      <c r="G7" t="n">
+        <v>899</v>
+      </c>
+      <c r="H7" t="n">
+        <v>-93</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>A+ speed</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>5.11</v>
+      </c>
+      <c r="K7" t="n">
+        <v>8</v>
+      </c>
+      <c r="L7" t="n">
+        <v>29851.25</v>
+      </c>
+      <c r="M7" t="n">
+        <v>29837.5</v>
+      </c>
+      <c r="N7" t="n">
+        <v>29823.75</v>
+      </c>
+      <c r="O7" t="n">
+        <v>55</v>
+      </c>
+      <c r="P7" t="n">
+        <v>55</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>29837.5</v>
+      </c>
+      <c r="R7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>POTENTIAL_RUNNER</t>
+        </is>
+      </c>
+      <c r="U7" t="n">
+        <v>0</v>
+      </c>
+      <c r="V7" t="n">
+        <v>30</v>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>score-exporter-2026-05-30-aplus-structure-export</t>
+        </is>
+      </c>
+      <c r="X7" s="5" t="inlineStr">
+        <is>
+          <t>09:35:12</t>
+        </is>
+      </c>
+      <c r="Y7" t="n">
+        <v>2075</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>-133</v>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>SessionDeltaSum</t>
+        </is>
+      </c>
+      <c r="AB7" t="n">
+        <v>-207</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>-133</v>
+      </c>
+      <c r="AD7" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="AE7" t="inlineStr">
+        <is>
+          <t>Riesgo de reversion</t>
+        </is>
+      </c>
+      <c r="AF7" t="n">
+        <v>2999</v>
+      </c>
+      <c r="AG7" t="n">
+        <v>-267</v>
+      </c>
+      <c r="AH7" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AI7" t="n">
+        <v>174</v>
+      </c>
+      <c r="AJ7" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AK7" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AL7" t="n">
+        <v>12.7093</v>
+      </c>
+      <c r="AM7" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AN7" t="inlineStr">
+        <is>
+          <t>LastTime</t>
+        </is>
+      </c>
+      <c r="AO7" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AP7" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AQ7" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AR7" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AS7" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AT7" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AU7" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AV7" t="inlineStr">
+        <is>
+          <t>BREAKOUT</t>
+        </is>
+      </c>
+      <c r="AW7" t="inlineStr">
+        <is>
+          <t>EXIT</t>
+        </is>
+      </c>
+      <c r="AX7" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AY7" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AZ7" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="BC7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD7" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="BE7" s="6" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="R8" s="4" t="n"/>
+    </row>
+    <row r="9">
+      <c r="R9" s="4" t="n"/>
+    </row>
+    <row r="10">
+      <c r="R10" s="4" t="n"/>
+    </row>
+    <row r="11">
+      <c r="R11" s="4" t="n"/>
+    </row>
+    <row r="12">
+      <c r="R12" s="4" t="n"/>
+    </row>
+    <row r="13">
+      <c r="R13" s="4" t="n"/>
+    </row>
+    <row r="14">
+      <c r="R14" s="4" t="n"/>
+    </row>
+    <row r="15">
+      <c r="R15" s="4" t="n"/>
+    </row>
+    <row r="16">
+      <c r="R16" s="4" t="n"/>
+    </row>
+    <row r="17">
+      <c r="R17" s="4" t="n"/>
+    </row>
+    <row r="18">
+      <c r="R18" s="4" t="n"/>
+    </row>
+    <row r="19">
+      <c r="R19" s="4" t="n"/>
+    </row>
+    <row r="20">
+      <c r="R20" s="4" t="n"/>
+    </row>
+    <row r="21">
+      <c r="R21" s="4" t="n"/>
+    </row>
+    <row r="22">
+      <c r="R22" s="4" t="n"/>
+    </row>
+    <row r="23">
+      <c r="R23" s="4" t="n"/>
+    </row>
+    <row r="24">
+      <c r="R24" s="4" t="n"/>
+    </row>
+    <row r="25">
+      <c r="R25" s="4" t="n"/>
+    </row>
+    <row r="26">
+      <c r="R26" s="4" t="n"/>
+    </row>
+    <row r="27">
+      <c r="R27" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>